<commit_message>
Restore all 47 products added via Admin Panel
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -401,43 +401,43 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Product Code</v>
+        <v>code</v>
       </c>
       <c r="B1" t="str">
-        <v>Product Name</v>
+        <v>name</v>
       </c>
       <c r="C1" t="str">
-        <v>Category</v>
+        <v>category</v>
       </c>
       <c r="D1" t="str">
-        <v>Subcategory</v>
+        <v>subcategory</v>
       </c>
       <c r="E1" t="str">
-        <v>Price</v>
+        <v>price</v>
       </c>
       <c r="F1" t="str">
-        <v>Original Price</v>
+        <v>originalPrice</v>
       </c>
       <c r="G1" t="str">
-        <v>Stock Status</v>
+        <v>discountPct</v>
       </c>
       <c r="H1" t="str">
-        <v>Size</v>
+        <v>stockStatus</v>
       </c>
       <c r="I1" t="str">
-        <v>Image 1</v>
+        <v>image</v>
       </c>
       <c r="J1" t="str">
-        <v>Image 2</v>
+        <v>images</v>
       </c>
       <c r="K1" t="str">
-        <v>Image 3</v>
+        <v>size</v>
       </c>
       <c r="L1" t="str">
-        <v>Description</v>
+        <v>description</v>
       </c>
       <c r="M1" t="str">
-        <v>Featured</v>
+        <v>featured</v>
       </c>
     </row>
     <row r="2">
@@ -459,17 +459,14 @@
       <c r="F2">
         <v>10</v>
       </c>
-      <c r="G2" t="str">
-        <v>INSTOCK</v>
+      <c r="G2">
+        <v>40</v>
       </c>
       <c r="H2" t="str">
-        <v/>
+        <v>INSTOCK</v>
       </c>
       <c r="I2" t="str">
-        <v>1.jpeg</v>
-      </c>
-      <c r="J2" t="str">
-        <v/>
+        <v>images/1.jpeg</v>
       </c>
       <c r="K2" t="str">
         <v/>
@@ -477,8 +474,8 @@
       <c r="L2" t="str">
         <v>Add a touch of tradition without breaking the budget! 💛 Our beautiful Jimukkas are available in a variety of stunning shades to perfectly match your outfit.  🌸 Affordable • Stylish • Perfect for Every Occasion.</v>
       </c>
-      <c r="M2" t="str">
-        <v>No</v>
+      <c r="M2" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -500,17 +497,14 @@
       <c r="F3">
         <v>35</v>
       </c>
-      <c r="G3" t="str">
-        <v>INSTOCK</v>
+      <c r="G3">
+        <v>17</v>
       </c>
       <c r="H3" t="str">
-        <v/>
+        <v>INSTOCK</v>
       </c>
       <c r="I3" t="str">
-        <v>4.jpeg</v>
-      </c>
-      <c r="J3" t="str">
-        <v/>
+        <v>images/4.jpeg</v>
       </c>
       <c r="K3" t="str">
         <v/>
@@ -518,8 +512,8 @@
       <c r="L3" t="str">
         <v>A beautifully crafted choker necklace featuring elegant green stones and a comfortable adjustable thread closure. The perfect statement piece for sarees, lehengas, weddings, festive occasions, and traditional celebrations. 💚✨</v>
       </c>
-      <c r="M3" t="str">
-        <v>No</v>
+      <c r="M3" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -541,17 +535,14 @@
       <c r="F4">
         <v>90</v>
       </c>
-      <c r="G4" t="str">
-        <v>INSTOCK</v>
+      <c r="G4">
+        <v>18</v>
       </c>
       <c r="H4" t="str">
-        <v/>
+        <v>INSTOCK</v>
       </c>
       <c r="I4" t="str">
-        <v>5.jpeg</v>
-      </c>
-      <c r="J4" t="str">
-        <v/>
+        <v>images/5.jpeg</v>
       </c>
       <c r="K4" t="str">
         <v/>
@@ -559,8 +550,8 @@
       <c r="L4" t="str">
         <v>Grace meets elegance in this dreamy Soft Organza Saree, adorned with delicate floral prints and a beautifully finished scalloped border. Perfect for festive celebrations, parties, and special occasions. 🌸</v>
       </c>
-      <c r="M4" t="str">
-        <v>No</v>
+      <c r="M4" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -582,17 +573,14 @@
       <c r="F5">
         <v>68</v>
       </c>
-      <c r="G5" t="str">
-        <v>INSTOCK</v>
+      <c r="G5">
+        <v>0</v>
       </c>
       <c r="H5" t="str">
-        <v/>
+        <v>INSTOCK</v>
       </c>
       <c r="I5" t="str">
-        <v>6.jpeg</v>
-      </c>
-      <c r="J5" t="str">
-        <v/>
+        <v>images/6.jpeg</v>
       </c>
       <c r="K5" t="str">
         <v/>
@@ -600,8 +588,8 @@
       <c r="L5" t="str">
         <v>Graceful, lightweight, and effortlessly elegant. This beautiful Mul Chanderi 3-piece set features delicate embroidery with a matching bottom and soft dupatta—perfect for festive celebrations, family gatherings, and everyday elegance  SIZE TILL 44</v>
       </c>
-      <c r="M5" t="str">
-        <v>No</v>
+      <c r="M5" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -623,17 +611,14 @@
       <c r="F6">
         <v>50</v>
       </c>
-      <c r="G6" t="str">
-        <v>INSTOCK</v>
+      <c r="G6">
+        <v>10</v>
       </c>
       <c r="H6" t="str">
-        <v/>
+        <v>INSTOCK</v>
       </c>
       <c r="I6" t="str">
-        <v>7.jpeg</v>
-      </c>
-      <c r="J6" t="str">
-        <v/>
+        <v>images/7.jpeg</v>
       </c>
       <c r="K6" t="str">
         <v/>
@@ -641,8 +626,8 @@
       <c r="L6" t="str">
         <v>Celebrate every special moment in timeless tradition! ❤️ This elegant Kids Pattu Pavada features a beautifully printed lotus skirt with a rich maroon puff-sleeve blouse, making it a perfect choice for Onam, festivals, temple visits, and family celebrations. Size -3 yrs /5yrs /6yrs</v>
       </c>
-      <c r="M6" t="str">
-        <v>No</v>
+      <c r="M6" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -664,17 +649,14 @@
       <c r="F7">
         <v>41</v>
       </c>
-      <c r="G7" t="str">
-        <v>INSTOCK</v>
+      <c r="G7">
+        <v>29</v>
       </c>
       <c r="H7" t="str">
-        <v/>
+        <v>INSTOCK</v>
       </c>
       <c r="I7" t="str">
-        <v>8.jpg</v>
-      </c>
-      <c r="J7" t="str">
-        <v/>
+        <v>images/8.jpg</v>
       </c>
       <c r="K7" t="str">
         <v/>
@@ -682,8 +664,8 @@
       <c r="L7" t="str">
         <v>A beautifully crafted choker necklace featuring elegant green stones and a comfortable adjustable thread closure. The perfect statement piece for sarees, lehengas, weddings, festive occasions, and traditional celebrations. 💚✨</v>
       </c>
-      <c r="M7" t="str">
-        <v>No</v>
+      <c r="M7" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -705,17 +687,14 @@
       <c r="F8">
         <v>83</v>
       </c>
-      <c r="G8" t="str">
-        <v>INSTOCK</v>
+      <c r="G8">
+        <v>18</v>
       </c>
       <c r="H8" t="str">
-        <v/>
+        <v>INSTOCK</v>
       </c>
       <c r="I8" t="str">
-        <v>9.jpeg</v>
-      </c>
-      <c r="J8" t="str">
-        <v/>
+        <v>images/9.jpeg</v>
       </c>
       <c r="K8" t="str">
         <v/>
@@ -723,8 +702,8 @@
       <c r="L8" t="str">
         <v>Grace meets tradition in this elegant soft tissue saree, beautifully finished with a stunning floral Kalamkari-inspired border. A timeless choice for festive celebrations and special occasions.</v>
       </c>
-      <c r="M8" t="str">
-        <v>No</v>
+      <c r="M8" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -746,17 +725,14 @@
       <c r="F9">
         <v>70</v>
       </c>
-      <c r="G9" t="str">
-        <v>INSTOCK</v>
+      <c r="G9">
+        <v>11</v>
       </c>
       <c r="H9" t="str">
-        <v/>
+        <v>INSTOCK</v>
       </c>
       <c r="I9" t="str">
-        <v>10.jpeg</v>
-      </c>
-      <c r="J9" t="str">
-        <v/>
+        <v>images/10.jpeg</v>
       </c>
       <c r="K9" t="str">
         <v/>
@@ -764,8 +740,8 @@
       <c r="L9" t="str">
         <v>Make a statement with this elegant premium embroidered kurta, crafted for weddings, festivals, and special occasions.</v>
       </c>
-      <c r="M9" t="str">
-        <v>No</v>
+      <c r="M9" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -787,26 +763,23 @@
       <c r="F10">
         <v>43</v>
       </c>
-      <c r="G10" t="str">
-        <v>INSTOCK</v>
+      <c r="G10">
+        <v>19</v>
       </c>
       <c r="H10" t="str">
-        <v/>
+        <v>INSTOCK</v>
       </c>
       <c r="I10" t="str">
-        <v>11.jpeg</v>
-      </c>
-      <c r="J10" t="str">
-        <v>df3d9838-004b-4a86-9075-49c17538c55b.jpg</v>
+        <v>images/11.jpeg</v>
       </c>
       <c r="K10" t="str">
-        <v>11e4c6e5-82d6-479d-a903-4424e4b1a1e8.jpg</v>
+        <v/>
       </c>
       <c r="L10" t="str">
         <v>Elevate your saree look with our elegant free-size embroidered blouse, designed for both comfort and style. Free size – Fits 36–42 inches (with alteration margin)</v>
       </c>
-      <c r="M10" t="str">
-        <v>No</v>
+      <c r="M10" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -828,17 +801,14 @@
       <c r="F11">
         <v>35</v>
       </c>
-      <c r="G11" t="str">
+      <c r="G11">
+        <v>20</v>
+      </c>
+      <c r="H11" t="str">
         <v>LIMITED STOCK</v>
       </c>
-      <c r="H11" t="str">
-        <v/>
-      </c>
       <c r="I11" t="str">
-        <v>14.jpeg</v>
-      </c>
-      <c r="J11" t="str">
-        <v/>
+        <v>images/14.jpeg</v>
       </c>
       <c r="K11" t="str">
         <v/>
@@ -846,8 +816,8 @@
       <c r="L11" t="str">
         <v>A sparkling American Diamond pendant with matching earrings, designed to add effortless elegance to your look. Pair it with your favourite chain for a personalized style.</v>
       </c>
-      <c r="M11" t="str">
-        <v>No</v>
+      <c r="M11" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -869,17 +839,14 @@
       <c r="F12">
         <v>36</v>
       </c>
-      <c r="G12" t="str">
+      <c r="G12">
+        <v>17</v>
+      </c>
+      <c r="H12" t="str">
         <v>LIMITED STOCK</v>
       </c>
-      <c r="H12" t="str">
-        <v/>
-      </c>
       <c r="I12" t="str">
-        <v>16.jpeg</v>
-      </c>
-      <c r="J12" t="str">
-        <v/>
+        <v>images/16.jpeg</v>
       </c>
       <c r="K12" t="str">
         <v/>
@@ -887,8 +854,8 @@
       <c r="L12" t="str">
         <v>A stunning antique-finish pendant set accented with rich purple stones and matching earrings. Designed to bring a touch of vintage elegance to every festive look.</v>
       </c>
-      <c r="M12" t="str">
-        <v>No</v>
+      <c r="M12" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -910,17 +877,14 @@
       <c r="F13">
         <v>49</v>
       </c>
-      <c r="G13" t="str">
+      <c r="G13">
+        <v>39</v>
+      </c>
+      <c r="H13" t="str">
         <v>LIMITED STOCK</v>
       </c>
-      <c r="H13" t="str">
-        <v/>
-      </c>
       <c r="I13" t="str">
-        <v>18.jpeg</v>
-      </c>
-      <c r="J13" t="str">
-        <v/>
+        <v>images/18.jpeg</v>
       </c>
       <c r="K13" t="str">
         <v/>
@@ -928,8 +892,8 @@
       <c r="L13" t="str">
         <v>A graceful antique-finish pendant set featuring a stunning emerald-green stone with matching earrings. Perfect for adding timeless elegance to your ethnic look.</v>
       </c>
-      <c r="M13" t="str">
-        <v>No</v>
+      <c r="M13" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -951,17 +915,14 @@
       <c r="F14">
         <v>63</v>
       </c>
-      <c r="G14" t="str">
-        <v>INSTOCK</v>
+      <c r="G14">
+        <v>8</v>
       </c>
       <c r="H14" t="str">
-        <v/>
+        <v>INSTOCK</v>
       </c>
       <c r="I14" t="str">
-        <v>20.jpeg</v>
-      </c>
-      <c r="J14" t="str">
-        <v/>
+        <v>images/20.jpeg</v>
       </c>
       <c r="K14" t="str">
         <v/>
@@ -969,8 +930,8 @@
       <c r="L14" t="str">
         <v>Light as a breeze, elegant in every drape. A soft tissue saree with beautiful lotus floral prints and a matching blouse piece—perfect for festive and special occasions.</v>
       </c>
-      <c r="M14" t="str">
-        <v>No</v>
+      <c r="M14" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -992,17 +953,14 @@
       <c r="F15">
         <v>36</v>
       </c>
-      <c r="G15" t="str">
-        <v>INSTOCK</v>
+      <c r="G15">
+        <v>17</v>
       </c>
       <c r="H15" t="str">
-        <v/>
+        <v>INSTOCK</v>
       </c>
       <c r="I15" t="str">
-        <v>23.jpeg</v>
-      </c>
-      <c r="J15" t="str">
-        <v/>
+        <v>images/23.jpeg</v>
       </c>
       <c r="K15" t="str">
         <v/>
@@ -1010,8 +968,8 @@
       <c r="L15" t="str">
         <v>A timeless Nagapadam necklace with matching jhumkas, beautifully crafted in royal blue and emerald green for a graceful traditional look.</v>
       </c>
-      <c r="M15" t="str">
-        <v>No</v>
+      <c r="M15" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -1033,17 +991,14 @@
       <c r="F16">
         <v>100</v>
       </c>
-      <c r="G16" t="str">
-        <v>INSTOCK</v>
+      <c r="G16">
+        <v>20</v>
       </c>
       <c r="H16" t="str">
-        <v/>
+        <v>INSTOCK</v>
       </c>
       <c r="I16" t="str">
-        <v>24.jpeg</v>
-      </c>
-      <c r="J16" t="str">
-        <v/>
+        <v>images/24.jpeg</v>
       </c>
       <c r="K16" t="str">
         <v/>
@@ -1051,8 +1006,8 @@
       <c r="L16" t="str">
         <v>Rich wine-red semi tusser saree featuring an exquisite floral embroidered lace border. Elegant, lightweight, and perfect for festive celebrations, weddings, and special occasions.</v>
       </c>
-      <c r="M16" t="str">
-        <v>No</v>
+      <c r="M16" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="17">
@@ -1074,17 +1029,14 @@
       <c r="F17">
         <v>28</v>
       </c>
-      <c r="G17" t="str">
+      <c r="G17">
+        <v>25</v>
+      </c>
+      <c r="H17" t="str">
         <v>LIMITED STOCK</v>
       </c>
-      <c r="H17" t="str">
-        <v/>
-      </c>
       <c r="I17" t="str">
-        <v>e2a2ec34-dc2e-4090-b325-67b69445b9dd.jpg</v>
-      </c>
-      <c r="J17" t="str">
-        <v/>
+        <v>images/e2a2ec34-dc2e-4090-b325-67b69445b9dd.jpg</v>
       </c>
       <c r="K17" t="str">
         <v/>
@@ -1092,8 +1044,8 @@
       <c r="L17" t="str">
         <v/>
       </c>
-      <c r="M17" t="str">
-        <v>No</v>
+      <c r="M17" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="18">
@@ -1115,26 +1067,23 @@
       <c r="F18">
         <v>110</v>
       </c>
-      <c r="G18" t="str">
-        <v>INSTOCK</v>
+      <c r="G18">
+        <v>19</v>
       </c>
       <c r="H18" t="str">
-        <v/>
+        <v>INSTOCK</v>
       </c>
       <c r="I18" t="str">
-        <v>e67c8e99-625e-4772-b3cc-daeca03c1dd4.jpg</v>
-      </c>
-      <c r="J18" t="str">
-        <v>ff6718dd-402c-49e9-bf6e-4f5bca42721f.jpg</v>
+        <v>images/e67c8e99-625e-4772-b3cc-daeca03c1dd4.jpg</v>
       </c>
       <c r="K18" t="str">
-        <v>d8259ec9-5688-4b4d-9bb9-5572dbc0ab41.jpg</v>
+        <v/>
       </c>
       <c r="L18" t="str">
         <v>A rich maroon saree featuring an elegant gold saree border and beautifully woven traditional motifs—perfect for weddings, festive occasions and celebrations.</v>
       </c>
-      <c r="M18" t="str">
-        <v>No</v>
+      <c r="M18" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="19">
@@ -1156,17 +1105,14 @@
       <c r="F19">
         <v>50</v>
       </c>
-      <c r="G19" t="str">
-        <v>INSTOCK</v>
+      <c r="G19">
+        <v>16</v>
       </c>
       <c r="H19" t="str">
-        <v/>
+        <v>INSTOCK</v>
       </c>
       <c r="I19" t="str">
-        <v>eb7df1cd-6b0d-42f9-9be7-44d51c6d527e.jpg</v>
-      </c>
-      <c r="J19" t="str">
-        <v/>
+        <v>images/eb7df1cd-6b0d-42f9-9be7-44d51c6d527e.jpg</v>
       </c>
       <c r="K19" t="str">
         <v/>
@@ -1174,8 +1120,8 @@
       <c r="L19" t="str">
         <v>A rich emerald-green blouse featuring elegant gold floral weaving and a stylish tie-back detail—perfect for pairing with silk, tissue, or festive sarees.</v>
       </c>
-      <c r="M19" t="str">
-        <v>No</v>
+      <c r="M19" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="20">
@@ -1197,17 +1143,14 @@
       <c r="F20">
         <v>50</v>
       </c>
-      <c r="G20" t="str">
+      <c r="G20">
+        <v>12</v>
+      </c>
+      <c r="H20" t="str">
         <v>LIMITED STOCK</v>
       </c>
-      <c r="H20" t="str">
-        <v/>
-      </c>
       <c r="I20" t="str">
-        <v>a1c56268-4968-4ea5-ab01-51b256c4f4a6.jpg</v>
-      </c>
-      <c r="J20" t="str">
-        <v/>
+        <v>images/a1c56268-4968-4ea5-ab01-51b256c4f4a6.jpg</v>
       </c>
       <c r="K20" t="str">
         <v/>
@@ -1215,8 +1158,8 @@
       <c r="L20" t="str">
         <v>A graceful gold-toned choker adorned with ruby-green stones and sparkling accents—perfect for sarees, lehengas and festive looks.</v>
       </c>
-      <c r="M20" t="str">
-        <v>No</v>
+      <c r="M20" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="21">
@@ -1238,17 +1181,14 @@
       <c r="F21">
         <v>60</v>
       </c>
-      <c r="G21" t="str">
+      <c r="G21">
+        <v>32</v>
+      </c>
+      <c r="H21" t="str">
         <v>LIMITED STOCK</v>
       </c>
-      <c r="H21" t="str">
-        <v/>
-      </c>
       <c r="I21" t="str">
-        <v>4a69a0a6-847f-4a32-83e5-743f681ad6b9.jpg</v>
-      </c>
-      <c r="J21" t="str">
-        <v/>
+        <v>images/4a69a0a6-847f-4a32-83e5-743f681ad6b9.jpg</v>
       </c>
       <c r="K21" t="str">
         <v/>
@@ -1256,8 +1196,8 @@
       <c r="L21" t="str">
         <v>A graceful stone-studded necklace with matching earrings—perfect for adding a rich, elegant sparkle to any special occasion.</v>
       </c>
-      <c r="M21" t="str">
-        <v>No</v>
+      <c r="M21" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="22">
@@ -1279,17 +1219,14 @@
       <c r="F22">
         <v>45</v>
       </c>
-      <c r="G22" t="str">
+      <c r="G22">
+        <v>24</v>
+      </c>
+      <c r="H22" t="str">
         <v>LIMITED STOCK</v>
       </c>
-      <c r="H22" t="str">
-        <v/>
-      </c>
       <c r="I22" t="str">
-        <v>3366e4f8-6047-4d0e-81ba-c81b83319764.jpg</v>
-      </c>
-      <c r="J22" t="str">
-        <v>54b330a1-5c22-45b7-8fbc-5c12387a8d04.jpg</v>
+        <v>images/3366e4f8-6047-4d0e-81ba-c81b83319764.jpg</v>
       </c>
       <c r="K22" t="str">
         <v/>
@@ -1297,8 +1234,8 @@
       <c r="L22" t="str">
         <v>A delicate gold-finish design with sparkling stones and matching studs—perfect for parties and special occasions.</v>
       </c>
-      <c r="M22" t="str">
-        <v>No</v>
+      <c r="M22" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="23">
@@ -1320,17 +1257,14 @@
       <c r="F23">
         <v>40</v>
       </c>
-      <c r="G23" t="str">
+      <c r="G23">
+        <v>35</v>
+      </c>
+      <c r="H23" t="str">
         <v>LIMITED STOCK</v>
       </c>
-      <c r="H23" t="str">
-        <v/>
-      </c>
       <c r="I23" t="str">
-        <v>bfc3ccbe-db6b-494b-96a1-d4dcbb46e9a6.jpg</v>
-      </c>
-      <c r="J23" t="str">
-        <v>aed5ffa5-8e72-4973-89ef-03fcd711aef3.jpg</v>
+        <v>images/bfc3ccbe-db6b-494b-96a1-d4dcbb46e9a6.jpg</v>
       </c>
       <c r="K23" t="str">
         <v/>
@@ -1338,8 +1272,8 @@
       <c r="L23" t="str">
         <v>A graceful traditional AD necklace featuring rich ruby-toned stones, a striking emerald-green centerpiece, and elegant pearl drops. Perfect for weddings, festive celebrations, and special occasions.</v>
       </c>
-      <c r="M23" t="str">
-        <v>No</v>
+      <c r="M23" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="24">
@@ -1361,17 +1295,14 @@
       <c r="F24">
         <v>46</v>
       </c>
-      <c r="G24" t="str">
-        <v>INSTOCK</v>
+      <c r="G24">
+        <v>35</v>
       </c>
       <c r="H24" t="str">
-        <v/>
+        <v>INSTOCK</v>
       </c>
       <c r="I24" t="str">
-        <v>d260a0ff-0114-4653-8285-8a5afe33ec43.jpg</v>
-      </c>
-      <c r="J24" t="str">
-        <v>749df6e2-3b93-4e55-928d-6a51fb361d97.jpg</v>
+        <v>images/d260a0ff-0114-4653-8285-8a5afe33ec43.jpg</v>
       </c>
       <c r="K24" t="str">
         <v/>
@@ -1379,8 +1310,8 @@
       <c r="L24" t="str">
         <v>Elegant antique-finish necklace featuring delicate pearl florals, rich ruby-toned stones and a beautifully detailed pendant. A graceful choice for festive and traditional looks.</v>
       </c>
-      <c r="M24" t="str">
-        <v>No</v>
+      <c r="M24" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="25" xml:space="preserve">
@@ -1402,17 +1333,14 @@
       <c r="F25">
         <v>55</v>
       </c>
-      <c r="G25" t="str">
-        <v>INSTOCK</v>
+      <c r="G25">
+        <v>31</v>
       </c>
       <c r="H25" t="str">
-        <v/>
+        <v>INSTOCK</v>
       </c>
       <c r="I25" t="str">
-        <v>c129d1b5-a9d7-413e-a9ba-ed756e6b96ce.jpg</v>
-      </c>
-      <c r="J25" t="str">
-        <v/>
+        <v>images/c129d1b5-a9d7-413e-a9ba-ed756e6b96ce.jpg</v>
       </c>
       <c r="K25" t="str">
         <v/>
@@ -1421,8 +1349,8 @@
         <v xml:space="preserve">Emerald Glow Necklace Set 💚
 A stunning emerald-green stone necklace with matching earrings, beautifully framed with sparkling accents. Perfect for festive occasions, parties and elegant traditional looks.</v>
       </c>
-      <c r="M25" t="str">
-        <v>No</v>
+      <c r="M25" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="26">
@@ -1444,17 +1372,14 @@
       <c r="F26">
         <v>46</v>
       </c>
-      <c r="G26" t="str">
-        <v>INSTOCK</v>
+      <c r="G26">
+        <v>26</v>
       </c>
       <c r="H26" t="str">
-        <v/>
+        <v>INSTOCK</v>
       </c>
       <c r="I26" t="str">
-        <v>efb45acd-3a86-4179-bc43-f4ed4608590c.jpg</v>
-      </c>
-      <c r="J26" t="str">
-        <v/>
+        <v>images/efb45acd-3a86-4179-bc43-f4ed4608590c.jpg</v>
       </c>
       <c r="K26" t="str">
         <v/>
@@ -1462,8 +1387,8 @@
       <c r="L26" t="str">
         <v>Pearl elegance with a radiant ruby-centred pendant—simple, graceful and timeless.</v>
       </c>
-      <c r="M26" t="str">
-        <v>No</v>
+      <c r="M26" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="27" xml:space="preserve">
@@ -1485,17 +1410,14 @@
       <c r="F27">
         <v>32</v>
       </c>
-      <c r="G27" t="str">
-        <v>INSTOCK</v>
+      <c r="G27">
+        <v>28</v>
       </c>
       <c r="H27" t="str">
-        <v/>
+        <v>INSTOCK</v>
       </c>
       <c r="I27" t="str">
-        <v>19c70259-71e8-4892-b897-5ffe5b75a8a2.jpg</v>
-      </c>
-      <c r="J27" t="str">
-        <v/>
+        <v>images/19c70259-71e8-4892-b897-5ffe5b75a8a2.jpg</v>
       </c>
       <c r="K27" t="str">
         <v/>
@@ -1505,8 +1427,8 @@
 Beautifully crafted gold-tone bangles with striking ruby-pink stones—perfect for adding a royal touch to any outfit.
 $12 per piece.</v>
       </c>
-      <c r="M27" t="str">
-        <v>No</v>
+      <c r="M27" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="28" xml:space="preserve">
@@ -1528,17 +1450,14 @@
       <c r="F28">
         <v>45</v>
       </c>
-      <c r="G28" t="str">
-        <v>INSTOCK</v>
+      <c r="G28">
+        <v>24</v>
       </c>
       <c r="H28" t="str">
-        <v/>
+        <v>INSTOCK</v>
       </c>
       <c r="I28" t="str">
-        <v>36a990df-97b7-4102-87c7-e8ece22eb01c.jpg</v>
-      </c>
-      <c r="J28" t="str">
-        <v/>
+        <v>images/36a990df-97b7-4102-87c7-e8ece22eb01c.jpg</v>
       </c>
       <c r="K28" t="str">
         <v/>
@@ -1547,8 +1466,8 @@
         <v xml:space="preserve">Royal Ruby AD Necklace ✨
 An elegant gold-tone necklace adorned with sparkling white stones and rich ruby accents—perfect for weddings, parties and festive occasions.</v>
       </c>
-      <c r="M28" t="str">
-        <v>No</v>
+      <c r="M28" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="29">
@@ -1570,17 +1489,14 @@
       <c r="F29">
         <v>53</v>
       </c>
-      <c r="G29" t="str">
-        <v>INSTOCK</v>
+      <c r="G29">
+        <v>23</v>
       </c>
       <c r="H29" t="str">
-        <v/>
+        <v>INSTOCK</v>
       </c>
       <c r="I29" t="str">
-        <v>cf2f6a9e-6775-46d3-81a6-71d59978a4d4.jpg</v>
-      </c>
-      <c r="J29" t="str">
-        <v/>
+        <v>images/cf2f6a9e-6775-46d3-81a6-71d59978a4d4.jpg</v>
       </c>
       <c r="K29" t="str">
         <v/>
@@ -1588,8 +1504,8 @@
       <c r="L29" t="str">
         <v>A grand gold-tone necklace adorned with ruby, emerald and sparkling stones, finished with elegant pearl drops and matching earrings—perfect for weddings and traditional celebrations.</v>
       </c>
-      <c r="M29" t="str">
-        <v>No</v>
+      <c r="M29" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="30">
@@ -1611,17 +1527,14 @@
       <c r="F30">
         <v>30</v>
       </c>
-      <c r="G30" t="str">
-        <v>INSTOCK</v>
+      <c r="G30">
+        <v>13</v>
       </c>
       <c r="H30" t="str">
-        <v/>
+        <v>INSTOCK</v>
       </c>
       <c r="I30" t="str">
-        <v>d685200c-aa2a-49aa-a40c-ff0e81b77b31.jpg</v>
-      </c>
-      <c r="J30" t="str">
-        <v>76bcda54-8fcc-4d26-8d44-47ef8efa0999.jpg</v>
+        <v>images/d685200c-aa2a-49aa-a40c-ff0e81b77b31.jpg</v>
       </c>
       <c r="K30" t="str">
         <v/>
@@ -1629,8 +1542,8 @@
       <c r="L30" t="str">
         <v/>
       </c>
-      <c r="M30" t="str">
-        <v>Yes</v>
+      <c r="M30" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="31">
@@ -1652,17 +1565,14 @@
       <c r="F31">
         <v>16</v>
       </c>
-      <c r="G31" t="str">
-        <v>INSTOCK</v>
+      <c r="G31">
+        <v>13</v>
       </c>
       <c r="H31" t="str">
-        <v/>
+        <v>INSTOCK</v>
       </c>
       <c r="I31" t="str">
-        <v>c7105671-a5a0-4d8e-ac6b-cd5ddaac98c6.jpg</v>
-      </c>
-      <c r="J31" t="str">
-        <v>536799ba-7341-40bd-9449-3467d1cd5f62.jpg</v>
+        <v>images/c7105671-a5a0-4d8e-ac6b-cd5ddaac98c6.jpg</v>
       </c>
       <c r="K31" t="str">
         <v/>
@@ -1670,8 +1580,8 @@
       <c r="L31" t="str">
         <v/>
       </c>
-      <c r="M31" t="str">
-        <v>No</v>
+      <c r="M31" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="32">
@@ -1693,26 +1603,23 @@
       <c r="F32">
         <v>56</v>
       </c>
-      <c r="G32" t="str">
-        <v>INSTOCK</v>
+      <c r="G32">
+        <v>11</v>
       </c>
       <c r="H32" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="I32" t="str">
+        <v>images/db1f3be6-3522-4112-8f3b-69d800c64db6.jpg</v>
+      </c>
+      <c r="K32" t="str">
         <v>38</v>
       </c>
-      <c r="I32" t="str">
-        <v>db1f3be6-3522-4112-8f3b-69d800c64db6.jpg</v>
-      </c>
-      <c r="J32" t="str">
-        <v/>
-      </c>
-      <c r="K32" t="str">
-        <v/>
-      </c>
       <c r="L32" t="str">
         <v/>
       </c>
-      <c r="M32" t="str">
-        <v>No</v>
+      <c r="M32" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="33">
@@ -1734,17 +1641,14 @@
       <c r="F33">
         <v>80</v>
       </c>
-      <c r="G33" t="str">
-        <v>INSTOCK</v>
+      <c r="G33">
+        <v>8</v>
       </c>
       <c r="H33" t="str">
-        <v/>
+        <v>INSTOCK</v>
       </c>
       <c r="I33" t="str">
-        <v>a12db22a-a74a-40f8-b684-c0e8a4fc7a39.jpg</v>
-      </c>
-      <c r="J33" t="str">
-        <v>e687a50e-173b-4f3f-860e-d3712e2ab7de.jpg</v>
+        <v>images/a12db22a-a74a-40f8-b684-c0e8a4fc7a39.jpg</v>
       </c>
       <c r="K33" t="str">
         <v/>
@@ -1752,8 +1656,8 @@
       <c r="L33" t="str">
         <v/>
       </c>
-      <c r="M33" t="str">
-        <v>No</v>
+      <c r="M33" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="34">
@@ -1775,17 +1679,14 @@
       <c r="F34">
         <v>31</v>
       </c>
-      <c r="G34" t="str">
-        <v>INSTOCK</v>
+      <c r="G34">
+        <v>23</v>
       </c>
       <c r="H34" t="str">
-        <v/>
+        <v>INSTOCK</v>
       </c>
       <c r="I34" t="str">
-        <v>e489f3b2-e2ef-4f46-9271-149637630891.jpg</v>
-      </c>
-      <c r="J34" t="str">
-        <v/>
+        <v>images/e489f3b2-e2ef-4f46-9271-149637630891.jpg</v>
       </c>
       <c r="K34" t="str">
         <v/>
@@ -1793,8 +1694,8 @@
       <c r="L34" t="str">
         <v/>
       </c>
-      <c r="M34" t="str">
-        <v>No</v>
+      <c r="M34" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="35">
@@ -1816,17 +1717,14 @@
       <c r="F35">
         <v>72</v>
       </c>
-      <c r="G35" t="str">
-        <v>INSTOCK</v>
+      <c r="G35">
+        <v>4</v>
       </c>
       <c r="H35" t="str">
-        <v/>
+        <v>INSTOCK</v>
       </c>
       <c r="I35" t="str">
-        <v>c499e627-94d4-474f-97a9-795d83c56bba.jpg</v>
-      </c>
-      <c r="J35" t="str">
-        <v/>
+        <v>images/c499e627-94d4-474f-97a9-795d83c56bba.jpg</v>
       </c>
       <c r="K35" t="str">
         <v/>
@@ -1834,8 +1732,8 @@
       <c r="L35" t="str">
         <v/>
       </c>
-      <c r="M35" t="str">
-        <v>No</v>
+      <c r="M35" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="36">
@@ -1857,17 +1755,14 @@
       <c r="F36">
         <v>100</v>
       </c>
-      <c r="G36" t="str">
-        <v>INSTOCK</v>
+      <c r="G36">
+        <v>14</v>
       </c>
       <c r="H36" t="str">
-        <v/>
+        <v>INSTOCK</v>
       </c>
       <c r="I36" t="str">
-        <v>f87f53fe-3742-4c06-8f10-173b9fa436a1.jpg</v>
-      </c>
-      <c r="J36" t="str">
-        <v/>
+        <v>images/f87f53fe-3742-4c06-8f10-173b9fa436a1.jpg</v>
       </c>
       <c r="K36" t="str">
         <v/>
@@ -1875,8 +1770,8 @@
       <c r="L36" t="str">
         <v/>
       </c>
-      <c r="M36" t="str">
-        <v>No</v>
+      <c r="M36" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="37">
@@ -1898,17 +1793,14 @@
       <c r="F37">
         <v>22</v>
       </c>
-      <c r="G37" t="str">
-        <v>INSTOCK</v>
+      <c r="G37">
+        <v>18</v>
       </c>
       <c r="H37" t="str">
-        <v/>
+        <v>INSTOCK</v>
       </c>
       <c r="I37" t="str">
-        <v>8efcb74e-96d4-4e9c-9a0e-1c4e0edfdb0b.jpg</v>
-      </c>
-      <c r="J37" t="str">
-        <v/>
+        <v>images/8efcb74e-96d4-4e9c-9a0e-1c4e0edfdb0b.jpg</v>
       </c>
       <c r="K37" t="str">
         <v/>
@@ -1916,8 +1808,8 @@
       <c r="L37" t="str">
         <v/>
       </c>
-      <c r="M37" t="str">
-        <v>No</v>
+      <c r="M37" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="38">
@@ -1939,17 +1831,14 @@
       <c r="F38">
         <v>90</v>
       </c>
-      <c r="G38" t="str">
-        <v>INSTOCK</v>
+      <c r="G38">
+        <v>16</v>
       </c>
       <c r="H38" t="str">
-        <v/>
+        <v>INSTOCK</v>
       </c>
       <c r="I38" t="str">
-        <v>7924eaaa-b32b-43bc-aa78-1e3dc81e9141.jpg</v>
-      </c>
-      <c r="J38" t="str">
-        <v/>
+        <v>images/7924eaaa-b32b-43bc-aa78-1e3dc81e9141.jpg</v>
       </c>
       <c r="K38" t="str">
         <v/>
@@ -1957,8 +1846,8 @@
       <c r="L38" t="str">
         <v/>
       </c>
-      <c r="M38" t="str">
-        <v>No</v>
+      <c r="M38" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="39">
@@ -1980,17 +1869,14 @@
       <c r="F39">
         <v>69</v>
       </c>
-      <c r="G39" t="str">
-        <v>INSTOCK</v>
+      <c r="G39">
+        <v>13</v>
       </c>
       <c r="H39" t="str">
-        <v/>
+        <v>INSTOCK</v>
       </c>
       <c r="I39" t="str">
-        <v>2f2517ba-9ed9-45c9-9dec-38bc51668a15.jpg</v>
-      </c>
-      <c r="J39" t="str">
-        <v/>
+        <v>images/2f2517ba-9ed9-45c9-9dec-38bc51668a15.jpg</v>
       </c>
       <c r="K39" t="str">
         <v/>
@@ -1998,8 +1884,8 @@
       <c r="L39" t="str">
         <v/>
       </c>
-      <c r="M39" t="str">
-        <v>No</v>
+      <c r="M39" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="40">
@@ -2021,17 +1907,14 @@
       <c r="F40">
         <v>70</v>
       </c>
-      <c r="G40" t="str">
-        <v>INSTOCK</v>
+      <c r="G40">
+        <v>7</v>
       </c>
       <c r="H40" t="str">
-        <v/>
+        <v>INSTOCK</v>
       </c>
       <c r="I40" t="str">
-        <v>c0c95e56-1226-4f27-a8dc-f91a08506f09.jpg</v>
-      </c>
-      <c r="J40" t="str">
-        <v/>
+        <v>images/c0c95e56-1226-4f27-a8dc-f91a08506f09.jpg</v>
       </c>
       <c r="K40" t="str">
         <v/>
@@ -2039,8 +1922,8 @@
       <c r="L40" t="str">
         <v/>
       </c>
-      <c r="M40" t="str">
-        <v>No</v>
+      <c r="M40" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="41">
@@ -2062,17 +1945,14 @@
       <c r="F41">
         <v>80</v>
       </c>
-      <c r="G41" t="str">
-        <v>INSTOCK</v>
+      <c r="G41">
+        <v>8</v>
       </c>
       <c r="H41" t="str">
-        <v/>
+        <v>INSTOCK</v>
       </c>
       <c r="I41" t="str">
-        <v>d0d50de4-ecce-48ef-a2a4-d41988b98860.jpg</v>
-      </c>
-      <c r="J41" t="str">
-        <v/>
+        <v>images/d0d50de4-ecce-48ef-a2a4-d41988b98860.jpg</v>
       </c>
       <c r="K41" t="str">
         <v/>
@@ -2080,8 +1960,8 @@
       <c r="L41" t="str">
         <v/>
       </c>
-      <c r="M41" t="str">
-        <v>No</v>
+      <c r="M41" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="42">
@@ -2103,17 +1983,14 @@
       <c r="F42">
         <v>80</v>
       </c>
-      <c r="G42" t="str">
-        <v>INSTOCK</v>
+      <c r="G42">
+        <v>14</v>
       </c>
       <c r="H42" t="str">
-        <v/>
+        <v>INSTOCK</v>
       </c>
       <c r="I42" t="str">
-        <v>493b7819-92bf-4b24-93eb-67f3e4520217.jpg</v>
-      </c>
-      <c r="J42" t="str">
-        <v/>
+        <v>images/493b7819-92bf-4b24-93eb-67f3e4520217.jpg</v>
       </c>
       <c r="K42" t="str">
         <v/>
@@ -2121,8 +1998,8 @@
       <c r="L42" t="str">
         <v/>
       </c>
-      <c r="M42" t="str">
-        <v>No</v>
+      <c r="M42" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="43">
@@ -2144,17 +2021,14 @@
       <c r="F43">
         <v>71</v>
       </c>
-      <c r="G43" t="str">
-        <v>INSTOCK</v>
+      <c r="G43">
+        <v>4</v>
       </c>
       <c r="H43" t="str">
-        <v/>
+        <v>INSTOCK</v>
       </c>
       <c r="I43" t="str">
-        <v>bdd10649-fb6d-442a-b7cc-e001b3b03b9a.jpg</v>
-      </c>
-      <c r="J43" t="str">
-        <v/>
+        <v>images/bdd10649-fb6d-442a-b7cc-e001b3b03b9a.jpg</v>
       </c>
       <c r="K43" t="str">
         <v/>
@@ -2162,8 +2036,8 @@
       <c r="L43" t="str">
         <v/>
       </c>
-      <c r="M43" t="str">
-        <v>No</v>
+      <c r="M43" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="44" xml:space="preserve">
@@ -2185,17 +2059,14 @@
       <c r="F44">
         <v>50</v>
       </c>
-      <c r="G44" t="str">
-        <v>INSTOCK</v>
+      <c r="G44">
+        <v>20</v>
       </c>
       <c r="H44" t="str">
-        <v/>
+        <v>INSTOCK</v>
       </c>
       <c r="I44" t="str">
-        <v>628f1d8e-a466-43bb-8e5c-4876365a6096.jpg</v>
-      </c>
-      <c r="J44" t="str">
-        <v/>
+        <v>images/628f1d8e-a466-43bb-8e5c-4876365a6096.jpg</v>
       </c>
       <c r="K44" t="str">
         <v/>
@@ -2204,8 +2075,8 @@
         <v xml:space="preserve">Margin -34 to 42
 Alterable</v>
       </c>
-      <c r="M44" t="str">
-        <v>No</v>
+      <c r="M44" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="45">
@@ -2227,17 +2098,14 @@
       <c r="F45">
         <v>35</v>
       </c>
-      <c r="G45" t="str">
-        <v>INSTOCK</v>
+      <c r="G45">
+        <v>20</v>
       </c>
       <c r="H45" t="str">
-        <v/>
+        <v>INSTOCK</v>
       </c>
       <c r="I45" t="str">
-        <v>da52d908-0880-4f1d-9f67-284a718958ce.jpg</v>
-      </c>
-      <c r="J45" t="str">
-        <v/>
+        <v>images/da52d908-0880-4f1d-9f67-284a718958ce.jpg</v>
       </c>
       <c r="K45" t="str">
         <v/>
@@ -2245,8 +2113,8 @@
       <c r="L45" t="str">
         <v/>
       </c>
-      <c r="M45" t="str">
-        <v>No</v>
+      <c r="M45" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="46">
@@ -2268,17 +2136,14 @@
       <c r="F46">
         <v>30</v>
       </c>
-      <c r="G46" t="str">
-        <v>INSTOCK</v>
+      <c r="G46">
+        <v>13</v>
       </c>
       <c r="H46" t="str">
-        <v/>
+        <v>INSTOCK</v>
       </c>
       <c r="I46" t="str">
-        <v>4d5b216e-8aef-41dc-a65e-b54c4a1709ef.jpg</v>
-      </c>
-      <c r="J46" t="str">
-        <v>af387eb5-0ddd-42c9-ab3d-106eba12725c.jpg</v>
+        <v>images/4d5b216e-8aef-41dc-a65e-b54c4a1709ef.jpg</v>
       </c>
       <c r="K46" t="str">
         <v/>
@@ -2286,8 +2151,8 @@
       <c r="L46" t="str">
         <v/>
       </c>
-      <c r="M46" t="str">
-        <v>No</v>
+      <c r="M46" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="47">
@@ -2309,17 +2174,14 @@
       <c r="F47">
         <v>36</v>
       </c>
-      <c r="G47" t="str">
-        <v>INSTOCK</v>
+      <c r="G47">
+        <v>18</v>
       </c>
       <c r="H47" t="str">
-        <v/>
+        <v>INSTOCK</v>
       </c>
       <c r="I47" t="str">
-        <v>429ab56c-c1ab-48e7-b73f-013faa1af682.jpg</v>
-      </c>
-      <c r="J47" t="str">
-        <v>dac18abe-3775-46dd-9807-e1a9071f97e2.jpg</v>
+        <v>images/429ab56c-c1ab-48e7-b73f-013faa1af682.jpg</v>
       </c>
       <c r="K47" t="str">
         <v/>
@@ -2327,8 +2189,8 @@
       <c r="L47" t="str">
         <v/>
       </c>
-      <c r="M47" t="str">
-        <v>No</v>
+      <c r="M47" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="48">
@@ -2350,26 +2212,23 @@
       <c r="F48">
         <v>115</v>
       </c>
-      <c r="G48" t="str">
-        <v>INSTOCK</v>
+      <c r="G48">
+        <v>14</v>
       </c>
       <c r="H48" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="I48" t="str">
+        <v>images/4520a6aa-2043-4f3f-8a5f-ffed176ef87e.jpg</v>
+      </c>
+      <c r="K48" t="str">
         <v>BLOUSE -FREE SIZE</v>
-      </c>
-      <c r="I48" t="str">
-        <v>4520a6aa-2043-4f3f-8a5f-ffed176ef87e.jpg</v>
-      </c>
-      <c r="J48" t="str">
-        <v/>
-      </c>
-      <c r="K48" t="str">
-        <v/>
       </c>
       <c r="L48" t="str">
         <v>Fully stitched blouse and skirt.</v>
       </c>
-      <c r="M48" t="str">
-        <v>No</v>
+      <c r="M48" t="b">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Restore all 46 real products with full details and image files
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M48"/>
+  <dimension ref="A1:M47"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2193,47 +2193,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" t="str">
-        <v>LW-28</v>
-      </c>
-      <c r="B48" t="str">
-        <v>Premium  silk davani set</v>
-      </c>
-      <c r="C48" t="str">
-        <v>Ladies Wear</v>
-      </c>
-      <c r="D48" t="str">
-        <v/>
-      </c>
-      <c r="E48">
-        <v>99</v>
-      </c>
-      <c r="F48">
-        <v>115</v>
-      </c>
-      <c r="G48">
-        <v>14</v>
-      </c>
-      <c r="H48" t="str">
-        <v>INSTOCK</v>
-      </c>
-      <c r="I48" t="str">
-        <v>images/4520a6aa-2043-4f3f-8a5f-ffed176ef87e.jpg</v>
-      </c>
-      <c r="K48" t="str">
-        <v>BLOUSE -FREE SIZE</v>
-      </c>
-      <c r="L48" t="str">
-        <v>Fully stitched blouse and skirt.</v>
-      </c>
-      <c r="M48" t="b">
-        <v>0</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M48"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M47"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update store products via Admin Panel - 03/08/2026, 14:08:22
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -397,131 +397,142 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M47"/>
+  <dimension ref="A1:M46"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>code</v>
+        <v>Product Code</v>
       </c>
       <c r="B1" t="str">
-        <v>name</v>
+        <v>Product Name</v>
       </c>
       <c r="C1" t="str">
-        <v>category</v>
+        <v>Category</v>
       </c>
       <c r="D1" t="str">
-        <v>subcategory</v>
+        <v>Subcategory</v>
       </c>
       <c r="E1" t="str">
-        <v>price</v>
+        <v>Price</v>
       </c>
       <c r="F1" t="str">
-        <v>originalPrice</v>
+        <v>Original Price</v>
       </c>
       <c r="G1" t="str">
-        <v>discountPct</v>
+        <v>Stock Status</v>
       </c>
       <c r="H1" t="str">
-        <v>stockStatus</v>
+        <v>Size</v>
       </c>
       <c r="I1" t="str">
-        <v>image</v>
+        <v>Image 1</v>
       </c>
       <c r="J1" t="str">
-        <v>images</v>
+        <v>Image 2</v>
       </c>
       <c r="K1" t="str">
-        <v>size</v>
+        <v>Image 3</v>
       </c>
       <c r="L1" t="str">
-        <v>description</v>
+        <v>Description</v>
       </c>
       <c r="M1" t="str">
-        <v>featured</v>
-      </c>
-    </row>
-    <row r="2">
+        <v>Featured</v>
+      </c>
+    </row>
+    <row r="2" xml:space="preserve">
       <c r="A2" t="str">
         <v>JW-01</v>
       </c>
       <c r="B2" t="str">
-        <v>Jimukka</v>
+        <v>Premium Adjustable Choker Necklace</v>
       </c>
       <c r="C2" t="str">
         <v>Jewellery</v>
       </c>
       <c r="D2" t="str">
-        <v>Earring</v>
+        <v>Necklace</v>
       </c>
       <c r="E2">
-        <v>6</v>
+        <v>29</v>
       </c>
       <c r="F2">
-        <v>10</v>
-      </c>
-      <c r="G2">
-        <v>40</v>
+        <v>36</v>
+      </c>
+      <c r="G2" t="str">
+        <v>INSTOCK</v>
       </c>
       <c r="H2" t="str">
-        <v>INSTOCK</v>
+        <v/>
       </c>
       <c r="I2" t="str">
-        <v>images/1.jpeg</v>
+        <v>67a1e7d8-1fd4-4420-971b-f4acbc6fc58f.jpg</v>
+      </c>
+      <c r="J2" t="str">
+        <v/>
       </c>
       <c r="K2" t="str">
         <v/>
       </c>
-      <c r="L2" t="str">
-        <v>Add a touch of tradition without breaking the budget! 💛 Our beautiful Jimukkas are available in a variety of stunning shades to perfectly match your outfit.  🌸 Affordable • Stylish • Perfect for Every Occasion.</v>
-      </c>
-      <c r="M2" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3">
+      <c r="L2" t="str" xml:space="preserve">
+        <v xml:space="preserve">A beautifully crafted choker necklace featuring elegant green stones and a comfortable adjustable thread closure. The perfect statement piece for sarees, lehengas, weddings, festive occasions, and traditional celebrations. 💚✨
+🌿 Available in different stone shades</v>
+      </c>
+      <c r="M2" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="3" xml:space="preserve">
       <c r="A3" t="str">
-        <v>JW-02</v>
+        <v>LW-02</v>
       </c>
       <c r="B3" t="str">
-        <v>Necklace</v>
+        <v>Soft Organza Floral Saree</v>
       </c>
       <c r="C3" t="str">
-        <v>Jewellery</v>
+        <v>Ladies Wear</v>
       </c>
       <c r="D3" t="str">
-        <v>Necklace</v>
+        <v/>
       </c>
       <c r="E3">
-        <v>29</v>
+        <v>74</v>
       </c>
       <c r="F3">
-        <v>35</v>
-      </c>
-      <c r="G3">
-        <v>17</v>
+        <v>86</v>
+      </c>
+      <c r="G3" t="str">
+        <v>INSTOCK</v>
       </c>
       <c r="H3" t="str">
-        <v>INSTOCK</v>
+        <v/>
       </c>
       <c r="I3" t="str">
-        <v>images/4.jpeg</v>
+        <v>ab9d7274-8489-4076-b611-25fd125fad6e.jpg</v>
+      </c>
+      <c r="J3" t="str">
+        <v/>
       </c>
       <c r="K3" t="str">
         <v/>
       </c>
-      <c r="L3" t="str">
-        <v>A beautifully crafted choker necklace featuring elegant green stones and a comfortable adjustable thread closure. The perfect statement piece for sarees, lehengas, weddings, festive occasions, and traditional celebrations. 💚✨</v>
-      </c>
-      <c r="M3" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4">
+      <c r="L3" t="str" xml:space="preserve">
+        <v xml:space="preserve">Grace meets elegance in this dreamy Soft Organza Saree, adorned with delicate floral prints and a beautifully finished scalloped border. Perfect for festive celebrations, parties, and special occasions. 🌸
+🌿 Soft &amp; lightweight fabric
+🌸 Elegant floral design
+✨ Beautiful scalloped border
+💖 Limited pieces available</v>
+      </c>
+      <c r="M3" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="4" xml:space="preserve">
       <c r="A4" t="str">
         <v>LW-03</v>
       </c>
       <c r="B4" t="str">
-        <v>Organza Floral Saree</v>
+        <v>Mul Chanderi 3-Piece Suit Set</v>
       </c>
       <c r="C4" t="str">
         <v>Ladies Wear</v>
@@ -530,226 +541,252 @@
         <v/>
       </c>
       <c r="E4">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="F4">
-        <v>90</v>
-      </c>
-      <c r="G4">
-        <v>18</v>
+        <v>80</v>
+      </c>
+      <c r="G4" t="str">
+        <v>INSTOCK</v>
       </c>
       <c r="H4" t="str">
-        <v>INSTOCK</v>
+        <v>44</v>
       </c>
       <c r="I4" t="str">
-        <v>images/5.jpeg</v>
+        <v>875ccf12-ab69-4093-ae53-63765a3a2896.jpg</v>
+      </c>
+      <c r="J4" t="str">
+        <v/>
       </c>
       <c r="K4" t="str">
         <v/>
       </c>
-      <c r="L4" t="str">
-        <v>Grace meets elegance in this dreamy Soft Organza Saree, adorned with delicate floral prints and a beautifully finished scalloped border. Perfect for festive celebrations, parties, and special occasions. 🌸</v>
-      </c>
-      <c r="M4" t="b">
-        <v>0</v>
+      <c r="L4" t="str" xml:space="preserve">
+        <v xml:space="preserve">Graceful, lightweight, and effortlessly elegant. This beautiful Mul Chanderi 3-piece set features delicate embroidery with a matching bottom and soft dupatta—perfect for festive celebrations, family gatherings, and everyday elegance. 💕
+🌸 Premium Mul Chanderi fabric
+✨ Elegant embroidery
+🧣 Matching dupatta &amp; bottom included
+💖 Limited pieces available</v>
+      </c>
+      <c r="M4" t="str">
+        <v>No</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>LW-04</v>
+        <v>KW-01</v>
       </c>
       <c r="B5" t="str">
-        <v>Chanderi 3-Piece Suit Set</v>
+        <v>Kids Pattu Pavada Set</v>
       </c>
       <c r="C5" t="str">
-        <v>Ladies Wear</v>
+        <v>Kids Wear</v>
       </c>
       <c r="D5" t="str">
         <v/>
       </c>
       <c r="E5">
-        <v>68</v>
+        <v>45</v>
       </c>
       <c r="F5">
-        <v>68</v>
-      </c>
-      <c r="G5">
-        <v>0</v>
+        <v>56</v>
+      </c>
+      <c r="G5" t="str">
+        <v>INSTOCK</v>
       </c>
       <c r="H5" t="str">
-        <v>INSTOCK</v>
+        <v>3 yrs /5yrs /6yrs</v>
       </c>
       <c r="I5" t="str">
-        <v>images/6.jpeg</v>
+        <v>63d7a112-b27b-4944-8795-30941a5a1955.jpg</v>
+      </c>
+      <c r="J5" t="str">
+        <v/>
       </c>
       <c r="K5" t="str">
         <v/>
       </c>
       <c r="L5" t="str">
-        <v>Graceful, lightweight, and effortlessly elegant. This beautiful Mul Chanderi 3-piece set features delicate embroidery with a matching bottom and soft dupatta—perfect for festive celebrations, family gatherings, and everyday elegance  SIZE TILL 44</v>
-      </c>
-      <c r="M5" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6">
+        <v>Celebrate every special moment in timeless tradition! ❤️ This elegant Kids Pattu Pavada features a beautifully printed lotus skirt with a rich maroon puff-sleeve blouse, making it a perfect choice for Onam, festivals, temple visits, and family celebrations.</v>
+      </c>
+      <c r="M5" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="6" xml:space="preserve">
       <c r="A6" t="str">
-        <v>KW-05</v>
+        <v>JW-02</v>
       </c>
       <c r="B6" t="str">
-        <v>Kids Pattu Pavada Set</v>
+        <v>Ruby Antique Choker</v>
       </c>
       <c r="C6" t="str">
-        <v>Kids Wear</v>
+        <v>Jewellery</v>
       </c>
       <c r="D6" t="str">
-        <v/>
+        <v>Necklace</v>
       </c>
       <c r="E6">
-        <v>45</v>
+        <v>29</v>
       </c>
       <c r="F6">
-        <v>50</v>
-      </c>
-      <c r="G6">
-        <v>10</v>
+        <v>39</v>
+      </c>
+      <c r="G6" t="str">
+        <v>INSTOCK</v>
       </c>
       <c r="H6" t="str">
-        <v>INSTOCK</v>
+        <v/>
       </c>
       <c r="I6" t="str">
-        <v>images/7.jpeg</v>
+        <v>a1076eed-fc2e-41cc-b5f0-ef19263e1051.jpg</v>
+      </c>
+      <c r="J6" t="str">
+        <v/>
       </c>
       <c r="K6" t="str">
         <v/>
       </c>
-      <c r="L6" t="str">
-        <v>Celebrate every special moment in timeless tradition! ❤️ This elegant Kids Pattu Pavada features a beautifully printed lotus skirt with a rich maroon puff-sleeve blouse, making it a perfect choice for Onam, festivals, temple visits, and family celebrations. Size -3 yrs /5yrs /6yrs</v>
-      </c>
-      <c r="M6" t="b">
-        <v>0</v>
+      <c r="L6" t="str" xml:space="preserve">
+        <v xml:space="preserve">A graceful antique-finish choker adorned with rich ruby stones, crafted to add timeless elegance to your festive and bridal look.
+❤️ Perfect for weddings, festive wear &amp; Kerala sarees.</v>
+      </c>
+      <c r="M6" t="str">
+        <v>No</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>JW-06</v>
+        <v>LW-04</v>
       </c>
       <c r="B7" t="str">
-        <v>Ruby Antique Choke</v>
+        <v>Semi Tusser Saree</v>
       </c>
       <c r="C7" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D7" t="str">
+        <v/>
+      </c>
+      <c r="E7">
+        <v>80</v>
+      </c>
+      <c r="F7">
+        <v>100</v>
+      </c>
+      <c r="G7" t="str">
+        <v>LIMITED STOCK</v>
+      </c>
+      <c r="H7" t="str">
+        <v/>
+      </c>
+      <c r="I7" t="str">
+        <v>e6914ddc-d37f-4dc0-bf7d-3b930bbccf2e.jpg</v>
+      </c>
+      <c r="J7" t="str">
+        <v/>
+      </c>
+      <c r="K7" t="str">
+        <v/>
+      </c>
+      <c r="L7" t="str">
+        <v>Rich wine-red semi tusser saree featuring an exquisite floral embroidered lace border. Elegant, lightweight, and perfect for festive celebrations, weddings, and special occasions.</v>
+      </c>
+      <c r="M7" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="8" xml:space="preserve">
+      <c r="A8" t="str">
+        <v>JW-03</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Nagapadam Necklace Set</v>
+      </c>
+      <c r="C8" t="str">
         <v>Jewellery</v>
       </c>
-      <c r="D7" t="str">
+      <c r="D8" t="str">
         <v>Necklace</v>
       </c>
-      <c r="E7">
-        <v>29</v>
-      </c>
-      <c r="F7">
-        <v>41</v>
-      </c>
-      <c r="G7">
-        <v>29</v>
-      </c>
-      <c r="H7" t="str">
-        <v>INSTOCK</v>
-      </c>
-      <c r="I7" t="str">
-        <v>images/8.jpg</v>
-      </c>
-      <c r="K7" t="str">
-        <v/>
-      </c>
-      <c r="L7" t="str">
-        <v>A beautifully crafted choker necklace featuring elegant green stones and a comfortable adjustable thread closure. The perfect statement piece for sarees, lehengas, weddings, festive occasions, and traditional celebrations. 💚✨</v>
-      </c>
-      <c r="M7" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>LW-07</v>
-      </c>
-      <c r="B8" t="str">
+      <c r="E8">
+        <v>30</v>
+      </c>
+      <c r="F8">
+        <v>45</v>
+      </c>
+      <c r="G8" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H8" t="str">
+        <v/>
+      </c>
+      <c r="I8" t="str">
+        <v>a59617a0-1ae8-4e5b-b364-2274db188b3f.jpg</v>
+      </c>
+      <c r="J8" t="str">
+        <v/>
+      </c>
+      <c r="K8" t="str">
+        <v/>
+      </c>
+      <c r="L8" t="str" xml:space="preserve">
+        <v xml:space="preserve">A timeless Nagapadam necklace with matching jhumkas, beautifully crafted in royal blue and emerald green for a graceful traditional look.
+Perfect for: Kerala sarees, set mundu, weddings &amp; festive occasions.
+Limited pieces available.</v>
+      </c>
+      <c r="M8" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="9" xml:space="preserve">
+      <c r="A9" t="str">
+        <v>JW-04</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Jimukka</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Jewellery</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Earring</v>
+      </c>
+      <c r="E9">
+        <v>6</v>
+      </c>
+      <c r="F9">
+        <v>10</v>
+      </c>
+      <c r="G9" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H9" t="str">
+        <v/>
+      </c>
+      <c r="I9" t="str">
+        <v>e23c987b-36da-4a76-b090-823e2d5d6d7c.jpg</v>
+      </c>
+      <c r="J9" t="str">
+        <v>6d320665-0057-4a58-b01e-2ded9a2c6dd1.jpg</v>
+      </c>
+      <c r="K9" t="str">
+        <v>385b2f68-1591-4763-a432-1299e0d8f609.jpg</v>
+      </c>
+      <c r="L9" t="str" xml:space="preserve">
+        <v xml:space="preserve">Budjet friendly Jimukka 
+ Available in different shades</v>
+      </c>
+      <c r="M9" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="10" xml:space="preserve">
+      <c r="A10" t="str">
+        <v>LW-05</v>
+      </c>
+      <c r="B10" t="str">
         <v>Soft Tissue Saree</v>
-      </c>
-      <c r="C8" t="str">
-        <v>Ladies Wear</v>
-      </c>
-      <c r="D8" t="str">
-        <v/>
-      </c>
-      <c r="E8">
-        <v>68</v>
-      </c>
-      <c r="F8">
-        <v>83</v>
-      </c>
-      <c r="G8">
-        <v>18</v>
-      </c>
-      <c r="H8" t="str">
-        <v>INSTOCK</v>
-      </c>
-      <c r="I8" t="str">
-        <v>images/9.jpeg</v>
-      </c>
-      <c r="K8" t="str">
-        <v/>
-      </c>
-      <c r="L8" t="str">
-        <v>Grace meets tradition in this elegant soft tissue saree, beautifully finished with a stunning floral Kalamkari-inspired border. A timeless choice for festive celebrations and special occasions.</v>
-      </c>
-      <c r="M8" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>GW-08</v>
-      </c>
-      <c r="B9" t="str">
-        <v>Men’s Kurta</v>
-      </c>
-      <c r="C9" t="str">
-        <v>Men's Wear</v>
-      </c>
-      <c r="D9" t="str">
-        <v/>
-      </c>
-      <c r="E9">
-        <v>62</v>
-      </c>
-      <c r="F9">
-        <v>70</v>
-      </c>
-      <c r="G9">
-        <v>11</v>
-      </c>
-      <c r="H9" t="str">
-        <v>INSTOCK</v>
-      </c>
-      <c r="I9" t="str">
-        <v>images/10.jpeg</v>
-      </c>
-      <c r="K9" t="str">
-        <v/>
-      </c>
-      <c r="L9" t="str">
-        <v>Make a statement with this elegant premium embroidered kurta, crafted for weddings, festivals, and special occasions.</v>
-      </c>
-      <c r="M9" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>LW-09</v>
-      </c>
-      <c r="B10" t="str">
-        <v>Cotton Embroidered Blouse</v>
       </c>
       <c r="C10" t="str">
         <v>Ladies Wear</v>
@@ -758,36 +795,40 @@
         <v/>
       </c>
       <c r="E10">
-        <v>35</v>
+        <v>58</v>
       </c>
       <c r="F10">
-        <v>43</v>
-      </c>
-      <c r="G10">
-        <v>19</v>
+        <v>60</v>
+      </c>
+      <c r="G10" t="str">
+        <v>LIMITED STOCK</v>
       </c>
       <c r="H10" t="str">
-        <v>INSTOCK</v>
+        <v/>
       </c>
       <c r="I10" t="str">
-        <v>images/11.jpeg</v>
+        <v>5dcf9d33-94b4-4fcc-a36d-48c593a9d9f9.jpg</v>
+      </c>
+      <c r="J10" t="str">
+        <v>8764d90f-7020-4bd3-8031-5d35f330d75c.jpg</v>
       </c>
       <c r="K10" t="str">
-        <v/>
-      </c>
-      <c r="L10" t="str">
-        <v>Elevate your saree look with our elegant free-size embroidered blouse, designed for both comfort and style. Free size – Fits 36–42 inches (with alteration margin)</v>
-      </c>
-      <c r="M10" t="b">
-        <v>0</v>
+        <v>25c00901-eb8b-4011-9a29-9be4d224135e.jpg</v>
+      </c>
+      <c r="L10" t="str" xml:space="preserve">
+        <v xml:space="preserve">Light as a breeze, elegant in every drape. A soft tissue saree with beautiful lotus floral prints and a matching blouse piece—perfect for festive and special occasions.
+Limited pieces available.</v>
+      </c>
+      <c r="M10" t="str">
+        <v>No</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>JW-10</v>
+        <v>JW-05</v>
       </c>
       <c r="B11" t="str">
-        <v>AD Pendant (Without Chain)</v>
+        <v>Emerald Antique Pendant Set</v>
       </c>
       <c r="C11" t="str">
         <v>Jewellery</v>
@@ -796,33 +837,36 @@
         <v>Pendants</v>
       </c>
       <c r="E11">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F11">
-        <v>35</v>
-      </c>
-      <c r="G11">
-        <v>20</v>
+        <v>45</v>
+      </c>
+      <c r="G11" t="str">
+        <v>LIMITED STOCK</v>
       </c>
       <c r="H11" t="str">
-        <v>LIMITED STOCK</v>
+        <v/>
       </c>
       <c r="I11" t="str">
-        <v>images/14.jpeg</v>
+        <v>690cf14c-289b-48eb-bcbf-ddbc5b143df3.jpg</v>
+      </c>
+      <c r="J11" t="str">
+        <v>700adc94-fc82-4a87-b0da-cac54f4c5c6e.jpg</v>
       </c>
       <c r="K11" t="str">
         <v/>
       </c>
       <c r="L11" t="str">
-        <v>A sparkling American Diamond pendant with matching earrings, designed to add effortless elegance to your look. Pair it with your favourite chain for a personalized style.</v>
-      </c>
-      <c r="M11" t="b">
-        <v>0</v>
+        <v>A graceful antique-finish pendant set featuring a stunning emerald-green stone with matching earrings. Perfect for adding timeless elegance to your ethnic look.</v>
+      </c>
+      <c r="M11" t="str">
+        <v>No</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>JW-11</v>
+        <v>JW-06</v>
       </c>
       <c r="B12" t="str">
         <v>Antique Pendant Set</v>
@@ -837,16 +881,19 @@
         <v>30</v>
       </c>
       <c r="F12">
-        <v>36</v>
-      </c>
-      <c r="G12">
-        <v>17</v>
+        <v>45</v>
+      </c>
+      <c r="G12" t="str">
+        <v>INSTOCK</v>
       </c>
       <c r="H12" t="str">
-        <v>LIMITED STOCK</v>
+        <v/>
       </c>
       <c r="I12" t="str">
-        <v>images/16.jpeg</v>
+        <v>36ecbdd8-bf43-454d-95b5-1ef07e8782f2.jpg</v>
+      </c>
+      <c r="J12" t="str">
+        <v>072b44aa-d196-461e-8f36-f658eeb7f9e7.jpg</v>
       </c>
       <c r="K12" t="str">
         <v/>
@@ -854,16 +901,16 @@
       <c r="L12" t="str">
         <v>A stunning antique-finish pendant set accented with rich purple stones and matching earrings. Designed to bring a touch of vintage elegance to every festive look.</v>
       </c>
-      <c r="M12" t="b">
-        <v>0</v>
+      <c r="M12" t="str">
+        <v>No</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>JW-12</v>
+        <v>JW-07</v>
       </c>
       <c r="B13" t="str">
-        <v>Emerald Antique Pendant Set</v>
+        <v>AD Pendant (Without Chain)</v>
       </c>
       <c r="C13" t="str">
         <v>Jewellery</v>
@@ -872,36 +919,39 @@
         <v>Pendants</v>
       </c>
       <c r="E13">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="F13">
-        <v>49</v>
-      </c>
-      <c r="G13">
-        <v>39</v>
+        <v>28</v>
+      </c>
+      <c r="G13" t="str">
+        <v>INSTOCK</v>
       </c>
       <c r="H13" t="str">
-        <v>LIMITED STOCK</v>
+        <v/>
       </c>
       <c r="I13" t="str">
-        <v>images/18.jpeg</v>
+        <v>06d90bdb-d79a-4dad-935e-1e5928889944.jpg</v>
+      </c>
+      <c r="J13" t="str">
+        <v>406879f9-9d7d-49cd-a00c-0092446d9745.jpg</v>
       </c>
       <c r="K13" t="str">
         <v/>
       </c>
       <c r="L13" t="str">
-        <v>A graceful antique-finish pendant set featuring a stunning emerald-green stone with matching earrings. Perfect for adding timeless elegance to your ethnic look.</v>
-      </c>
-      <c r="M13" t="b">
-        <v>0</v>
+        <v/>
+      </c>
+      <c r="M13" t="str">
+        <v>No</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>LW-13</v>
+        <v>LW-06</v>
       </c>
       <c r="B14" t="str">
-        <v>Soft Tissue Saree</v>
+        <v>Premium Cotton Embroidered Blouse</v>
       </c>
       <c r="C14" t="str">
         <v>Ladies Wear</v>
@@ -910,74 +960,83 @@
         <v/>
       </c>
       <c r="E14">
-        <v>58</v>
+        <v>35</v>
       </c>
       <c r="F14">
-        <v>63</v>
-      </c>
-      <c r="G14">
-        <v>8</v>
+        <v>35</v>
+      </c>
+      <c r="G14" t="str">
+        <v>INSTOCK</v>
       </c>
       <c r="H14" t="str">
-        <v>INSTOCK</v>
+        <v/>
       </c>
       <c r="I14" t="str">
-        <v>images/20.jpeg</v>
+        <v>1cd8f0bb-4162-4424-ab71-0447fe5bbc8e.jpg</v>
+      </c>
+      <c r="J14" t="str">
+        <v>316cece8-ed12-4b8e-b930-e02eb1f4f643.jpg</v>
       </c>
       <c r="K14" t="str">
-        <v/>
+        <v>10ab4c9a-7855-40f5-bb4b-23a50b41b728.jpg</v>
       </c>
       <c r="L14" t="str">
-        <v>Light as a breeze, elegant in every drape. A soft tissue saree with beautiful lotus floral prints and a matching blouse piece—perfect for festive and special occasions.</v>
-      </c>
-      <c r="M14" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15">
+        <v/>
+      </c>
+      <c r="M14" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="15" xml:space="preserve">
       <c r="A15" t="str">
-        <v>JW-13</v>
+        <v>GW-01</v>
       </c>
       <c r="B15" t="str">
-        <v>Nagapadam Necklace Set</v>
+        <v>Premium Men’s Kurta</v>
       </c>
       <c r="C15" t="str">
-        <v>Jewellery</v>
+        <v>Mens Wear</v>
       </c>
       <c r="D15" t="str">
-        <v>Necklace</v>
+        <v/>
       </c>
       <c r="E15">
-        <v>30</v>
+        <v>62</v>
       </c>
       <c r="F15">
-        <v>36</v>
-      </c>
-      <c r="G15">
-        <v>17</v>
+        <v>62</v>
+      </c>
+      <c r="G15" t="str">
+        <v>LIMITED STOCK</v>
       </c>
       <c r="H15" t="str">
-        <v>INSTOCK</v>
+        <v/>
       </c>
       <c r="I15" t="str">
-        <v>images/23.jpeg</v>
+        <v>9767ca6f-f214-48ec-94b7-b5895ef0c285.jpg</v>
+      </c>
+      <c r="J15" t="str">
+        <v/>
       </c>
       <c r="K15" t="str">
         <v/>
       </c>
-      <c r="L15" t="str">
-        <v>A timeless Nagapadam necklace with matching jhumkas, beautifully crafted in royal blue and emerald green for a graceful traditional look.</v>
-      </c>
-      <c r="M15" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16">
+      <c r="L15" t="str" xml:space="preserve">
+        <v xml:space="preserve">Make a statement with this elegant premium embroidered kurta, crafted for weddings, festivals, and special occasions.
+✨ Rich detailing
+✨ Comfortable fit
+✨ Perfect for festive celebrations</v>
+      </c>
+      <c r="M15" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="16" xml:space="preserve">
       <c r="A16" t="str">
-        <v>JW-15</v>
+        <v>LW-07</v>
       </c>
       <c r="B16" t="str">
-        <v>Semi Tusser Saree</v>
+        <v>Premium Soft Tissue Saree</v>
       </c>
       <c r="C16" t="str">
         <v>Ladies Wear</v>
@@ -986,74 +1045,84 @@
         <v/>
       </c>
       <c r="E16">
-        <v>80</v>
+        <v>68</v>
       </c>
       <c r="F16">
-        <v>100</v>
-      </c>
-      <c r="G16">
-        <v>20</v>
+        <v>68</v>
+      </c>
+      <c r="G16" t="str">
+        <v>LIMITED STOCK</v>
       </c>
       <c r="H16" t="str">
-        <v>INSTOCK</v>
+        <v/>
       </c>
       <c r="I16" t="str">
-        <v>images/24.jpeg</v>
+        <v>3c07c2fc-3597-449d-a572-1f6f136e5b9d.jpg</v>
+      </c>
+      <c r="J16" t="str">
+        <v/>
       </c>
       <c r="K16" t="str">
         <v/>
       </c>
-      <c r="L16" t="str">
-        <v>Rich wine-red semi tusser saree featuring an exquisite floral embroidered lace border. Elegant, lightweight, and perfect for festive celebrations, weddings, and special occasions.</v>
-      </c>
-      <c r="M16" t="b">
-        <v>0</v>
+      <c r="L16" t="str" xml:space="preserve">
+        <v xml:space="preserve">Grace meets tradition in this elegant soft tissue saree, beautifully finished with a stunning floral Kalamkari-inspired border. A timeless choice for festive celebrations and special occasions.
+✨ Soft &amp; lightweight
+✨ Elegant floral border
+✨ Matching blouse piece included
+✨ Limited pieces available 🌸</v>
+      </c>
+      <c r="M16" t="str">
+        <v>No</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>JW-16</v>
+        <v>LW-08</v>
       </c>
       <c r="B17" t="str">
-        <v>flower ear rings</v>
+        <v>Maroon Soft Premium Warm Silk Saree</v>
       </c>
       <c r="C17" t="str">
-        <v>Jewellery</v>
+        <v>Ladies Wear</v>
       </c>
       <c r="D17" t="str">
-        <v>Earring</v>
+        <v/>
       </c>
       <c r="E17">
-        <v>21</v>
+        <v>89</v>
       </c>
       <c r="F17">
-        <v>28</v>
-      </c>
-      <c r="G17">
-        <v>25</v>
+        <v>115</v>
+      </c>
+      <c r="G17" t="str">
+        <v>INSTOCK</v>
       </c>
       <c r="H17" t="str">
-        <v>LIMITED STOCK</v>
+        <v/>
       </c>
       <c r="I17" t="str">
-        <v>images/e2a2ec34-dc2e-4090-b325-67b69445b9dd.jpg</v>
+        <v>542e9d71-6c39-4b17-af9f-a06a05fa946e.jpg</v>
+      </c>
+      <c r="J17" t="str">
+        <v>23a7c2fe-96ff-4818-b74a-e5c7417baca6.jpg</v>
       </c>
       <c r="K17" t="str">
-        <v/>
+        <v>1e798955-e174-4045-8af1-3dda1f00cfee.jpg</v>
       </c>
       <c r="L17" t="str">
         <v/>
       </c>
-      <c r="M17" t="b">
-        <v>0</v>
+      <c r="M17" t="str">
+        <v>No</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>LW-14</v>
+        <v>LW-09</v>
       </c>
       <c r="B18" t="str">
-        <v>Silk Saree</v>
+        <v>Royal Green Brocade Blouse</v>
       </c>
       <c r="C18" t="str">
         <v>Ladies Wear</v>
@@ -1062,74 +1131,80 @@
         <v/>
       </c>
       <c r="E18">
-        <v>89</v>
+        <v>42</v>
       </c>
       <c r="F18">
-        <v>110</v>
-      </c>
-      <c r="G18">
-        <v>19</v>
+        <v>56</v>
+      </c>
+      <c r="G18" t="str">
+        <v>INSTOCK</v>
       </c>
       <c r="H18" t="str">
-        <v>INSTOCK</v>
+        <v/>
       </c>
       <c r="I18" t="str">
-        <v>images/e67c8e99-625e-4772-b3cc-daeca03c1dd4.jpg</v>
+        <v>1c6eb980-39da-4172-b041-8c6e03ffd5c7.jpg</v>
+      </c>
+      <c r="J18" t="str">
+        <v/>
       </c>
       <c r="K18" t="str">
         <v/>
       </c>
       <c r="L18" t="str">
-        <v>A rich maroon saree featuring an elegant gold saree border and beautifully woven traditional motifs—perfect for weddings, festive occasions and celebrations.</v>
-      </c>
-      <c r="M18" t="b">
-        <v>0</v>
+        <v>A rich emerald-green blouse featuring elegant gold floral weaving and a stylish tie-back detail—perfect for pairing with silk, tissue, or festive sarees.</v>
+      </c>
+      <c r="M18" t="str">
+        <v>No</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>LW-15</v>
+        <v>JW-08</v>
       </c>
       <c r="B19" t="str">
-        <v>Royal Green Brocade Blouse</v>
+        <v>Traditional Stone Choker</v>
       </c>
       <c r="C19" t="str">
-        <v>Ladies Wear</v>
+        <v>Jewellery</v>
       </c>
       <c r="D19" t="str">
-        <v/>
+        <v>Necklace</v>
       </c>
       <c r="E19">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="F19">
-        <v>50</v>
-      </c>
-      <c r="G19">
-        <v>16</v>
+        <v>44</v>
+      </c>
+      <c r="G19" t="str">
+        <v>INSTOCK</v>
       </c>
       <c r="H19" t="str">
-        <v>INSTOCK</v>
+        <v/>
       </c>
       <c r="I19" t="str">
-        <v>images/eb7df1cd-6b0d-42f9-9be7-44d51c6d527e.jpg</v>
+        <v>aa8e3572-1a6c-43dc-8b15-7329f37dabdd.jpg</v>
+      </c>
+      <c r="J19" t="str">
+        <v/>
       </c>
       <c r="K19" t="str">
         <v/>
       </c>
       <c r="L19" t="str">
-        <v>A rich emerald-green blouse featuring elegant gold floral weaving and a stylish tie-back detail—perfect for pairing with silk, tissue, or festive sarees.</v>
-      </c>
-      <c r="M19" t="b">
-        <v>0</v>
+        <v/>
+      </c>
+      <c r="M19" t="str">
+        <v>No</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>JW-17</v>
+        <v>JW-09</v>
       </c>
       <c r="B20" t="str">
-        <v>Traditional Stone Choker</v>
+        <v>Ruby Radiance Necklace Set</v>
       </c>
       <c r="C20" t="str">
         <v>Jewellery</v>
@@ -1138,36 +1213,39 @@
         <v>Necklace</v>
       </c>
       <c r="E20">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="F20">
-        <v>50</v>
-      </c>
-      <c r="G20">
-        <v>12</v>
+        <v>41</v>
+      </c>
+      <c r="G20" t="str">
+        <v>INSTOCK</v>
       </c>
       <c r="H20" t="str">
-        <v>LIMITED STOCK</v>
+        <v/>
       </c>
       <c r="I20" t="str">
-        <v>images/a1c56268-4968-4ea5-ab01-51b256c4f4a6.jpg</v>
+        <v>70583151-04aa-4080-8f72-1f24bd934e8b.jpg</v>
+      </c>
+      <c r="J20" t="str">
+        <v/>
       </c>
       <c r="K20" t="str">
         <v/>
       </c>
       <c r="L20" t="str">
-        <v>A graceful gold-toned choker adorned with ruby-green stones and sparkling accents—perfect for sarees, lehengas and festive looks.</v>
-      </c>
-      <c r="M20" t="b">
-        <v>0</v>
+        <v/>
+      </c>
+      <c r="M20" t="str">
+        <v>No</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>JW-18</v>
+        <v>JW-10</v>
       </c>
       <c r="B21" t="str">
-        <v>Ruby Radiance Necklace Set</v>
+        <v>AD Stone Choker Set</v>
       </c>
       <c r="C21" t="str">
         <v>Jewellery</v>
@@ -1176,71 +1254,77 @@
         <v>Necklace</v>
       </c>
       <c r="E21">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="F21">
-        <v>60</v>
-      </c>
-      <c r="G21">
-        <v>32</v>
+        <v>34</v>
+      </c>
+      <c r="G21" t="str">
+        <v>INSTOCK</v>
       </c>
       <c r="H21" t="str">
-        <v>LIMITED STOCK</v>
+        <v/>
       </c>
       <c r="I21" t="str">
-        <v>images/4a69a0a6-847f-4a32-83e5-743f681ad6b9.jpg</v>
+        <v>48691bd3-22d6-496d-b04c-2be03ed8d1da.jpg</v>
+      </c>
+      <c r="J21" t="str">
+        <v>02412783-b2f9-4e99-a589-bed982e832f6.jpg</v>
       </c>
       <c r="K21" t="str">
         <v/>
       </c>
       <c r="L21" t="str">
-        <v>A graceful stone-studded necklace with matching earrings—perfect for adding a rich, elegant sparkle to any special occasion.</v>
-      </c>
-      <c r="M21" t="b">
-        <v>0</v>
+        <v/>
+      </c>
+      <c r="M21" t="str">
+        <v>No</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>JW-19</v>
+        <v>LW-10</v>
       </c>
       <c r="B22" t="str">
-        <v>AD Stone Choker Set</v>
+        <v>AD necklace</v>
       </c>
       <c r="C22" t="str">
-        <v>Jewellery</v>
+        <v>Ladies Wear</v>
       </c>
       <c r="D22" t="str">
-        <v>Necklace</v>
+        <v/>
       </c>
       <c r="E22">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="F22">
-        <v>45</v>
-      </c>
-      <c r="G22">
-        <v>24</v>
+        <v>26</v>
+      </c>
+      <c r="G22" t="str">
+        <v>LIMITED STOCK</v>
       </c>
       <c r="H22" t="str">
-        <v>LIMITED STOCK</v>
+        <v/>
       </c>
       <c r="I22" t="str">
-        <v>images/3366e4f8-6047-4d0e-81ba-c81b83319764.jpg</v>
+        <v>a21f7185-c33a-4d1b-9f49-62ffb934661d.jpg</v>
+      </c>
+      <c r="J22" t="str">
+        <v>1564f3e1-98ab-4cd9-af33-4fa0430db2f6.jpg</v>
       </c>
       <c r="K22" t="str">
         <v/>
       </c>
       <c r="L22" t="str">
-        <v>A delicate gold-finish design with sparkling stones and matching studs—perfect for parties and special occasions.</v>
-      </c>
-      <c r="M22" t="b">
-        <v>0</v>
+        <v/>
+      </c>
+      <c r="M22" t="str">
+        <v>No</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>JW-20</v>
+        <v>JW-11</v>
       </c>
       <c r="B23" t="str">
         <v>Necklace</v>
@@ -1252,36 +1336,39 @@
         <v>Necklace</v>
       </c>
       <c r="E23">
-        <v>26</v>
+        <v>29.96</v>
       </c>
       <c r="F23">
-        <v>40</v>
-      </c>
-      <c r="G23">
-        <v>35</v>
+        <v>29.96</v>
+      </c>
+      <c r="G23" t="str">
+        <v>INSTOCK</v>
       </c>
       <c r="H23" t="str">
-        <v>LIMITED STOCK</v>
+        <v/>
       </c>
       <c r="I23" t="str">
-        <v>images/bfc3ccbe-db6b-494b-96a1-d4dcbb46e9a6.jpg</v>
+        <v>ff6bc646-8aef-4ee5-8140-979ca027c604.jpg</v>
+      </c>
+      <c r="J23" t="str">
+        <v/>
       </c>
       <c r="K23" t="str">
         <v/>
       </c>
       <c r="L23" t="str">
-        <v>A graceful traditional AD necklace featuring rich ruby-toned stones, a striking emerald-green centerpiece, and elegant pearl drops. Perfect for weddings, festive celebrations, and special occasions.</v>
-      </c>
-      <c r="M23" t="b">
-        <v>0</v>
+        <v/>
+      </c>
+      <c r="M23" t="str">
+        <v>No</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>JW-21</v>
+        <v>JW-12</v>
       </c>
       <c r="B24" t="str">
-        <v>Necklace</v>
+        <v>Emerald Glow Necklace Set</v>
       </c>
       <c r="C24" t="str">
         <v>Jewellery</v>
@@ -1290,75 +1377,80 @@
         <v>Necklace</v>
       </c>
       <c r="E24">
-        <v>30</v>
+        <v>37.59</v>
       </c>
       <c r="F24">
-        <v>46</v>
-      </c>
-      <c r="G24">
-        <v>35</v>
+        <v>37.59</v>
+      </c>
+      <c r="G24" t="str">
+        <v>INSTOCK</v>
       </c>
       <c r="H24" t="str">
-        <v>INSTOCK</v>
+        <v/>
       </c>
       <c r="I24" t="str">
-        <v>images/d260a0ff-0114-4653-8285-8a5afe33ec43.jpg</v>
+        <v>35f84e9d-0684-461f-8569-40c3071da669.jpg</v>
+      </c>
+      <c r="J24" t="str">
+        <v/>
       </c>
       <c r="K24" t="str">
         <v/>
       </c>
       <c r="L24" t="str">
-        <v>Elegant antique-finish necklace featuring delicate pearl florals, rich ruby-toned stones and a beautifully detailed pendant. A graceful choice for festive and traditional looks.</v>
-      </c>
-      <c r="M24" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" xml:space="preserve">
+        <v/>
+      </c>
+      <c r="M24" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="25">
       <c r="A25" t="str">
-        <v>LW-16</v>
+        <v>JW-13</v>
       </c>
       <c r="B25" t="str">
-        <v>Necklace</v>
+        <v>ruby-centred pendant</v>
       </c>
       <c r="C25" t="str">
         <v>Jewellery</v>
       </c>
       <c r="D25" t="str">
-        <v>Necklace</v>
+        <v>Pendants</v>
       </c>
       <c r="E25">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="F25">
-        <v>55</v>
-      </c>
-      <c r="G25">
-        <v>31</v>
+        <v>34</v>
+      </c>
+      <c r="G25" t="str">
+        <v>LIMITED STOCK</v>
       </c>
       <c r="H25" t="str">
-        <v>INSTOCK</v>
+        <v/>
       </c>
       <c r="I25" t="str">
-        <v>images/c129d1b5-a9d7-413e-a9ba-ed756e6b96ce.jpg</v>
+        <v>8c016b51-9123-4238-83fd-82557b1a2fdb.jpg</v>
+      </c>
+      <c r="J25" t="str">
+        <v/>
       </c>
       <c r="K25" t="str">
         <v/>
       </c>
-      <c r="L25" t="str" xml:space="preserve">
-        <v xml:space="preserve">Emerald Glow Necklace Set 💚
-A stunning emerald-green stone necklace with matching earrings, beautifully framed with sparkling accents. Perfect for festive occasions, parties and elegant traditional looks.</v>
-      </c>
-      <c r="M25" t="b">
-        <v>0</v>
+      <c r="L25" t="str">
+        <v/>
+      </c>
+      <c r="M25" t="str">
+        <v>No</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>JW-22</v>
+        <v>JW-14</v>
       </c>
       <c r="B26" t="str">
-        <v>Pearl Necklace</v>
+        <v>Necklace</v>
       </c>
       <c r="C26" t="str">
         <v>Jewellery</v>
@@ -1367,174 +1459,186 @@
         <v>Necklace</v>
       </c>
       <c r="E26">
-        <v>34</v>
+        <v>23</v>
       </c>
       <c r="F26">
-        <v>46</v>
-      </c>
-      <c r="G26">
-        <v>26</v>
+        <v>23</v>
+      </c>
+      <c r="G26" t="str">
+        <v>LIMITED STOCK</v>
       </c>
       <c r="H26" t="str">
-        <v>INSTOCK</v>
+        <v/>
       </c>
       <c r="I26" t="str">
-        <v>images/efb45acd-3a86-4179-bc43-f4ed4608590c.jpg</v>
+        <v>4f776a2a-37e2-4d7d-ba32-68fd0a6e22b8.jpg</v>
+      </c>
+      <c r="J26" t="str">
+        <v/>
       </c>
       <c r="K26" t="str">
         <v/>
       </c>
       <c r="L26" t="str">
-        <v>Pearl elegance with a radiant ruby-centred pendant—simple, graceful and timeless.</v>
-      </c>
-      <c r="M26" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" xml:space="preserve">
+        <v/>
+      </c>
+      <c r="M26" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="27">
       <c r="A27" t="str">
-        <v>JW-23</v>
+        <v>JW-15</v>
       </c>
       <c r="B27" t="str">
-        <v>Bangles with striking ruby-pink stones</v>
+        <v>Necklace</v>
       </c>
       <c r="C27" t="str">
         <v>Jewellery</v>
       </c>
       <c r="D27" t="str">
-        <v>Bangles</v>
+        <v>Necklace</v>
       </c>
       <c r="E27">
-        <v>23</v>
+        <v>34</v>
       </c>
       <c r="F27">
-        <v>32</v>
-      </c>
-      <c r="G27">
-        <v>28</v>
+        <v>34</v>
+      </c>
+      <c r="G27" t="str">
+        <v>INSTOCK</v>
       </c>
       <c r="H27" t="str">
-        <v>INSTOCK</v>
+        <v/>
       </c>
       <c r="I27" t="str">
-        <v>images/19c70259-71e8-4892-b897-5ffe5b75a8a2.jpg</v>
+        <v>9d11da56-2aaa-43f5-8454-004e0bd1ec71.jpg</v>
+      </c>
+      <c r="J27" t="str">
+        <v/>
       </c>
       <c r="K27" t="str">
         <v/>
       </c>
-      <c r="L27" t="str" xml:space="preserve">
-        <v xml:space="preserve">Elegance in every detail ✨
-Beautifully crafted gold-tone bangles with striking ruby-pink stones—perfect for adding a royal touch to any outfit.
-$12 per piece.</v>
-      </c>
-      <c r="M27" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" xml:space="preserve">
+      <c r="L27" t="str">
+        <v/>
+      </c>
+      <c r="M27" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="28">
       <c r="A28" t="str">
-        <v>JW-24</v>
+        <v>LW-11</v>
       </c>
       <c r="B28" t="str">
-        <v>Royal Ruby AD Necklace</v>
+        <v>Necklace</v>
       </c>
       <c r="C28" t="str">
-        <v>Jewellery</v>
+        <v>Ladies Wear</v>
       </c>
       <c r="D28" t="str">
-        <v>Necklace</v>
+        <v/>
       </c>
       <c r="E28">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="F28">
-        <v>45</v>
-      </c>
-      <c r="G28">
-        <v>24</v>
+        <v>41</v>
+      </c>
+      <c r="G28" t="str">
+        <v>INSTOCK</v>
       </c>
       <c r="H28" t="str">
-        <v>INSTOCK</v>
+        <v/>
       </c>
       <c r="I28" t="str">
-        <v>images/36a990df-97b7-4102-87c7-e8ece22eb01c.jpg</v>
+        <v>7c78d744-0d42-4361-9c66-1e02464be5e8.jpg</v>
+      </c>
+      <c r="J28" t="str">
+        <v/>
       </c>
       <c r="K28" t="str">
         <v/>
       </c>
-      <c r="L28" t="str" xml:space="preserve">
-        <v xml:space="preserve">Royal Ruby AD Necklace ✨
-An elegant gold-tone necklace adorned with sparkling white stones and rich ruby accents—perfect for weddings, parties and festive occasions.</v>
-      </c>
-      <c r="M28" t="b">
-        <v>0</v>
+      <c r="L28" t="str">
+        <v/>
+      </c>
+      <c r="M28" t="str">
+        <v>No</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>JW-25</v>
+        <v>LW-12</v>
       </c>
       <c r="B29" t="str">
-        <v>Royal Kemp Bridal Necklace Set</v>
+        <v>Palakka necklace</v>
       </c>
       <c r="C29" t="str">
-        <v>Jewellery</v>
+        <v>Ladies Wear</v>
       </c>
       <c r="D29" t="str">
-        <v>Necklace</v>
+        <v/>
       </c>
       <c r="E29">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="F29">
-        <v>53</v>
-      </c>
-      <c r="G29">
-        <v>23</v>
+        <v>26</v>
+      </c>
+      <c r="G29" t="str">
+        <v>INSTOCK</v>
       </c>
       <c r="H29" t="str">
-        <v>INSTOCK</v>
+        <v/>
       </c>
       <c r="I29" t="str">
-        <v>images/cf2f6a9e-6775-46d3-81a6-71d59978a4d4.jpg</v>
+        <v>2b2b5453-5522-4ba0-b5da-d5b5d198e451.jpg</v>
+      </c>
+      <c r="J29" t="str">
+        <v>6e989513-46c8-4212-87f8-8b7e9915aa5d.jpg</v>
       </c>
       <c r="K29" t="str">
         <v/>
       </c>
       <c r="L29" t="str">
-        <v>A grand gold-tone necklace adorned with ruby, emerald and sparkling stones, finished with elegant pearl drops and matching earrings—perfect for weddings and traditional celebrations.</v>
-      </c>
-      <c r="M29" t="b">
-        <v>0</v>
+        <v/>
+      </c>
+      <c r="M29" t="str">
+        <v>No</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>JW-26</v>
+        <v>KW-02</v>
       </c>
       <c r="B30" t="str">
-        <v>Palakka necklace</v>
+        <v>Kids wear</v>
       </c>
       <c r="C30" t="str">
-        <v>Jewellery</v>
+        <v>Kids Wear</v>
       </c>
       <c r="D30" t="str">
-        <v>Necklace</v>
+        <v/>
       </c>
       <c r="E30">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="F30">
-        <v>30</v>
-      </c>
-      <c r="G30">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="G30" t="str">
+        <v>INSTOCK</v>
       </c>
       <c r="H30" t="str">
-        <v>INSTOCK</v>
+        <v/>
       </c>
       <c r="I30" t="str">
-        <v>images/d685200c-aa2a-49aa-a40c-ff0e81b77b31.jpg</v>
+        <v>03145264-b0c4-4965-8906-e957b12dbfc4.jpg</v>
+      </c>
+      <c r="J30" t="str">
+        <v>db746ae9-4ab3-452d-9a71-6629c58904bb.jpg</v>
       </c>
       <c r="K30" t="str">
         <v/>
@@ -1542,37 +1646,40 @@
       <c r="L30" t="str">
         <v/>
       </c>
-      <c r="M30" t="b">
-        <v>1</v>
+      <c r="M30" t="str">
+        <v>No</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>KW-06</v>
+        <v>LW-13</v>
       </c>
       <c r="B31" t="str">
-        <v>Frock</v>
+        <v>Soft cotton cord set</v>
       </c>
       <c r="C31" t="str">
-        <v>Kids Wear</v>
+        <v>Ladies Wear</v>
       </c>
       <c r="D31" t="str">
         <v/>
       </c>
       <c r="E31">
-        <v>14</v>
+        <v>49.96</v>
       </c>
       <c r="F31">
-        <v>16</v>
-      </c>
-      <c r="G31">
-        <v>13</v>
+        <v>49.96</v>
+      </c>
+      <c r="G31" t="str">
+        <v>INSTOCK</v>
       </c>
       <c r="H31" t="str">
-        <v>INSTOCK</v>
+        <v>38</v>
       </c>
       <c r="I31" t="str">
-        <v>images/c7105671-a5a0-4d8e-ac6b-cd5ddaac98c6.jpg</v>
+        <v>131d7cf6-af15-4826-a46e-33cb967aa3f9.jpg</v>
+      </c>
+      <c r="J31" t="str">
+        <v/>
       </c>
       <c r="K31" t="str">
         <v/>
@@ -1580,16 +1687,16 @@
       <c r="L31" t="str">
         <v/>
       </c>
-      <c r="M31" t="b">
-        <v>0</v>
+      <c r="M31" t="str">
+        <v>No</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>LW-17</v>
+        <v>LW-14</v>
       </c>
       <c r="B32" t="str">
-        <v>Soft cotton cord set</v>
+        <v>Crushed organza</v>
       </c>
       <c r="C32" t="str">
         <v>Ladies Wear</v>
@@ -1598,95 +1705,104 @@
         <v/>
       </c>
       <c r="E32">
-        <v>49.96</v>
+        <v>74</v>
       </c>
       <c r="F32">
-        <v>56</v>
-      </c>
-      <c r="G32">
-        <v>11</v>
+        <v>85</v>
+      </c>
+      <c r="G32" t="str">
+        <v>INSTOCK</v>
       </c>
       <c r="H32" t="str">
-        <v>INSTOCK</v>
+        <v/>
       </c>
       <c r="I32" t="str">
-        <v>images/db1f3be6-3522-4112-8f3b-69d800c64db6.jpg</v>
+        <v>c4457846-0852-4bbf-bda0-af763d7be377.jpg</v>
+      </c>
+      <c r="J32" t="str">
+        <v>26e8d00c-047f-4b8d-b126-6d0f9508ec2e.jpg</v>
       </c>
       <c r="K32" t="str">
-        <v>38</v>
+        <v/>
       </c>
       <c r="L32" t="str">
         <v/>
       </c>
-      <c r="M32" t="b">
-        <v>0</v>
+      <c r="M32" t="str">
+        <v>No</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>LW-18</v>
+        <v>JW-16</v>
       </c>
       <c r="B33" t="str">
-        <v>Crushed organza</v>
+        <v>Kids bangle</v>
       </c>
       <c r="C33" t="str">
-        <v>Ladies Wear</v>
+        <v>Jewellery</v>
       </c>
       <c r="D33" t="str">
-        <v/>
+        <v>Bangles</v>
       </c>
       <c r="E33">
-        <v>74</v>
+        <v>24</v>
       </c>
       <c r="F33">
-        <v>80</v>
-      </c>
-      <c r="G33">
-        <v>8</v>
+        <v>30</v>
+      </c>
+      <c r="G33" t="str">
+        <v>INSTOCK</v>
       </c>
       <c r="H33" t="str">
-        <v>INSTOCK</v>
+        <v/>
       </c>
       <c r="I33" t="str">
-        <v>images/a12db22a-a74a-40f8-b684-c0e8a4fc7a39.jpg</v>
+        <v>84d90345-211a-4380-8820-c0e5bb78e0a6.jpg</v>
+      </c>
+      <c r="J33" t="str">
+        <v/>
       </c>
       <c r="K33" t="str">
         <v/>
       </c>
       <c r="L33" t="str">
-        <v/>
-      </c>
-      <c r="M33" t="b">
-        <v>0</v>
+        <v>4 sets - $24</v>
+      </c>
+      <c r="M33" t="str">
+        <v>No</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>JW-27</v>
+        <v>LW-15</v>
       </c>
       <c r="B34" t="str">
-        <v>Kids Bangle</v>
+        <v>Semi linen saree with blouse material</v>
       </c>
       <c r="C34" t="str">
-        <v>Jewellery</v>
+        <v>Ladies Wear</v>
       </c>
       <c r="D34" t="str">
-        <v>Bangles</v>
+        <v/>
       </c>
       <c r="E34">
-        <v>24</v>
+        <v>69</v>
       </c>
       <c r="F34">
-        <v>31</v>
-      </c>
-      <c r="G34">
-        <v>23</v>
+        <v>69</v>
+      </c>
+      <c r="G34" t="str">
+        <v>INSTOCK</v>
       </c>
       <c r="H34" t="str">
-        <v>INSTOCK</v>
+        <v/>
       </c>
       <c r="I34" t="str">
-        <v>images/e489f3b2-e2ef-4f46-9271-149637630891.jpg</v>
+        <v>ee36b63c-bca8-4b68-9e04-12d4c0bbbea5.jpg</v>
+      </c>
+      <c r="J34" t="str">
+        <v/>
       </c>
       <c r="K34" t="str">
         <v/>
@@ -1694,16 +1810,16 @@
       <c r="L34" t="str">
         <v/>
       </c>
-      <c r="M34" t="b">
-        <v>0</v>
+      <c r="M34" t="str">
+        <v>No</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>LW-19</v>
+        <v>LW-16</v>
       </c>
       <c r="B35" t="str">
-        <v>Semi linen saree with blouse material</v>
+        <v>Premium soft organza saree</v>
       </c>
       <c r="C35" t="str">
         <v>Ladies Wear</v>
@@ -1712,19 +1828,22 @@
         <v/>
       </c>
       <c r="E35">
-        <v>69</v>
+        <v>86</v>
       </c>
       <c r="F35">
-        <v>72</v>
-      </c>
-      <c r="G35">
-        <v>4</v>
+        <v>86</v>
+      </c>
+      <c r="G35" t="str">
+        <v>INSTOCK</v>
       </c>
       <c r="H35" t="str">
-        <v>INSTOCK</v>
+        <v/>
       </c>
       <c r="I35" t="str">
-        <v>images/c499e627-94d4-474f-97a9-795d83c56bba.jpg</v>
+        <v>1d9090d6-1473-4866-ad03-3fafa41909e3.jpg</v>
+      </c>
+      <c r="J35" t="str">
+        <v/>
       </c>
       <c r="K35" t="str">
         <v/>
@@ -1732,37 +1851,40 @@
       <c r="L35" t="str">
         <v/>
       </c>
-      <c r="M35" t="b">
-        <v>0</v>
+      <c r="M35" t="str">
+        <v>No</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>LW-20</v>
+        <v>JW-17</v>
       </c>
       <c r="B36" t="str">
-        <v>Premium  soft organza saree</v>
+        <v>Earrings</v>
       </c>
       <c r="C36" t="str">
-        <v>Ladies Wear</v>
+        <v>Jewellery</v>
       </c>
       <c r="D36" t="str">
         <v/>
       </c>
       <c r="E36">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="F36">
-        <v>100</v>
-      </c>
-      <c r="G36">
-        <v>14</v>
+        <v>18</v>
+      </c>
+      <c r="G36" t="str">
+        <v>INSTOCK</v>
       </c>
       <c r="H36" t="str">
-        <v>INSTOCK</v>
+        <v/>
       </c>
       <c r="I36" t="str">
-        <v>images/f87f53fe-3742-4c06-8f10-173b9fa436a1.jpg</v>
+        <v>51ec9771-0991-4c7b-b196-a61c691dd3a1.jpg</v>
+      </c>
+      <c r="J36" t="str">
+        <v/>
       </c>
       <c r="K36" t="str">
         <v/>
@@ -1770,37 +1892,40 @@
       <c r="L36" t="str">
         <v/>
       </c>
-      <c r="M36" t="b">
-        <v>0</v>
+      <c r="M36" t="str">
+        <v>No</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>JW-28</v>
+        <v>LW-17</v>
       </c>
       <c r="B37" t="str">
-        <v>Earrings</v>
+        <v>Blouse material</v>
       </c>
       <c r="C37" t="str">
-        <v>Jewellery</v>
+        <v>Ladies Wear</v>
       </c>
       <c r="D37" t="str">
-        <v>Earring</v>
+        <v/>
       </c>
       <c r="E37">
-        <v>18</v>
+        <v>76</v>
       </c>
       <c r="F37">
-        <v>22</v>
-      </c>
-      <c r="G37">
-        <v>18</v>
+        <v>76</v>
+      </c>
+      <c r="G37" t="str">
+        <v>INSTOCK</v>
       </c>
       <c r="H37" t="str">
-        <v>INSTOCK</v>
+        <v/>
       </c>
       <c r="I37" t="str">
-        <v>images/8efcb74e-96d4-4e9c-9a0e-1c4e0edfdb0b.jpg</v>
+        <v>e1f92a4b-28c4-4441-8e58-7fbf8519aab4.jpg</v>
+      </c>
+      <c r="J37" t="str">
+        <v/>
       </c>
       <c r="K37" t="str">
         <v/>
@@ -1808,16 +1933,16 @@
       <c r="L37" t="str">
         <v/>
       </c>
-      <c r="M37" t="b">
-        <v>0</v>
+      <c r="M37" t="str">
+        <v>No</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>LW-21</v>
+        <v>LW-18</v>
       </c>
       <c r="B38" t="str">
-        <v>Saree with blouse material</v>
+        <v>Kerala saree</v>
       </c>
       <c r="C38" t="str">
         <v>Ladies Wear</v>
@@ -1826,19 +1951,22 @@
         <v/>
       </c>
       <c r="E38">
-        <v>76</v>
+        <v>60</v>
       </c>
       <c r="F38">
-        <v>90</v>
-      </c>
-      <c r="G38">
-        <v>16</v>
+        <v>60</v>
+      </c>
+      <c r="G38" t="str">
+        <v>INSTOCK</v>
       </c>
       <c r="H38" t="str">
-        <v>INSTOCK</v>
+        <v/>
       </c>
       <c r="I38" t="str">
-        <v>images/7924eaaa-b32b-43bc-aa78-1e3dc81e9141.jpg</v>
+        <v>0d679b5f-20e1-4ea6-af23-4592780e6b26.jpg</v>
+      </c>
+      <c r="J38" t="str">
+        <v/>
       </c>
       <c r="K38" t="str">
         <v/>
@@ -1846,16 +1974,16 @@
       <c r="L38" t="str">
         <v/>
       </c>
-      <c r="M38" t="b">
-        <v>0</v>
+      <c r="M38" t="str">
+        <v>No</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>LW-22</v>
+        <v>LW-19</v>
       </c>
       <c r="B39" t="str">
-        <v>Designer Kerala saree</v>
+        <v>Tissue saree</v>
       </c>
       <c r="C39" t="str">
         <v>Ladies Wear</v>
@@ -1864,19 +1992,22 @@
         <v/>
       </c>
       <c r="E39">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="F39">
-        <v>69</v>
-      </c>
-      <c r="G39">
-        <v>13</v>
+        <v>65</v>
+      </c>
+      <c r="G39" t="str">
+        <v>INSTOCK</v>
       </c>
       <c r="H39" t="str">
-        <v>INSTOCK</v>
+        <v/>
       </c>
       <c r="I39" t="str">
-        <v>images/2f2517ba-9ed9-45c9-9dec-38bc51668a15.jpg</v>
+        <v>18db0c07-988d-4d1c-af0e-cdfb1d9d3287.jpg</v>
+      </c>
+      <c r="J39" t="str">
+        <v/>
       </c>
       <c r="K39" t="str">
         <v/>
@@ -1884,16 +2015,16 @@
       <c r="L39" t="str">
         <v/>
       </c>
-      <c r="M39" t="b">
-        <v>0</v>
+      <c r="M39" t="str">
+        <v>No</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>LW-23</v>
+        <v>LW-20</v>
       </c>
       <c r="B40" t="str">
-        <v>Tissue saree</v>
+        <v>Saree with unstitched  house</v>
       </c>
       <c r="C40" t="str">
         <v>Ladies Wear</v>
@@ -1902,19 +2033,22 @@
         <v/>
       </c>
       <c r="E40">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="F40">
-        <v>70</v>
-      </c>
-      <c r="G40">
-        <v>7</v>
+        <v>74</v>
+      </c>
+      <c r="G40" t="str">
+        <v>INSTOCK</v>
       </c>
       <c r="H40" t="str">
-        <v>INSTOCK</v>
+        <v/>
       </c>
       <c r="I40" t="str">
-        <v>images/c0c95e56-1226-4f27-a8dc-f91a08506f09.jpg</v>
+        <v>6956590e-bfbc-4fff-8397-7f35f2e53183.jpg</v>
+      </c>
+      <c r="J40" t="str">
+        <v/>
       </c>
       <c r="K40" t="str">
         <v/>
@@ -1922,16 +2056,16 @@
       <c r="L40" t="str">
         <v/>
       </c>
-      <c r="M40" t="b">
-        <v>0</v>
+      <c r="M40" t="str">
+        <v>No</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>LW-24</v>
+        <v>LW-21</v>
       </c>
       <c r="B41" t="str">
-        <v>Saree with unstitched  house</v>
+        <v>Saree  with unstitched  house</v>
       </c>
       <c r="C41" t="str">
         <v>Ladies Wear</v>
@@ -1940,19 +2074,22 @@
         <v/>
       </c>
       <c r="E41">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="F41">
-        <v>80</v>
-      </c>
-      <c r="G41">
-        <v>8</v>
+        <v>69</v>
+      </c>
+      <c r="G41" t="str">
+        <v>INSTOCK</v>
       </c>
       <c r="H41" t="str">
-        <v>INSTOCK</v>
+        <v/>
       </c>
       <c r="I41" t="str">
-        <v>images/d0d50de4-ecce-48ef-a2a4-d41988b98860.jpg</v>
+        <v>e567a3a9-2582-49d3-a4a6-3fc8e5f06330.jpg</v>
+      </c>
+      <c r="J41" t="str">
+        <v/>
       </c>
       <c r="K41" t="str">
         <v/>
@@ -1960,16 +2097,16 @@
       <c r="L41" t="str">
         <v/>
       </c>
-      <c r="M41" t="b">
-        <v>0</v>
+      <c r="M41" t="str">
+        <v>No</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>LW-25</v>
+        <v>LW-22</v>
       </c>
       <c r="B42" t="str">
-        <v>Saree with unstitched blouse</v>
+        <v>Readymade 3 piece Churidar</v>
       </c>
       <c r="C42" t="str">
         <v>Ladies Wear</v>
@@ -1978,19 +2115,22 @@
         <v/>
       </c>
       <c r="E42">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F42">
-        <v>80</v>
-      </c>
-      <c r="G42">
-        <v>14</v>
+        <v>68</v>
+      </c>
+      <c r="G42" t="str">
+        <v>INSTOCK</v>
       </c>
       <c r="H42" t="str">
-        <v>INSTOCK</v>
+        <v/>
       </c>
       <c r="I42" t="str">
-        <v>images/493b7819-92bf-4b24-93eb-67f3e4520217.jpg</v>
+        <v>2c2e75b4-e458-4156-ac43-fdb2653debba.jpg</v>
+      </c>
+      <c r="J42" t="str">
+        <v/>
       </c>
       <c r="K42" t="str">
         <v/>
@@ -1998,16 +2138,16 @@
       <c r="L42" t="str">
         <v/>
       </c>
-      <c r="M42" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43">
+      <c r="M42" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="43" xml:space="preserve">
       <c r="A43" t="str">
-        <v>LW-26</v>
+        <v>LW-23</v>
       </c>
       <c r="B43" t="str">
-        <v>Readymade 3 piece Churidar</v>
+        <v>Ready made blouse - free size</v>
       </c>
       <c r="C43" t="str">
         <v>Ladies Wear</v>
@@ -2016,96 +2156,105 @@
         <v/>
       </c>
       <c r="E43">
-        <v>68</v>
+        <v>40</v>
       </c>
       <c r="F43">
-        <v>71</v>
-      </c>
-      <c r="G43">
-        <v>4</v>
+        <v>40</v>
+      </c>
+      <c r="G43" t="str">
+        <v>INSTOCK</v>
       </c>
       <c r="H43" t="str">
-        <v>INSTOCK</v>
+        <v/>
       </c>
       <c r="I43" t="str">
-        <v>images/bdd10649-fb6d-442a-b7cc-e001b3b03b9a.jpg</v>
+        <v>5c008d60-5f79-4e29-b2b4-8265a90f6087.jpg</v>
+      </c>
+      <c r="J43" t="str">
+        <v/>
       </c>
       <c r="K43" t="str">
         <v/>
       </c>
-      <c r="L43" t="str">
-        <v/>
-      </c>
-      <c r="M43" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44" xml:space="preserve">
-      <c r="A44" t="str">
-        <v>LW-27</v>
-      </c>
-      <c r="B44" t="str">
-        <v>Ready made blouse - free size</v>
-      </c>
-      <c r="C44" t="str">
-        <v>Ladies Wear</v>
-      </c>
-      <c r="D44" t="str">
-        <v/>
-      </c>
-      <c r="E44">
-        <v>40</v>
-      </c>
-      <c r="F44">
-        <v>50</v>
-      </c>
-      <c r="G44">
-        <v>20</v>
-      </c>
-      <c r="H44" t="str">
-        <v>INSTOCK</v>
-      </c>
-      <c r="I44" t="str">
-        <v>images/628f1d8e-a466-43bb-8e5c-4876365a6096.jpg</v>
-      </c>
-      <c r="K44" t="str">
-        <v/>
-      </c>
-      <c r="L44" t="str" xml:space="preserve">
+      <c r="L43" t="str" xml:space="preserve">
         <v xml:space="preserve">Margin -34 to 42
 Alterable</v>
       </c>
-      <c r="M44" t="b">
-        <v>0</v>
+      <c r="M43" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>JW-18</v>
+      </c>
+      <c r="B44" t="str">
+        <v>Necklace</v>
+      </c>
+      <c r="C44" t="str">
+        <v>Jewellery</v>
+      </c>
+      <c r="D44" t="str">
+        <v>Necklace</v>
+      </c>
+      <c r="E44">
+        <v>28</v>
+      </c>
+      <c r="F44">
+        <v>28</v>
+      </c>
+      <c r="G44" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H44" t="str">
+        <v/>
+      </c>
+      <c r="I44" t="str">
+        <v>b0a70b5a-4cb4-46ca-91b0-c9cd8afd0df0.jpg</v>
+      </c>
+      <c r="J44" t="str">
+        <v>24678d15-eda5-4507-81bf-4c86646fd43a.jpg</v>
+      </c>
+      <c r="K44" t="str">
+        <v/>
+      </c>
+      <c r="L44" t="str">
+        <v/>
+      </c>
+      <c r="M44" t="str">
+        <v>No</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>JW-29</v>
+        <v>LW-24</v>
       </c>
       <c r="B45" t="str">
         <v>Necklace</v>
       </c>
       <c r="C45" t="str">
-        <v>Jewellery</v>
+        <v>Ladies Wear</v>
       </c>
       <c r="D45" t="str">
-        <v>Necklace</v>
+        <v/>
       </c>
       <c r="E45">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="F45">
-        <v>35</v>
-      </c>
-      <c r="G45">
-        <v>20</v>
+        <v>16</v>
+      </c>
+      <c r="G45" t="str">
+        <v>INSTOCK</v>
       </c>
       <c r="H45" t="str">
-        <v>INSTOCK</v>
+        <v/>
       </c>
       <c r="I45" t="str">
-        <v>images/da52d908-0880-4f1d-9f67-284a718958ce.jpg</v>
+        <v>036ee668-3ec3-4f7c-9636-93d97e51734f.jpg</v>
+      </c>
+      <c r="J45" t="str">
+        <v>0bf2d876-c09a-45aa-9d36-ab47201d98a0.jpg</v>
       </c>
       <c r="K45" t="str">
         <v/>
@@ -2113,37 +2262,40 @@
       <c r="L45" t="str">
         <v/>
       </c>
-      <c r="M45" t="b">
-        <v>0</v>
+      <c r="M45" t="str">
+        <v>No</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>JW-30</v>
+        <v>LW-25</v>
       </c>
       <c r="B46" t="str">
         <v>Necklace</v>
       </c>
       <c r="C46" t="str">
-        <v>Jewellery</v>
+        <v>Ladies Wear</v>
       </c>
       <c r="D46" t="str">
-        <v>Necklace</v>
+        <v/>
       </c>
       <c r="E46">
-        <v>26</v>
+        <v>29.65</v>
       </c>
       <c r="F46">
-        <v>30</v>
-      </c>
-      <c r="G46">
-        <v>13</v>
+        <v>29.65</v>
+      </c>
+      <c r="G46" t="str">
+        <v>INSTOCK</v>
       </c>
       <c r="H46" t="str">
-        <v>INSTOCK</v>
+        <v/>
       </c>
       <c r="I46" t="str">
-        <v>images/4d5b216e-8aef-41dc-a65e-b54c4a1709ef.jpg</v>
+        <v>67d8f155-16b3-4bd5-bd05-885bdf6a7953.jpg</v>
+      </c>
+      <c r="J46" t="str">
+        <v>5e50b530-e4b2-4c95-98f0-71282845fb62.jpg</v>
       </c>
       <c r="K46" t="str">
         <v/>
@@ -2151,51 +2303,13 @@
       <c r="L46" t="str">
         <v/>
       </c>
-      <c r="M46" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="str">
-        <v>JW-31</v>
-      </c>
-      <c r="B47" t="str">
-        <v>Necklace</v>
-      </c>
-      <c r="C47" t="str">
-        <v>Jewellery</v>
-      </c>
-      <c r="D47" t="str">
-        <v>Necklace</v>
-      </c>
-      <c r="E47">
-        <v>29.65</v>
-      </c>
-      <c r="F47">
-        <v>36</v>
-      </c>
-      <c r="G47">
-        <v>18</v>
-      </c>
-      <c r="H47" t="str">
-        <v>INSTOCK</v>
-      </c>
-      <c r="I47" t="str">
-        <v>images/429ab56c-c1ab-48e7-b73f-013faa1af682.jpg</v>
-      </c>
-      <c r="K47" t="str">
-        <v/>
-      </c>
-      <c r="L47" t="str">
-        <v/>
-      </c>
-      <c r="M47" t="b">
-        <v>0</v>
+      <c r="M46" t="str">
+        <v>No</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M47"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M46"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update store products via Admin Panel - 08/08/2026, 12:47:13 am
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M50"/>
+  <dimension ref="A1:M53"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1939,10 +1939,10 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>LW-19</v>
+        <v>LW-20</v>
       </c>
       <c r="B38" t="str">
-        <v>Tissue saree</v>
+        <v>Saree with unstitched  house</v>
       </c>
       <c r="C38" t="str">
         <v>Ladies Wear</v>
@@ -1951,10 +1951,10 @@
         <v/>
       </c>
       <c r="E38">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="F38">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="G38" t="str">
         <v>INSTOCK</v>
@@ -1963,7 +1963,7 @@
         <v/>
       </c>
       <c r="I38" t="str">
-        <v>18db0c07-988d-4d1c-af0e-cdfb1d9d3287.jpg</v>
+        <v>6956590e-bfbc-4fff-8397-7f35f2e53183.jpg</v>
       </c>
       <c r="J38" t="str">
         <v/>
@@ -1980,10 +1980,10 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>LW-20</v>
+        <v>LW-21</v>
       </c>
       <c r="B39" t="str">
-        <v>Saree with unstitched  house</v>
+        <v>Saree  with unstitched  house</v>
       </c>
       <c r="C39" t="str">
         <v>Ladies Wear</v>
@@ -1992,10 +1992,10 @@
         <v/>
       </c>
       <c r="E39">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="F39">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="G39" t="str">
         <v>INSTOCK</v>
@@ -2004,7 +2004,7 @@
         <v/>
       </c>
       <c r="I39" t="str">
-        <v>6956590e-bfbc-4fff-8397-7f35f2e53183.jpg</v>
+        <v>e567a3a9-2582-49d3-a4a6-3fc8e5f06330.jpg</v>
       </c>
       <c r="J39" t="str">
         <v/>
@@ -2021,10 +2021,10 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>LW-21</v>
+        <v>LW-22</v>
       </c>
       <c r="B40" t="str">
-        <v>Saree  with unstitched  house</v>
+        <v>Readymade 3 piece Churidar</v>
       </c>
       <c r="C40" t="str">
         <v>Ladies Wear</v>
@@ -2033,10 +2033,10 @@
         <v/>
       </c>
       <c r="E40">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F40">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G40" t="str">
         <v>INSTOCK</v>
@@ -2045,7 +2045,7 @@
         <v/>
       </c>
       <c r="I40" t="str">
-        <v>e567a3a9-2582-49d3-a4a6-3fc8e5f06330.jpg</v>
+        <v>2c2e75b4-e458-4156-ac43-fdb2653debba.jpg</v>
       </c>
       <c r="J40" t="str">
         <v/>
@@ -2060,12 +2060,12 @@
         <v>No</v>
       </c>
     </row>
-    <row r="41">
+    <row r="41" xml:space="preserve">
       <c r="A41" t="str">
-        <v>LW-22</v>
+        <v>LW-23</v>
       </c>
       <c r="B41" t="str">
-        <v>Readymade 3 piece Churidar</v>
+        <v>Ready made blouse - free size</v>
       </c>
       <c r="C41" t="str">
         <v>Ladies Wear</v>
@@ -2074,10 +2074,10 @@
         <v/>
       </c>
       <c r="E41">
-        <v>68</v>
+        <v>40</v>
       </c>
       <c r="F41">
-        <v>68</v>
+        <v>40</v>
       </c>
       <c r="G41" t="str">
         <v>INSTOCK</v>
@@ -2086,7 +2086,7 @@
         <v/>
       </c>
       <c r="I41" t="str">
-        <v>2c2e75b4-e458-4156-ac43-fdb2653debba.jpg</v>
+        <v>5c008d60-5f79-4e29-b2b4-8265a90f6087.jpg</v>
       </c>
       <c r="J41" t="str">
         <v/>
@@ -2094,58 +2094,58 @@
       <c r="K41" t="str">
         <v/>
       </c>
-      <c r="L41" t="str">
-        <v/>
-      </c>
-      <c r="M41" t="str">
-        <v>No</v>
-      </c>
-    </row>
-    <row r="42" xml:space="preserve">
-      <c r="A42" t="str">
-        <v>LW-23</v>
-      </c>
-      <c r="B42" t="str">
-        <v>Ready made blouse - free size</v>
-      </c>
-      <c r="C42" t="str">
-        <v>Ladies Wear</v>
-      </c>
-      <c r="D42" t="str">
-        <v/>
-      </c>
-      <c r="E42">
-        <v>40</v>
-      </c>
-      <c r="F42">
-        <v>40</v>
-      </c>
-      <c r="G42" t="str">
-        <v>INSTOCK</v>
-      </c>
-      <c r="H42" t="str">
-        <v/>
-      </c>
-      <c r="I42" t="str">
-        <v>5c008d60-5f79-4e29-b2b4-8265a90f6087.jpg</v>
-      </c>
-      <c r="J42" t="str">
-        <v/>
-      </c>
-      <c r="K42" t="str">
-        <v/>
-      </c>
-      <c r="L42" t="str" xml:space="preserve">
+      <c r="L41" t="str" xml:space="preserve">
         <v xml:space="preserve">Margin -34 to 42
 Alterable</v>
       </c>
+      <c r="M41" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>JW-18</v>
+      </c>
+      <c r="B42" t="str">
+        <v>Necklace</v>
+      </c>
+      <c r="C42" t="str">
+        <v>Jewellery</v>
+      </c>
+      <c r="D42" t="str">
+        <v>Necklace</v>
+      </c>
+      <c r="E42">
+        <v>28</v>
+      </c>
+      <c r="F42">
+        <v>32</v>
+      </c>
+      <c r="G42" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H42" t="str">
+        <v/>
+      </c>
+      <c r="I42" t="str">
+        <v>d1f27456-8744-4fcc-98f2-e5a8c4d3cdd9.jpg</v>
+      </c>
+      <c r="J42" t="str">
+        <v>f9e7ad8e-1d10-47b5-b41f-e4a92b4288d7.jpg</v>
+      </c>
+      <c r="K42" t="str">
+        <v/>
+      </c>
+      <c r="L42" t="str">
+        <v/>
+      </c>
       <c r="M42" t="str">
         <v>No</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>JW-18</v>
+        <v>LW-24</v>
       </c>
       <c r="B43" t="str">
         <v>Necklace</v>
@@ -2157,10 +2157,10 @@
         <v>Necklace</v>
       </c>
       <c r="E43">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="F43">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="G43" t="str">
         <v>INSTOCK</v>
@@ -2169,10 +2169,10 @@
         <v/>
       </c>
       <c r="I43" t="str">
-        <v>d1f27456-8744-4fcc-98f2-e5a8c4d3cdd9.jpg</v>
+        <v>036ee668-3ec3-4f7c-9636-93d97e51734f.jpg</v>
       </c>
       <c r="J43" t="str">
-        <v>f9e7ad8e-1d10-47b5-b41f-e4a92b4288d7.jpg</v>
+        <v>0bf2d876-c09a-45aa-9d36-ab47201d98a0.jpg</v>
       </c>
       <c r="K43" t="str">
         <v/>
@@ -2186,7 +2186,7 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>LW-24</v>
+        <v>LW-25</v>
       </c>
       <c r="B44" t="str">
         <v>Necklace</v>
@@ -2198,10 +2198,10 @@
         <v>Necklace</v>
       </c>
       <c r="E44">
-        <v>16</v>
+        <v>29.65</v>
       </c>
       <c r="F44">
-        <v>16</v>
+        <v>29.65</v>
       </c>
       <c r="G44" t="str">
         <v>INSTOCK</v>
@@ -2210,10 +2210,10 @@
         <v/>
       </c>
       <c r="I44" t="str">
-        <v>036ee668-3ec3-4f7c-9636-93d97e51734f.jpg</v>
+        <v>67d8f155-16b3-4bd5-bd05-885bdf6a7953.jpg</v>
       </c>
       <c r="J44" t="str">
-        <v>0bf2d876-c09a-45aa-9d36-ab47201d98a0.jpg</v>
+        <v>5e50b530-e4b2-4c95-98f0-71282845fb62.jpg</v>
       </c>
       <c r="K44" t="str">
         <v/>
@@ -2227,7 +2227,7 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>LW-25</v>
+        <v>JW-20</v>
       </c>
       <c r="B45" t="str">
         <v>Necklace</v>
@@ -2239,10 +2239,10 @@
         <v>Necklace</v>
       </c>
       <c r="E45">
-        <v>29.65</v>
+        <v>41</v>
       </c>
       <c r="F45">
-        <v>29.65</v>
+        <v>41</v>
       </c>
       <c r="G45" t="str">
         <v>INSTOCK</v>
@@ -2251,10 +2251,10 @@
         <v/>
       </c>
       <c r="I45" t="str">
-        <v>67d8f155-16b3-4bd5-bd05-885bdf6a7953.jpg</v>
+        <v>7c78d744-0d42-4361-9c66-1e02464be5e8.jpg</v>
       </c>
       <c r="J45" t="str">
-        <v>5e50b530-e4b2-4c95-98f0-71282845fb62.jpg</v>
+        <v/>
       </c>
       <c r="K45" t="str">
         <v/>
@@ -2268,22 +2268,22 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>JW-20</v>
+        <v>LW-26</v>
       </c>
       <c r="B46" t="str">
-        <v>Necklace</v>
+        <v>Bandhani print saree</v>
       </c>
       <c r="C46" t="str">
-        <v>Jewellery</v>
+        <v>Ladies Wear</v>
       </c>
       <c r="D46" t="str">
-        <v>Necklace</v>
+        <v/>
       </c>
       <c r="E46">
-        <v>41</v>
+        <v>54</v>
       </c>
       <c r="F46">
-        <v>41</v>
+        <v>54</v>
       </c>
       <c r="G46" t="str">
         <v>INSTOCK</v>
@@ -2292,7 +2292,7 @@
         <v/>
       </c>
       <c r="I46" t="str">
-        <v>7c78d744-0d42-4361-9c66-1e02464be5e8.jpg</v>
+        <v>118f5da2-2e4e-44d9-b82f-49aa8ebfaaff.jpg</v>
       </c>
       <c r="J46" t="str">
         <v/>
@@ -2309,10 +2309,10 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>LW-26</v>
+        <v>LW-27</v>
       </c>
       <c r="B47" t="str">
-        <v>Bandhani print saree</v>
+        <v>Saree with unstitched blouse</v>
       </c>
       <c r="C47" t="str">
         <v>Ladies Wear</v>
@@ -2321,10 +2321,10 @@
         <v/>
       </c>
       <c r="E47">
-        <v>54</v>
+        <v>64</v>
       </c>
       <c r="F47">
-        <v>54</v>
+        <v>64</v>
       </c>
       <c r="G47" t="str">
         <v>INSTOCK</v>
@@ -2333,7 +2333,7 @@
         <v/>
       </c>
       <c r="I47" t="str">
-        <v>118f5da2-2e4e-44d9-b82f-49aa8ebfaaff.jpg</v>
+        <v>0a92f30f-f280-498d-a0c8-35924794ff3a.jpg</v>
       </c>
       <c r="J47" t="str">
         <v/>
@@ -2350,10 +2350,10 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>LW-27</v>
+        <v>LW-28</v>
       </c>
       <c r="B48" t="str">
-        <v>Saree with unstitched blouse</v>
+        <v>Soft cotton Saree with stiched blouse</v>
       </c>
       <c r="C48" t="str">
         <v>Ladies Wear</v>
@@ -2362,10 +2362,10 @@
         <v/>
       </c>
       <c r="E48">
-        <v>64</v>
+        <v>75</v>
       </c>
       <c r="F48">
-        <v>64</v>
+        <v>75</v>
       </c>
       <c r="G48" t="str">
         <v>INSTOCK</v>
@@ -2374,7 +2374,7 @@
         <v/>
       </c>
       <c r="I48" t="str">
-        <v>0a92f30f-f280-498d-a0c8-35924794ff3a.jpg</v>
+        <v>d033924f-94ca-41d0-8288-068f80400151.jpg</v>
       </c>
       <c r="J48" t="str">
         <v/>
@@ -2391,10 +2391,10 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>LW-28</v>
+        <v>LW-29</v>
       </c>
       <c r="B49" t="str">
-        <v>Soft cotton Saree with stiched blouse</v>
+        <v>Bandhani print saree</v>
       </c>
       <c r="C49" t="str">
         <v>Ladies Wear</v>
@@ -2403,10 +2403,10 @@
         <v/>
       </c>
       <c r="E49">
-        <v>75</v>
+        <v>54</v>
       </c>
       <c r="F49">
-        <v>75</v>
+        <v>54</v>
       </c>
       <c r="G49" t="str">
         <v>INSTOCK</v>
@@ -2415,7 +2415,7 @@
         <v/>
       </c>
       <c r="I49" t="str">
-        <v>d033924f-94ca-41d0-8288-068f80400151.jpg</v>
+        <v>2916adc5-cf5b-4ef3-a202-ac331ed10aec.jpg</v>
       </c>
       <c r="J49" t="str">
         <v/>
@@ -2432,10 +2432,10 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>LW-29</v>
+        <v>LW-30</v>
       </c>
       <c r="B50" t="str">
-        <v>Bandhani print saree</v>
+        <v>Kids frocks</v>
       </c>
       <c r="C50" t="str">
         <v>Ladies Wear</v>
@@ -2444,10 +2444,10 @@
         <v/>
       </c>
       <c r="E50">
-        <v>54</v>
+        <v>18</v>
       </c>
       <c r="F50">
-        <v>54</v>
+        <v>23.69</v>
       </c>
       <c r="G50" t="str">
         <v>INSTOCK</v>
@@ -2456,7 +2456,7 @@
         <v/>
       </c>
       <c r="I50" t="str">
-        <v>2916adc5-cf5b-4ef3-a202-ac331ed10aec.jpg</v>
+        <v>5A8C6FC2-D70C-41AE-87F1-96716CEED2B9.png</v>
       </c>
       <c r="J50" t="str">
         <v/>
@@ -2468,12 +2468,135 @@
         <v/>
       </c>
       <c r="M50" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>LW-31</v>
+      </c>
+      <c r="B51" t="str">
+        <v>chanderi  silk saree with  stitched blouse ( free size )</v>
+      </c>
+      <c r="C51" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D51" t="str">
+        <v/>
+      </c>
+      <c r="E51">
+        <v>75</v>
+      </c>
+      <c r="F51">
+        <v>90</v>
+      </c>
+      <c r="G51" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H51" t="str">
+        <v/>
+      </c>
+      <c r="I51" t="str">
+        <v>6b2561c8-6263-45cb-821b-c1f81f59241b.jpg</v>
+      </c>
+      <c r="J51" t="str">
+        <v/>
+      </c>
+      <c r="K51" t="str">
+        <v/>
+      </c>
+      <c r="L51" t="str">
+        <v/>
+      </c>
+      <c r="M51" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>LW-32</v>
+      </c>
+      <c r="B52" t="str">
+        <v>FROCK</v>
+      </c>
+      <c r="C52" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D52" t="str">
+        <v/>
+      </c>
+      <c r="E52">
+        <v>22</v>
+      </c>
+      <c r="F52">
+        <v>25</v>
+      </c>
+      <c r="G52" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H52" t="str">
+        <v>AVAILBALE SIZES .S/M/L</v>
+      </c>
+      <c r="I52" t="str">
+        <v>8A5CF031-FEB1-4236-AD91-70D34DC65552.png</v>
+      </c>
+      <c r="J52" t="str">
+        <v/>
+      </c>
+      <c r="K52" t="str">
+        <v/>
+      </c>
+      <c r="L52" t="str">
+        <v>Suitable for age group of 0-1 yr old</v>
+      </c>
+      <c r="M52" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>LW-33</v>
+      </c>
+      <c r="B53" t="str">
+        <v>Partywear saree</v>
+      </c>
+      <c r="C53" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D53" t="str">
+        <v/>
+      </c>
+      <c r="E53">
+        <v>78</v>
+      </c>
+      <c r="F53">
+        <v>90</v>
+      </c>
+      <c r="G53" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H53" t="str">
+        <v/>
+      </c>
+      <c r="I53" t="str">
+        <v>44e37f34-a892-465c-a00e-a19925035acc.jpg</v>
+      </c>
+      <c r="J53" t="str">
+        <v/>
+      </c>
+      <c r="K53" t="str">
+        <v/>
+      </c>
+      <c r="L53" t="str">
+        <v/>
+      </c>
+      <c r="M53" t="str">
         <v>No</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M50"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M53"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update store products via Admin Panel - 08/08/2026, 1:45:37 am
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M53"/>
+  <dimension ref="A1:M63"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1910,7 +1910,7 @@
         <v/>
       </c>
       <c r="E37">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="F37">
         <v>60</v>
@@ -2476,7 +2476,7 @@
         <v>LW-31</v>
       </c>
       <c r="B51" t="str">
-        <v>chanderi  silk saree with  stitched blouse ( free size )</v>
+        <v>litchy silk saree</v>
       </c>
       <c r="C51" t="str">
         <v>Ladies Wear</v>
@@ -2485,10 +2485,10 @@
         <v/>
       </c>
       <c r="E51">
-        <v>75</v>
+        <v>53</v>
       </c>
       <c r="F51">
-        <v>90</v>
+        <v>70</v>
       </c>
       <c r="G51" t="str">
         <v>INSTOCK</v>
@@ -2497,7 +2497,7 @@
         <v/>
       </c>
       <c r="I51" t="str">
-        <v>6b2561c8-6263-45cb-821b-c1f81f59241b.jpg</v>
+        <v>adf28d79-0446-4144-b06a-fa915d368878.jpg</v>
       </c>
       <c r="J51" t="str">
         <v/>
@@ -2594,9 +2594,420 @@
         <v>No</v>
       </c>
     </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>KW-03</v>
+      </c>
+      <c r="B54" t="str">
+        <v>Baby frocks</v>
+      </c>
+      <c r="C54" t="str">
+        <v>Kids Wear</v>
+      </c>
+      <c r="D54" t="str">
+        <v/>
+      </c>
+      <c r="E54">
+        <v>19</v>
+      </c>
+      <c r="F54">
+        <v>25</v>
+      </c>
+      <c r="G54" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H54" t="str">
+        <v/>
+      </c>
+      <c r="I54" t="str">
+        <v>A66ACE60-BDFF-4977-A1A5-D447993B2321.png</v>
+      </c>
+      <c r="J54" t="str">
+        <v/>
+      </c>
+      <c r="K54" t="str">
+        <v/>
+      </c>
+      <c r="L54" t="str">
+        <v/>
+      </c>
+      <c r="M54" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="55" xml:space="preserve">
+      <c r="A55" t="str">
+        <v>KW-04</v>
+      </c>
+      <c r="B55" t="str">
+        <v>ONAM outfits for toddler group</v>
+      </c>
+      <c r="C55" t="str">
+        <v>Kids Wear</v>
+      </c>
+      <c r="D55" t="str">
+        <v/>
+      </c>
+      <c r="E55">
+        <v>21.96</v>
+      </c>
+      <c r="F55">
+        <v>25</v>
+      </c>
+      <c r="G55" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H55" t="str">
+        <v/>
+      </c>
+      <c r="I55" t="str">
+        <v>a15ed8bb-cd13-4da1-8b8c-c1b11fe90f16.jpg</v>
+      </c>
+      <c r="J55" t="str">
+        <v/>
+      </c>
+      <c r="K55" t="str">
+        <v/>
+      </c>
+      <c r="L55" t="str" xml:space="preserve">
+        <v xml:space="preserve">Available in Small, Medium, and Large sizes. Suitable for ages 0–12 months.
+Sizes: S, M, L — Recommended for babies up to 12 months of age.</v>
+      </c>
+      <c r="M55" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>LW-34</v>
+      </c>
+      <c r="B56" t="str">
+        <v>Necklace</v>
+      </c>
+      <c r="C56" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D56" t="str">
+        <v/>
+      </c>
+      <c r="E56">
+        <v>39</v>
+      </c>
+      <c r="F56">
+        <v>46</v>
+      </c>
+      <c r="G56" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H56" t="str">
+        <v/>
+      </c>
+      <c r="I56" t="str">
+        <v>DSCF1224_Original.JPG</v>
+      </c>
+      <c r="J56" t="str">
+        <v/>
+      </c>
+      <c r="K56" t="str">
+        <v/>
+      </c>
+      <c r="L56" t="str">
+        <v>Multicoloured Statement Necklace</v>
+      </c>
+      <c r="M56" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>KW-05</v>
+      </c>
+      <c r="B57" t="str">
+        <v>Kids frocks</v>
+      </c>
+      <c r="C57" t="str">
+        <v>Kids Wear</v>
+      </c>
+      <c r="D57" t="str">
+        <v/>
+      </c>
+      <c r="E57">
+        <v>22</v>
+      </c>
+      <c r="F57">
+        <v>25</v>
+      </c>
+      <c r="G57" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H57" t="str">
+        <v/>
+      </c>
+      <c r="I57" t="str">
+        <v>E67B61A0-E989-44EA-81DF-5D659645CADE_1_.png</v>
+      </c>
+      <c r="J57" t="str">
+        <v/>
+      </c>
+      <c r="K57" t="str">
+        <v/>
+      </c>
+      <c r="L57" t="str">
+        <v/>
+      </c>
+      <c r="M57" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>KW-06</v>
+      </c>
+      <c r="B58" t="str">
+        <v>Kids frocks</v>
+      </c>
+      <c r="C58" t="str">
+        <v>Kids Wear</v>
+      </c>
+      <c r="D58" t="str">
+        <v/>
+      </c>
+      <c r="E58">
+        <v>16</v>
+      </c>
+      <c r="F58">
+        <v>25</v>
+      </c>
+      <c r="G58" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H58" t="str">
+        <v/>
+      </c>
+      <c r="I58" t="str">
+        <v>ead697a2-7165-4b75-b6b2-857994b4cb9f.jpg</v>
+      </c>
+      <c r="J58" t="str">
+        <v/>
+      </c>
+      <c r="K58" t="str">
+        <v/>
+      </c>
+      <c r="L58" t="str">
+        <v>Recommended for babies up to 12 months of age.</v>
+      </c>
+      <c r="M58" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>KW-07</v>
+      </c>
+      <c r="B59" t="str">
+        <v>Onam Kids frocks</v>
+      </c>
+      <c r="C59" t="str">
+        <v>Kids Wear</v>
+      </c>
+      <c r="D59" t="str">
+        <v/>
+      </c>
+      <c r="E59">
+        <v>22</v>
+      </c>
+      <c r="F59">
+        <v>25</v>
+      </c>
+      <c r="G59" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H59" t="str">
+        <v/>
+      </c>
+      <c r="I59" t="str">
+        <v>ec2c93c7-60f2-4ef0-8a21-3cd88e5d1fa4.jpg</v>
+      </c>
+      <c r="J59" t="str">
+        <v/>
+      </c>
+      <c r="K59" t="str">
+        <v/>
+      </c>
+      <c r="L59" t="str">
+        <v>Recommended for babies up to 12 months of age.</v>
+      </c>
+      <c r="M59" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>KW-08</v>
+      </c>
+      <c r="B60" t="str">
+        <v>Kids frocks</v>
+      </c>
+      <c r="C60" t="str">
+        <v>Kids Wear</v>
+      </c>
+      <c r="D60" t="str">
+        <v/>
+      </c>
+      <c r="E60">
+        <v>30</v>
+      </c>
+      <c r="F60">
+        <v>30</v>
+      </c>
+      <c r="G60" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H60" t="str">
+        <v/>
+      </c>
+      <c r="I60" t="str">
+        <v>fc45e14f-c5c5-4019-9985-dcd19f9c981d.jpg</v>
+      </c>
+      <c r="J60" t="str">
+        <v/>
+      </c>
+      <c r="K60" t="str">
+        <v/>
+      </c>
+      <c r="L60" t="str">
+        <v/>
+      </c>
+      <c r="M60" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <v>KW-09</v>
+      </c>
+      <c r="B61" t="str">
+        <v>kids pattu pavada</v>
+      </c>
+      <c r="C61" t="str">
+        <v>Kids Wear</v>
+      </c>
+      <c r="D61" t="str">
+        <v/>
+      </c>
+      <c r="E61">
+        <v>38</v>
+      </c>
+      <c r="F61">
+        <v>45</v>
+      </c>
+      <c r="G61" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H61" t="str">
+        <v/>
+      </c>
+      <c r="I61" t="str">
+        <v>c88e7aaa-974a-4a2c-99ca-da73b75487da.jpg</v>
+      </c>
+      <c r="J61" t="str">
+        <v/>
+      </c>
+      <c r="K61" t="str">
+        <v/>
+      </c>
+      <c r="L61" t="str">
+        <v/>
+      </c>
+      <c r="M61" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <v>JW-21</v>
+      </c>
+      <c r="B62" t="str">
+        <v>stoned earrings</v>
+      </c>
+      <c r="C62" t="str">
+        <v>Jewellery</v>
+      </c>
+      <c r="D62" t="str">
+        <v>Earring</v>
+      </c>
+      <c r="E62">
+        <v>12.99</v>
+      </c>
+      <c r="F62">
+        <v>18</v>
+      </c>
+      <c r="G62" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H62" t="str">
+        <v/>
+      </c>
+      <c r="I62" t="str">
+        <v>f20a73b3-e5e9-4e60-a3be-7734accd7388.jpg</v>
+      </c>
+      <c r="J62" t="str">
+        <v/>
+      </c>
+      <c r="K62" t="str">
+        <v/>
+      </c>
+      <c r="L62" t="str">
+        <v/>
+      </c>
+      <c r="M62" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>LW-35</v>
+      </c>
+      <c r="B63" t="str">
+        <v>Jewellery</v>
+      </c>
+      <c r="C63" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D63" t="str">
+        <v/>
+      </c>
+      <c r="E63">
+        <v>15</v>
+      </c>
+      <c r="F63">
+        <v>24</v>
+      </c>
+      <c r="G63" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H63" t="str">
+        <v/>
+      </c>
+      <c r="I63" t="str">
+        <v>be5aecd5-ee30-4c54-919e-87aa0dd0992d.jpg</v>
+      </c>
+      <c r="J63" t="str">
+        <v/>
+      </c>
+      <c r="K63" t="str">
+        <v/>
+      </c>
+      <c r="L63" t="str">
+        <v/>
+      </c>
+      <c r="M63" t="str">
+        <v>No</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M53"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M63"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update store products via Admin Panel - 08/08/2026, 10:13:45 am
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M63"/>
+  <dimension ref="A1:M74"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2198,10 +2198,10 @@
         <v>Necklace</v>
       </c>
       <c r="E44">
-        <v>29.65</v>
+        <v>34</v>
       </c>
       <c r="F44">
-        <v>29.65</v>
+        <v>38</v>
       </c>
       <c r="G44" t="str">
         <v>INSTOCK</v>
@@ -3005,9 +3005,464 @@
         <v>No</v>
       </c>
     </row>
+    <row r="64">
+      <c r="A64" t="str">
+        <v>LW-36</v>
+      </c>
+      <c r="B64" t="str">
+        <v>Premium Bangle</v>
+      </c>
+      <c r="C64" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D64" t="str">
+        <v/>
+      </c>
+      <c r="E64">
+        <v>18</v>
+      </c>
+      <c r="F64">
+        <v>18</v>
+      </c>
+      <c r="G64" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H64" t="str">
+        <v/>
+      </c>
+      <c r="I64" t="str">
+        <v>455d2183-c9f1-4bbf-9f4f-f3d7ce5d688b.jpg</v>
+      </c>
+      <c r="J64" t="str">
+        <v/>
+      </c>
+      <c r="K64" t="str">
+        <v/>
+      </c>
+      <c r="L64" t="str">
+        <v>Limited stock</v>
+      </c>
+      <c r="M64" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="str">
+        <v>JW-22</v>
+      </c>
+      <c r="B65" t="str">
+        <v>Petal Jimukka</v>
+      </c>
+      <c r="C65" t="str">
+        <v>Jewellery</v>
+      </c>
+      <c r="D65" t="str">
+        <v>Earring</v>
+      </c>
+      <c r="E65">
+        <v>24</v>
+      </c>
+      <c r="F65">
+        <v>24</v>
+      </c>
+      <c r="G65" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H65" t="str">
+        <v/>
+      </c>
+      <c r="I65" t="str">
+        <v>989e9fab-ee88-4645-a544-a61880a527b7.jpg</v>
+      </c>
+      <c r="J65" t="str">
+        <v/>
+      </c>
+      <c r="K65" t="str">
+        <v/>
+      </c>
+      <c r="L65" t="str">
+        <v/>
+      </c>
+      <c r="M65" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="str">
+        <v>JW-23</v>
+      </c>
+      <c r="B66" t="str">
+        <v>Kasimala with stones</v>
+      </c>
+      <c r="C66" t="str">
+        <v>Jewellery</v>
+      </c>
+      <c r="D66" t="str">
+        <v>Necklace</v>
+      </c>
+      <c r="E66">
+        <v>34</v>
+      </c>
+      <c r="F66">
+        <v>36</v>
+      </c>
+      <c r="G66" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H66" t="str">
+        <v/>
+      </c>
+      <c r="I66" t="str">
+        <v>62ef44bd-3127-4ecb-9d35-df699663797a.jpg</v>
+      </c>
+      <c r="J66" t="str">
+        <v/>
+      </c>
+      <c r="K66" t="str">
+        <v/>
+      </c>
+      <c r="L66" t="str">
+        <v/>
+      </c>
+      <c r="M66" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="67" xml:space="preserve">
+      <c r="A67" t="str">
+        <v>KW-10</v>
+      </c>
+      <c r="B67" t="str">
+        <v>Kids frocks</v>
+      </c>
+      <c r="C67" t="str">
+        <v>Kids Wear</v>
+      </c>
+      <c r="D67" t="str">
+        <v/>
+      </c>
+      <c r="E67">
+        <v>16</v>
+      </c>
+      <c r="F67">
+        <v>24</v>
+      </c>
+      <c r="G67" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H67" t="str">
+        <v/>
+      </c>
+      <c r="I67" t="str">
+        <v>51f84db3-d4bf-4aec-88e2-2a5b5ffc86be.jpg</v>
+      </c>
+      <c r="J67" t="str">
+        <v>b68d0f08-456c-4856-97b0-16ff12a60bfd.jpg</v>
+      </c>
+      <c r="K67" t="str">
+        <v>44e75bbc-1de7-4e05-a227-b1931edd7c3e.jpg</v>
+      </c>
+      <c r="L67" t="str" xml:space="preserve">
+        <v xml:space="preserve">Available Sizes: 0–3 Months | 3–6 Months | 6–9 Months | 9–12 Months
+Material- Soft Cotton</v>
+      </c>
+      <c r="M67" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="68" xml:space="preserve">
+      <c r="A68" t="str">
+        <v>LW-37</v>
+      </c>
+      <c r="B68" t="str">
+        <v>Kids frocks</v>
+      </c>
+      <c r="C68" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D68" t="str">
+        <v/>
+      </c>
+      <c r="E68">
+        <v>16</v>
+      </c>
+      <c r="F68">
+        <v>20</v>
+      </c>
+      <c r="G68" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H68" t="str">
+        <v/>
+      </c>
+      <c r="I68" t="str">
+        <v>e07e48ed-c2ba-4a79-8392-aeb18a6bc388.jpg</v>
+      </c>
+      <c r="J68" t="str">
+        <v>8bcde40e-95bf-48e4-8a1b-70f126aef16b.jpg</v>
+      </c>
+      <c r="K68" t="str">
+        <v/>
+      </c>
+      <c r="L68" t="str" xml:space="preserve">
+        <v xml:space="preserve">Available Sizes: 0–3 Months | 3–6 Months | 6–9 Months | 9–12 Months
+Material-Soft Georgette.
+Soft lining-included</v>
+      </c>
+      <c r="M68" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="69" xml:space="preserve">
+      <c r="A69" t="str">
+        <v>LW-38</v>
+      </c>
+      <c r="B69" t="str">
+        <v>Kids frocks</v>
+      </c>
+      <c r="C69" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D69" t="str">
+        <v/>
+      </c>
+      <c r="E69">
+        <v>23</v>
+      </c>
+      <c r="F69">
+        <v>30</v>
+      </c>
+      <c r="G69" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H69" t="str">
+        <v/>
+      </c>
+      <c r="I69" t="str">
+        <v>5031150e-3915-4443-801e-a24f17b8a3c6.jpg</v>
+      </c>
+      <c r="J69" t="str">
+        <v>cff7208c-1004-41c9-a035-c6656621bfec.jpg</v>
+      </c>
+      <c r="K69" t="str">
+        <v/>
+      </c>
+      <c r="L69" t="str" xml:space="preserve">
+        <v xml:space="preserve">Sizes available up to  3 year
+Fabric- Satin and Net</v>
+      </c>
+      <c r="M69" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="str">
+        <v>KW-11</v>
+      </c>
+      <c r="B70" t="str">
+        <v>Kids frocks</v>
+      </c>
+      <c r="C70" t="str">
+        <v>Kids Wear</v>
+      </c>
+      <c r="D70" t="str">
+        <v/>
+      </c>
+      <c r="E70">
+        <v>24</v>
+      </c>
+      <c r="F70">
+        <v>32</v>
+      </c>
+      <c r="G70" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H70" t="str">
+        <v/>
+      </c>
+      <c r="I70" t="str">
+        <v>a8acd117-01a4-4c8e-b2d7-6371aaa6d04f.jpg</v>
+      </c>
+      <c r="J70" t="str">
+        <v/>
+      </c>
+      <c r="K70" t="str">
+        <v/>
+      </c>
+      <c r="L70" t="str">
+        <v>sizes available up to 2 years</v>
+      </c>
+      <c r="M70" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="str">
+        <v>JW-24</v>
+      </c>
+      <c r="B71" t="str">
+        <v>Necklace</v>
+      </c>
+      <c r="C71" t="str">
+        <v>Jewellery</v>
+      </c>
+      <c r="D71" t="str">
+        <v>Necklace</v>
+      </c>
+      <c r="E71">
+        <v>14</v>
+      </c>
+      <c r="F71">
+        <v>19</v>
+      </c>
+      <c r="G71" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H71" t="str">
+        <v/>
+      </c>
+      <c r="I71" t="str">
+        <v>953e407b-d27a-4e5b-b6e1-f713f5754642.jpg</v>
+      </c>
+      <c r="J71" t="str">
+        <v>a00fcf05-b192-4188-93a8-827517720bc5.jpg</v>
+      </c>
+      <c r="K71" t="str">
+        <v/>
+      </c>
+      <c r="L71" t="str">
+        <v>Casual wear</v>
+      </c>
+      <c r="M71" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="str">
+        <v>JW-25</v>
+      </c>
+      <c r="B72" t="str">
+        <v>Premium AD stone necklace</v>
+      </c>
+      <c r="C72" t="str">
+        <v>Jewellery</v>
+      </c>
+      <c r="D72" t="str">
+        <v>Necklace</v>
+      </c>
+      <c r="E72">
+        <v>44</v>
+      </c>
+      <c r="F72">
+        <v>49</v>
+      </c>
+      <c r="G72" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H72" t="str">
+        <v/>
+      </c>
+      <c r="I72" t="str">
+        <v>32921a7c-6ea9-40e1-a74c-58afe2134b46.jpg</v>
+      </c>
+      <c r="J72" t="str">
+        <v/>
+      </c>
+      <c r="K72" t="str">
+        <v/>
+      </c>
+      <c r="L72" t="str">
+        <v/>
+      </c>
+      <c r="M72" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="str">
+        <v>JW-26</v>
+      </c>
+      <c r="B73" t="str">
+        <v>Jewellery</v>
+      </c>
+      <c r="C73" t="str">
+        <v>Jewellery</v>
+      </c>
+      <c r="D73" t="str">
+        <v>Earring</v>
+      </c>
+      <c r="E73">
+        <v>13</v>
+      </c>
+      <c r="F73">
+        <v>16</v>
+      </c>
+      <c r="G73" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H73" t="str">
+        <v/>
+      </c>
+      <c r="I73" t="str">
+        <v>d5db144a-3d37-47be-b9b0-398b05112869.jpg</v>
+      </c>
+      <c r="J73" t="str">
+        <v/>
+      </c>
+      <c r="K73" t="str">
+        <v/>
+      </c>
+      <c r="L73" t="str">
+        <v/>
+      </c>
+      <c r="M73" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="str">
+        <v>LW-39</v>
+      </c>
+      <c r="B74" t="str">
+        <v>Premium double layer</v>
+      </c>
+      <c r="C74" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D74" t="str">
+        <v/>
+      </c>
+      <c r="E74">
+        <v>39</v>
+      </c>
+      <c r="F74">
+        <v>46</v>
+      </c>
+      <c r="G74" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H74" t="str">
+        <v/>
+      </c>
+      <c r="I74" t="str">
+        <v>2842e9ba-4425-4141-a85f-5ef2fdcafb5a.jpg</v>
+      </c>
+      <c r="J74" t="str">
+        <v/>
+      </c>
+      <c r="K74" t="str">
+        <v/>
+      </c>
+      <c r="L74" t="str">
+        <v>double layer premium necklace</v>
+      </c>
+      <c r="M74" t="str">
+        <v>No</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M63"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M74"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update store products via Admin Panel - 08/08/2026, 1:00:39 pm
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M74"/>
+  <dimension ref="A1:M75"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1456,7 +1456,7 @@
         <v>Jewellery</v>
       </c>
       <c r="D26" t="str">
-        <v>Necklace</v>
+        <v>Bangles</v>
       </c>
       <c r="E26">
         <v>23</v>
@@ -1480,7 +1480,7 @@
         <v/>
       </c>
       <c r="L26" t="str">
-        <v/>
+        <v>Pair -$23</v>
       </c>
       <c r="M26" t="str">
         <v>No</v>
@@ -2608,10 +2608,10 @@
         <v/>
       </c>
       <c r="E54">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="F54">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="G54" t="str">
         <v>INSTOCK</v>
@@ -3460,9 +3460,50 @@
         <v>No</v>
       </c>
     </row>
+    <row r="75">
+      <c r="A75" t="str">
+        <v>LW-40</v>
+      </c>
+      <c r="B75" t="str">
+        <v>Ready made churidar</v>
+      </c>
+      <c r="C75" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D75" t="str">
+        <v/>
+      </c>
+      <c r="E75">
+        <v>75</v>
+      </c>
+      <c r="F75">
+        <v>85</v>
+      </c>
+      <c r="G75" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H75" t="str">
+        <v>size-L</v>
+      </c>
+      <c r="I75" t="str">
+        <v>96ca04a7-3dca-467e-9673-8bc9c09cd520.jpg</v>
+      </c>
+      <c r="J75" t="str">
+        <v/>
+      </c>
+      <c r="K75" t="str">
+        <v/>
+      </c>
+      <c r="L75" t="str">
+        <v/>
+      </c>
+      <c r="M75" t="str">
+        <v>No</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M74"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M75"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update store products via Admin Panel - 08/08/2026, 7:38:34 pm
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M75"/>
+  <dimension ref="A1:M86"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2858,7 +2858,7 @@
         <v>30</v>
       </c>
       <c r="F60">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="G60" t="str">
         <v>INSTOCK</v>
@@ -2896,7 +2896,7 @@
         <v/>
       </c>
       <c r="E61">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="F61">
         <v>45</v>
@@ -3501,9 +3501,474 @@
         <v>No</v>
       </c>
     </row>
+    <row r="76" xml:space="preserve">
+      <c r="A76" t="str">
+        <v>LW-41</v>
+      </c>
+      <c r="B76" t="str">
+        <v>Readymade blouse</v>
+      </c>
+      <c r="C76" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D76" t="str">
+        <v/>
+      </c>
+      <c r="E76">
+        <v>45</v>
+      </c>
+      <c r="F76">
+        <v>45</v>
+      </c>
+      <c r="G76" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H76" t="str">
+        <v>free size</v>
+      </c>
+      <c r="I76" t="str">
+        <v>c71315d5-087c-4e27-8627-641b744bc3a5.jpg</v>
+      </c>
+      <c r="J76" t="str">
+        <v/>
+      </c>
+      <c r="K76" t="str">
+        <v/>
+      </c>
+      <c r="L76" t="str" xml:space="preserve">
+        <v xml:space="preserve">Free size
+Chest  margin 34-40 inch 
+Alterable</v>
+      </c>
+      <c r="M76" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="77" xml:space="preserve">
+      <c r="A77" t="str">
+        <v>LW-42</v>
+      </c>
+      <c r="B77" t="str">
+        <v>Readymade Blouse</v>
+      </c>
+      <c r="C77" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D77" t="str">
+        <v/>
+      </c>
+      <c r="E77">
+        <v>40</v>
+      </c>
+      <c r="F77">
+        <v>45</v>
+      </c>
+      <c r="G77" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H77" t="str">
+        <v>Free size</v>
+      </c>
+      <c r="I77" t="str">
+        <v>bef0ca17-dab0-455f-a404-d2144e3dc2a0.jpg</v>
+      </c>
+      <c r="J77" t="str">
+        <v/>
+      </c>
+      <c r="K77" t="str">
+        <v/>
+      </c>
+      <c r="L77" t="str" xml:space="preserve">
+        <v xml:space="preserve">Free size
+Chest  margin 34-40 inch 
+Alterable</v>
+      </c>
+      <c r="M77" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="78" xml:space="preserve">
+      <c r="A78" t="str">
+        <v>LW-43</v>
+      </c>
+      <c r="B78" t="str">
+        <v>Free Size</v>
+      </c>
+      <c r="C78" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D78" t="str">
+        <v/>
+      </c>
+      <c r="E78">
+        <v>40</v>
+      </c>
+      <c r="F78">
+        <v>45</v>
+      </c>
+      <c r="G78" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H78" t="str">
+        <v>Free Size</v>
+      </c>
+      <c r="I78" t="str">
+        <v>e2a182ea-ccca-4e02-a77e-8512a4471618.jpg</v>
+      </c>
+      <c r="J78" t="str">
+        <v/>
+      </c>
+      <c r="K78" t="str">
+        <v/>
+      </c>
+      <c r="L78" t="str" xml:space="preserve">
+        <v xml:space="preserve">Free size
+Chest  margin 34-40 inch 
+Alterable</v>
+      </c>
+      <c r="M78" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="79" xml:space="preserve">
+      <c r="A79" t="str">
+        <v>LW-44</v>
+      </c>
+      <c r="B79" t="str">
+        <v>Ready made blouse</v>
+      </c>
+      <c r="C79" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D79" t="str">
+        <v/>
+      </c>
+      <c r="E79">
+        <v>45</v>
+      </c>
+      <c r="F79">
+        <v>48</v>
+      </c>
+      <c r="G79" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H79" t="str">
+        <v/>
+      </c>
+      <c r="I79" t="str">
+        <v>f9ec3b8b-ef32-4114-a076-22acf36d6858.jpg</v>
+      </c>
+      <c r="J79" t="str">
+        <v/>
+      </c>
+      <c r="K79" t="str">
+        <v/>
+      </c>
+      <c r="L79" t="str" xml:space="preserve">
+        <v xml:space="preserve">Free size
+Chest  margin 34-40 inch 
+Alterable</v>
+      </c>
+      <c r="M79" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="80" xml:space="preserve">
+      <c r="A80" t="str">
+        <v>LW-45</v>
+      </c>
+      <c r="B80" t="str">
+        <v>Readymade blouse</v>
+      </c>
+      <c r="C80" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D80" t="str">
+        <v/>
+      </c>
+      <c r="E80">
+        <v>45</v>
+      </c>
+      <c r="F80">
+        <v>48</v>
+      </c>
+      <c r="G80" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H80" t="str">
+        <v>Free size</v>
+      </c>
+      <c r="I80" t="str">
+        <v>33eaed97-ffa5-43b6-9e79-fe90c44b842c.jpg</v>
+      </c>
+      <c r="J80" t="str">
+        <v/>
+      </c>
+      <c r="K80" t="str">
+        <v/>
+      </c>
+      <c r="L80" t="str" xml:space="preserve">
+        <v xml:space="preserve">Free size
+Chest  margin 34-40 inch 
+Alterable</v>
+      </c>
+      <c r="M80" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="81" xml:space="preserve">
+      <c r="A81" t="str">
+        <v>LW-46</v>
+      </c>
+      <c r="B81" t="str">
+        <v>Ready made blouse</v>
+      </c>
+      <c r="C81" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D81" t="str">
+        <v/>
+      </c>
+      <c r="E81">
+        <v>45</v>
+      </c>
+      <c r="F81">
+        <v>48</v>
+      </c>
+      <c r="G81" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H81" t="str">
+        <v>Freesize</v>
+      </c>
+      <c r="I81" t="str">
+        <v>2705b52e-096c-4e79-b5f3-8754c6015f28.jpg</v>
+      </c>
+      <c r="J81" t="str">
+        <v/>
+      </c>
+      <c r="K81" t="str">
+        <v/>
+      </c>
+      <c r="L81" t="str" xml:space="preserve">
+        <v xml:space="preserve">Free size
+Chest  margin 34-40 inch 
+Alterable</v>
+      </c>
+      <c r="M81" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="82" xml:space="preserve">
+      <c r="A82" t="str">
+        <v>LW-47</v>
+      </c>
+      <c r="B82" t="str">
+        <v>Free size</v>
+      </c>
+      <c r="C82" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D82" t="str">
+        <v/>
+      </c>
+      <c r="E82">
+        <v>45</v>
+      </c>
+      <c r="F82">
+        <v>48</v>
+      </c>
+      <c r="G82" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H82" t="str">
+        <v>Free size</v>
+      </c>
+      <c r="I82" t="str">
+        <v>28151555-6c9c-4a86-b3bb-5fed1c7fcbdc.jpg</v>
+      </c>
+      <c r="J82" t="str">
+        <v/>
+      </c>
+      <c r="K82" t="str">
+        <v/>
+      </c>
+      <c r="L82" t="str" xml:space="preserve">
+        <v xml:space="preserve">Free size
+Chest  margin 34-40 inch 
+Alterable</v>
+      </c>
+      <c r="M82" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="str">
+        <v>LW-48</v>
+      </c>
+      <c r="B83" t="str">
+        <v>soft organza saree</v>
+      </c>
+      <c r="C83" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D83" t="str">
+        <v/>
+      </c>
+      <c r="E83">
+        <v>89</v>
+      </c>
+      <c r="F83">
+        <v>95</v>
+      </c>
+      <c r="G83" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H83" t="str">
+        <v/>
+      </c>
+      <c r="I83" t="str">
+        <v>ff4a2947-89fa-412c-91d7-6ebe043c24f9.jpg</v>
+      </c>
+      <c r="J83" t="str">
+        <v/>
+      </c>
+      <c r="K83" t="str">
+        <v/>
+      </c>
+      <c r="L83" t="str">
+        <v>unstitched blouse</v>
+      </c>
+      <c r="M83" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="str">
+        <v>LW-49</v>
+      </c>
+      <c r="B84" t="str">
+        <v>semi tusser silk</v>
+      </c>
+      <c r="C84" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D84" t="str">
+        <v/>
+      </c>
+      <c r="E84">
+        <v>76</v>
+      </c>
+      <c r="F84">
+        <v>85</v>
+      </c>
+      <c r="G84" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H84" t="str">
+        <v/>
+      </c>
+      <c r="I84" t="str">
+        <v>cf1b0bea-3bba-4185-936d-e21a7b9cb63e.jpg</v>
+      </c>
+      <c r="J84" t="str">
+        <v/>
+      </c>
+      <c r="K84" t="str">
+        <v/>
+      </c>
+      <c r="L84" t="str">
+        <v/>
+      </c>
+      <c r="M84" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="str">
+        <v>LW-50</v>
+      </c>
+      <c r="B85" t="str">
+        <v>semi tusser saree</v>
+      </c>
+      <c r="C85" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D85" t="str">
+        <v/>
+      </c>
+      <c r="E85">
+        <v>76</v>
+      </c>
+      <c r="F85">
+        <v>85</v>
+      </c>
+      <c r="G85" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H85" t="str">
+        <v/>
+      </c>
+      <c r="I85" t="str">
+        <v>057421ca-10bb-4a81-9f23-570e65d9dd5d.jpg</v>
+      </c>
+      <c r="J85" t="str">
+        <v/>
+      </c>
+      <c r="K85" t="str">
+        <v/>
+      </c>
+      <c r="L85" t="str">
+        <v/>
+      </c>
+      <c r="M85" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="str">
+        <v>LW-51</v>
+      </c>
+      <c r="B86" t="str">
+        <v>Semi tusser silk sarees</v>
+      </c>
+      <c r="C86" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D86" t="str">
+        <v/>
+      </c>
+      <c r="E86">
+        <v>83</v>
+      </c>
+      <c r="F86">
+        <v>90</v>
+      </c>
+      <c r="G86" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H86" t="str">
+        <v/>
+      </c>
+      <c r="I86" t="str">
+        <v>e5a4ba5d-7dfd-4106-830e-6f1527c6a7fc.jpg</v>
+      </c>
+      <c r="J86" t="str">
+        <v/>
+      </c>
+      <c r="K86" t="str">
+        <v/>
+      </c>
+      <c r="L86" t="str">
+        <v/>
+      </c>
+      <c r="M86" t="str">
+        <v>No</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M75"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M86"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update store products via Admin Panel - 08/08/2026, 7:54:02 pm
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -946,12 +946,12 @@
         <v>No</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" xml:space="preserve">
       <c r="A14" t="str">
         <v>LW-06</v>
       </c>
       <c r="B14" t="str">
-        <v>Premium Cotton Embroidered Blouse</v>
+        <v>Premium  Hakoba  Embroidered Blouse</v>
       </c>
       <c r="C14" t="str">
         <v>Ladies Wear</v>
@@ -980,8 +980,10 @@
       <c r="K14" t="str">
         <v>10ab4c9a-7855-40f5-bb4b-23a50b41b728.jpg</v>
       </c>
-      <c r="L14" t="str">
-        <v/>
+      <c r="L14" t="str" xml:space="preserve">
+        <v xml:space="preserve">Free size
+Chest  margin 34-40 inch 
+Alterable</v>
       </c>
       <c r="M14" t="str">
         <v>No</v>

</xml_diff>

<commit_message>
Update store products via Admin Panel - 09/08/2026, 1:21:04 am
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M86"/>
+  <dimension ref="A1:M118"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3009,22 +3009,22 @@
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>LW-36</v>
+        <v>JW-22</v>
       </c>
       <c r="B64" t="str">
-        <v>Premium Bangle</v>
+        <v>Petal Jimukka</v>
       </c>
       <c r="C64" t="str">
-        <v>Ladies Wear</v>
+        <v>Jewellery</v>
       </c>
       <c r="D64" t="str">
-        <v/>
+        <v>Earring</v>
       </c>
       <c r="E64">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="F64">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G64" t="str">
         <v>INSTOCK</v>
@@ -3033,7 +3033,7 @@
         <v/>
       </c>
       <c r="I64" t="str">
-        <v>455d2183-c9f1-4bbf-9f4f-f3d7ce5d688b.jpg</v>
+        <v>989e9fab-ee88-4645-a544-a61880a527b7.jpg</v>
       </c>
       <c r="J64" t="str">
         <v/>
@@ -3042,7 +3042,7 @@
         <v/>
       </c>
       <c r="L64" t="str">
-        <v>Limited stock</v>
+        <v/>
       </c>
       <c r="M64" t="str">
         <v>No</v>
@@ -3050,64 +3050,64 @@
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>JW-22</v>
+        <v>JW-23</v>
       </c>
       <c r="B65" t="str">
-        <v>Petal Jimukka</v>
+        <v>Kasimala with stones</v>
       </c>
       <c r="C65" t="str">
         <v>Jewellery</v>
       </c>
       <c r="D65" t="str">
-        <v>Earring</v>
+        <v>Necklace</v>
       </c>
       <c r="E65">
+        <v>34</v>
+      </c>
+      <c r="F65">
+        <v>36</v>
+      </c>
+      <c r="G65" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H65" t="str">
+        <v/>
+      </c>
+      <c r="I65" t="str">
+        <v>62ef44bd-3127-4ecb-9d35-df699663797a.jpg</v>
+      </c>
+      <c r="J65" t="str">
+        <v/>
+      </c>
+      <c r="K65" t="str">
+        <v/>
+      </c>
+      <c r="L65" t="str">
+        <v/>
+      </c>
+      <c r="M65" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="66" xml:space="preserve">
+      <c r="A66" t="str">
+        <v>KW-10</v>
+      </c>
+      <c r="B66" t="str">
+        <v>Kids frocks</v>
+      </c>
+      <c r="C66" t="str">
+        <v>Kids Wear</v>
+      </c>
+      <c r="D66" t="str">
+        <v/>
+      </c>
+      <c r="E66">
+        <v>16</v>
+      </c>
+      <c r="F66">
         <v>24</v>
       </c>
-      <c r="F65">
-        <v>24</v>
-      </c>
-      <c r="G65" t="str">
-        <v>INSTOCK</v>
-      </c>
-      <c r="H65" t="str">
-        <v/>
-      </c>
-      <c r="I65" t="str">
-        <v>989e9fab-ee88-4645-a544-a61880a527b7.jpg</v>
-      </c>
-      <c r="J65" t="str">
-        <v/>
-      </c>
-      <c r="K65" t="str">
-        <v/>
-      </c>
-      <c r="L65" t="str">
-        <v/>
-      </c>
-      <c r="M65" t="str">
-        <v>No</v>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="str">
-        <v>JW-23</v>
-      </c>
-      <c r="B66" t="str">
-        <v>Kasimala with stones</v>
-      </c>
-      <c r="C66" t="str">
-        <v>Jewellery</v>
-      </c>
-      <c r="D66" t="str">
-        <v>Necklace</v>
-      </c>
-      <c r="E66">
-        <v>34</v>
-      </c>
-      <c r="F66">
-        <v>36</v>
-      </c>
       <c r="G66" t="str">
         <v>INSTOCK</v>
       </c>
@@ -3115,16 +3115,17 @@
         <v/>
       </c>
       <c r="I66" t="str">
-        <v>62ef44bd-3127-4ecb-9d35-df699663797a.jpg</v>
+        <v>51f84db3-d4bf-4aec-88e2-2a5b5ffc86be.jpg</v>
       </c>
       <c r="J66" t="str">
-        <v/>
+        <v>b68d0f08-456c-4856-97b0-16ff12a60bfd.jpg</v>
       </c>
       <c r="K66" t="str">
-        <v/>
-      </c>
-      <c r="L66" t="str">
-        <v/>
+        <v>44e75bbc-1de7-4e05-a227-b1931edd7c3e.jpg</v>
+      </c>
+      <c r="L66" t="str" xml:space="preserve">
+        <v xml:space="preserve">Available Sizes: 0–3 Months | 3–6 Months | 6–9 Months | 9–12 Months
+Material- Soft Cotton</v>
       </c>
       <c r="M66" t="str">
         <v>No</v>
@@ -3132,13 +3133,13 @@
     </row>
     <row r="67" xml:space="preserve">
       <c r="A67" t="str">
-        <v>KW-10</v>
+        <v>LW-37</v>
       </c>
       <c r="B67" t="str">
         <v>Kids frocks</v>
       </c>
       <c r="C67" t="str">
-        <v>Kids Wear</v>
+        <v>Ladies Wear</v>
       </c>
       <c r="D67" t="str">
         <v/>
@@ -3147,7 +3148,7 @@
         <v>16</v>
       </c>
       <c r="F67">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="G67" t="str">
         <v>INSTOCK</v>
@@ -3156,83 +3157,83 @@
         <v/>
       </c>
       <c r="I67" t="str">
-        <v>51f84db3-d4bf-4aec-88e2-2a5b5ffc86be.jpg</v>
+        <v>e07e48ed-c2ba-4a79-8392-aeb18a6bc388.jpg</v>
       </c>
       <c r="J67" t="str">
-        <v>b68d0f08-456c-4856-97b0-16ff12a60bfd.jpg</v>
+        <v>8bcde40e-95bf-48e4-8a1b-70f126aef16b.jpg</v>
       </c>
       <c r="K67" t="str">
-        <v>44e75bbc-1de7-4e05-a227-b1931edd7c3e.jpg</v>
+        <v/>
       </c>
       <c r="L67" t="str" xml:space="preserve">
-        <v xml:space="preserve">Available Sizes: 0–3 Months | 3–6 Months | 6–9 Months | 9–12 Months
-Material- Soft Cotton</v>
-      </c>
-      <c r="M67" t="str">
-        <v>No</v>
-      </c>
-    </row>
-    <row r="68" xml:space="preserve">
-      <c r="A68" t="str">
-        <v>LW-37</v>
-      </c>
-      <c r="B68" t="str">
-        <v>Kids frocks</v>
-      </c>
-      <c r="C68" t="str">
-        <v>Ladies Wear</v>
-      </c>
-      <c r="D68" t="str">
-        <v/>
-      </c>
-      <c r="E68">
-        <v>16</v>
-      </c>
-      <c r="F68">
-        <v>20</v>
-      </c>
-      <c r="G68" t="str">
-        <v>INSTOCK</v>
-      </c>
-      <c r="H68" t="str">
-        <v/>
-      </c>
-      <c r="I68" t="str">
-        <v>e07e48ed-c2ba-4a79-8392-aeb18a6bc388.jpg</v>
-      </c>
-      <c r="J68" t="str">
-        <v>8bcde40e-95bf-48e4-8a1b-70f126aef16b.jpg</v>
-      </c>
-      <c r="K68" t="str">
-        <v/>
-      </c>
-      <c r="L68" t="str" xml:space="preserve">
         <v xml:space="preserve">Available Sizes: 0–3 Months | 3–6 Months | 6–9 Months | 9–12 Months
 Material-Soft Georgette.
 Soft lining-included</v>
       </c>
+      <c r="M67" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="68" xml:space="preserve">
+      <c r="A68" t="str">
+        <v>LW-38</v>
+      </c>
+      <c r="B68" t="str">
+        <v>Kids frocks</v>
+      </c>
+      <c r="C68" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D68" t="str">
+        <v/>
+      </c>
+      <c r="E68">
+        <v>23</v>
+      </c>
+      <c r="F68">
+        <v>30</v>
+      </c>
+      <c r="G68" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H68" t="str">
+        <v/>
+      </c>
+      <c r="I68" t="str">
+        <v>5031150e-3915-4443-801e-a24f17b8a3c6.jpg</v>
+      </c>
+      <c r="J68" t="str">
+        <v>cff7208c-1004-41c9-a035-c6656621bfec.jpg</v>
+      </c>
+      <c r="K68" t="str">
+        <v/>
+      </c>
+      <c r="L68" t="str" xml:space="preserve">
+        <v xml:space="preserve">Sizes available up to  3 year
+Fabric- Satin and Net</v>
+      </c>
       <c r="M68" t="str">
         <v>No</v>
       </c>
     </row>
-    <row r="69" xml:space="preserve">
+    <row r="69">
       <c r="A69" t="str">
-        <v>LW-38</v>
+        <v>KW-11</v>
       </c>
       <c r="B69" t="str">
         <v>Kids frocks</v>
       </c>
       <c r="C69" t="str">
-        <v>Ladies Wear</v>
+        <v>Kids Wear</v>
       </c>
       <c r="D69" t="str">
         <v/>
       </c>
       <c r="E69">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F69">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="G69" t="str">
         <v>INSTOCK</v>
@@ -3241,17 +3242,16 @@
         <v/>
       </c>
       <c r="I69" t="str">
-        <v>5031150e-3915-4443-801e-a24f17b8a3c6.jpg</v>
+        <v>a8acd117-01a4-4c8e-b2d7-6371aaa6d04f.jpg</v>
       </c>
       <c r="J69" t="str">
-        <v>cff7208c-1004-41c9-a035-c6656621bfec.jpg</v>
+        <v/>
       </c>
       <c r="K69" t="str">
         <v/>
       </c>
-      <c r="L69" t="str" xml:space="preserve">
-        <v xml:space="preserve">Sizes available up to  3 year
-Fabric- Satin and Net</v>
+      <c r="L69" t="str">
+        <v>sizes available up to 2 years</v>
       </c>
       <c r="M69" t="str">
         <v>No</v>
@@ -3259,22 +3259,22 @@
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>KW-11</v>
+        <v>JW-24</v>
       </c>
       <c r="B70" t="str">
-        <v>Kids frocks</v>
+        <v>Necklace</v>
       </c>
       <c r="C70" t="str">
-        <v>Kids Wear</v>
+        <v>Jewellery</v>
       </c>
       <c r="D70" t="str">
-        <v/>
+        <v>Necklace</v>
       </c>
       <c r="E70">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F70">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="G70" t="str">
         <v>INSTOCK</v>
@@ -3283,16 +3283,16 @@
         <v/>
       </c>
       <c r="I70" t="str">
-        <v>a8acd117-01a4-4c8e-b2d7-6371aaa6d04f.jpg</v>
+        <v>953e407b-d27a-4e5b-b6e1-f713f5754642.jpg</v>
       </c>
       <c r="J70" t="str">
-        <v/>
+        <v>a00fcf05-b192-4188-93a8-827517720bc5.jpg</v>
       </c>
       <c r="K70" t="str">
         <v/>
       </c>
       <c r="L70" t="str">
-        <v>sizes available up to 2 years</v>
+        <v>Casual wear</v>
       </c>
       <c r="M70" t="str">
         <v>No</v>
@@ -3300,10 +3300,10 @@
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>JW-24</v>
+        <v>JW-25</v>
       </c>
       <c r="B71" t="str">
-        <v>Necklace</v>
+        <v>Premium AD stone necklace</v>
       </c>
       <c r="C71" t="str">
         <v>Jewellery</v>
@@ -3312,10 +3312,10 @@
         <v>Necklace</v>
       </c>
       <c r="E71">
-        <v>14</v>
+        <v>44</v>
       </c>
       <c r="F71">
-        <v>19</v>
+        <v>49</v>
       </c>
       <c r="G71" t="str">
         <v>INSTOCK</v>
@@ -3324,39 +3324,39 @@
         <v/>
       </c>
       <c r="I71" t="str">
-        <v>953e407b-d27a-4e5b-b6e1-f713f5754642.jpg</v>
+        <v>32921a7c-6ea9-40e1-a74c-58afe2134b46.jpg</v>
       </c>
       <c r="J71" t="str">
-        <v>a00fcf05-b192-4188-93a8-827517720bc5.jpg</v>
+        <v/>
       </c>
       <c r="K71" t="str">
         <v/>
       </c>
       <c r="L71" t="str">
-        <v>Casual wear</v>
+        <v/>
       </c>
       <c r="M71" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>JW-25</v>
+        <v>JW-26</v>
       </c>
       <c r="B72" t="str">
-        <v>Premium AD stone necklace</v>
+        <v>Jewellery</v>
       </c>
       <c r="C72" t="str">
         <v>Jewellery</v>
       </c>
       <c r="D72" t="str">
-        <v>Necklace</v>
+        <v>Earring</v>
       </c>
       <c r="E72">
-        <v>44</v>
+        <v>13</v>
       </c>
       <c r="F72">
-        <v>49</v>
+        <v>16</v>
       </c>
       <c r="G72" t="str">
         <v>INSTOCK</v>
@@ -3365,7 +3365,7 @@
         <v/>
       </c>
       <c r="I72" t="str">
-        <v>32921a7c-6ea9-40e1-a74c-58afe2134b46.jpg</v>
+        <v>d5db144a-3d37-47be-b9b0-398b05112869.jpg</v>
       </c>
       <c r="J72" t="str">
         <v/>
@@ -3377,27 +3377,27 @@
         <v/>
       </c>
       <c r="M72" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>JW-26</v>
+        <v>LW-39</v>
       </c>
       <c r="B73" t="str">
-        <v>Jewellery</v>
+        <v>Premium double layer</v>
       </c>
       <c r="C73" t="str">
-        <v>Jewellery</v>
+        <v>Ladies Wear</v>
       </c>
       <c r="D73" t="str">
-        <v>Earring</v>
+        <v/>
       </c>
       <c r="E73">
-        <v>13</v>
+        <v>39</v>
       </c>
       <c r="F73">
-        <v>16</v>
+        <v>46</v>
       </c>
       <c r="G73" t="str">
         <v>INSTOCK</v>
@@ -3406,7 +3406,7 @@
         <v/>
       </c>
       <c r="I73" t="str">
-        <v>d5db144a-3d37-47be-b9b0-398b05112869.jpg</v>
+        <v>2842e9ba-4425-4141-a85f-5ef2fdcafb5a.jpg</v>
       </c>
       <c r="J73" t="str">
         <v/>
@@ -3415,7 +3415,7 @@
         <v/>
       </c>
       <c r="L73" t="str">
-        <v/>
+        <v>double layer premium necklace</v>
       </c>
       <c r="M73" t="str">
         <v>No</v>
@@ -3423,10 +3423,10 @@
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>LW-39</v>
+        <v>LW-40</v>
       </c>
       <c r="B74" t="str">
-        <v>Premium double layer</v>
+        <v>Ready made churidar</v>
       </c>
       <c r="C74" t="str">
         <v>Ladies Wear</v>
@@ -3435,19 +3435,19 @@
         <v/>
       </c>
       <c r="E74">
-        <v>39</v>
+        <v>75</v>
       </c>
       <c r="F74">
-        <v>46</v>
+        <v>85</v>
       </c>
       <c r="G74" t="str">
         <v>INSTOCK</v>
       </c>
       <c r="H74" t="str">
-        <v/>
+        <v>size-L</v>
       </c>
       <c r="I74" t="str">
-        <v>2842e9ba-4425-4141-a85f-5ef2fdcafb5a.jpg</v>
+        <v>96ca04a7-3dca-467e-9673-8bc9c09cd520.jpg</v>
       </c>
       <c r="J74" t="str">
         <v/>
@@ -3456,18 +3456,18 @@
         <v/>
       </c>
       <c r="L74" t="str">
-        <v>double layer premium necklace</v>
+        <v/>
       </c>
       <c r="M74" t="str">
         <v>No</v>
       </c>
     </row>
-    <row r="75">
+    <row r="75" xml:space="preserve">
       <c r="A75" t="str">
-        <v>LW-40</v>
+        <v>LW-41</v>
       </c>
       <c r="B75" t="str">
-        <v>Ready made churidar</v>
+        <v>Readymade blouse</v>
       </c>
       <c r="C75" t="str">
         <v>Ladies Wear</v>
@@ -3476,19 +3476,19 @@
         <v/>
       </c>
       <c r="E75">
-        <v>75</v>
+        <v>45</v>
       </c>
       <c r="F75">
-        <v>85</v>
+        <v>45</v>
       </c>
       <c r="G75" t="str">
         <v>INSTOCK</v>
       </c>
       <c r="H75" t="str">
-        <v>size-L</v>
+        <v>free size</v>
       </c>
       <c r="I75" t="str">
-        <v>96ca04a7-3dca-467e-9673-8bc9c09cd520.jpg</v>
+        <v>c71315d5-087c-4e27-8627-641b744bc3a5.jpg</v>
       </c>
       <c r="J75" t="str">
         <v/>
@@ -3496,8 +3496,10 @@
       <c r="K75" t="str">
         <v/>
       </c>
-      <c r="L75" t="str">
-        <v/>
+      <c r="L75" t="str" xml:space="preserve">
+        <v xml:space="preserve">Free size
+Chest  margin 34-40 inch 
+Alterable</v>
       </c>
       <c r="M75" t="str">
         <v>No</v>
@@ -3505,10 +3507,10 @@
     </row>
     <row r="76" xml:space="preserve">
       <c r="A76" t="str">
-        <v>LW-41</v>
+        <v>LW-42</v>
       </c>
       <c r="B76" t="str">
-        <v>Readymade blouse</v>
+        <v>Readymade Blouse</v>
       </c>
       <c r="C76" t="str">
         <v>Ladies Wear</v>
@@ -3517,7 +3519,7 @@
         <v/>
       </c>
       <c r="E76">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="F76">
         <v>45</v>
@@ -3526,10 +3528,10 @@
         <v>INSTOCK</v>
       </c>
       <c r="H76" t="str">
-        <v>free size</v>
+        <v>Free size</v>
       </c>
       <c r="I76" t="str">
-        <v>c71315d5-087c-4e27-8627-641b744bc3a5.jpg</v>
+        <v>bef0ca17-dab0-455f-a404-d2144e3dc2a0.jpg</v>
       </c>
       <c r="J76" t="str">
         <v/>
@@ -3548,10 +3550,10 @@
     </row>
     <row r="77" xml:space="preserve">
       <c r="A77" t="str">
-        <v>LW-42</v>
+        <v>LW-43</v>
       </c>
       <c r="B77" t="str">
-        <v>Readymade Blouse</v>
+        <v>Free Size</v>
       </c>
       <c r="C77" t="str">
         <v>Ladies Wear</v>
@@ -3569,10 +3571,10 @@
         <v>INSTOCK</v>
       </c>
       <c r="H77" t="str">
-        <v>Free size</v>
+        <v>Free Size</v>
       </c>
       <c r="I77" t="str">
-        <v>bef0ca17-dab0-455f-a404-d2144e3dc2a0.jpg</v>
+        <v>e2a182ea-ccca-4e02-a77e-8512a4471618.jpg</v>
       </c>
       <c r="J77" t="str">
         <v/>
@@ -3591,10 +3593,10 @@
     </row>
     <row r="78" xml:space="preserve">
       <c r="A78" t="str">
-        <v>LW-43</v>
+        <v>LW-44</v>
       </c>
       <c r="B78" t="str">
-        <v>Free Size</v>
+        <v>Ready made blouse</v>
       </c>
       <c r="C78" t="str">
         <v>Ladies Wear</v>
@@ -3603,19 +3605,19 @@
         <v/>
       </c>
       <c r="E78">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="F78">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="G78" t="str">
         <v>INSTOCK</v>
       </c>
       <c r="H78" t="str">
-        <v>Free Size</v>
+        <v/>
       </c>
       <c r="I78" t="str">
-        <v>e2a182ea-ccca-4e02-a77e-8512a4471618.jpg</v>
+        <v>f9ec3b8b-ef32-4114-a076-22acf36d6858.jpg</v>
       </c>
       <c r="J78" t="str">
         <v/>
@@ -3634,10 +3636,10 @@
     </row>
     <row r="79" xml:space="preserve">
       <c r="A79" t="str">
-        <v>LW-44</v>
+        <v>LW-45</v>
       </c>
       <c r="B79" t="str">
-        <v>Ready made blouse</v>
+        <v>Readymade blouse</v>
       </c>
       <c r="C79" t="str">
         <v>Ladies Wear</v>
@@ -3655,10 +3657,10 @@
         <v>INSTOCK</v>
       </c>
       <c r="H79" t="str">
-        <v/>
+        <v>Free size</v>
       </c>
       <c r="I79" t="str">
-        <v>f9ec3b8b-ef32-4114-a076-22acf36d6858.jpg</v>
+        <v>33eaed97-ffa5-43b6-9e79-fe90c44b842c.jpg</v>
       </c>
       <c r="J79" t="str">
         <v/>
@@ -3677,10 +3679,10 @@
     </row>
     <row r="80" xml:space="preserve">
       <c r="A80" t="str">
-        <v>LW-45</v>
+        <v>LW-46</v>
       </c>
       <c r="B80" t="str">
-        <v>Readymade blouse</v>
+        <v>Ready made blouse</v>
       </c>
       <c r="C80" t="str">
         <v>Ladies Wear</v>
@@ -3698,10 +3700,10 @@
         <v>INSTOCK</v>
       </c>
       <c r="H80" t="str">
-        <v>Free size</v>
+        <v>Freesize</v>
       </c>
       <c r="I80" t="str">
-        <v>33eaed97-ffa5-43b6-9e79-fe90c44b842c.jpg</v>
+        <v>2705b52e-096c-4e79-b5f3-8754c6015f28.jpg</v>
       </c>
       <c r="J80" t="str">
         <v/>
@@ -3720,10 +3722,10 @@
     </row>
     <row r="81" xml:space="preserve">
       <c r="A81" t="str">
-        <v>LW-46</v>
+        <v>LW-47</v>
       </c>
       <c r="B81" t="str">
-        <v>Ready made blouse</v>
+        <v>Free size</v>
       </c>
       <c r="C81" t="str">
         <v>Ladies Wear</v>
@@ -3741,10 +3743,10 @@
         <v>INSTOCK</v>
       </c>
       <c r="H81" t="str">
-        <v>Freesize</v>
+        <v>Free size</v>
       </c>
       <c r="I81" t="str">
-        <v>2705b52e-096c-4e79-b5f3-8754c6015f28.jpg</v>
+        <v>28151555-6c9c-4a86-b3bb-5fed1c7fcbdc.jpg</v>
       </c>
       <c r="J81" t="str">
         <v/>
@@ -3761,12 +3763,12 @@
         <v>No</v>
       </c>
     </row>
-    <row r="82" xml:space="preserve">
+    <row r="82">
       <c r="A82" t="str">
-        <v>LW-47</v>
+        <v>LW-48</v>
       </c>
       <c r="B82" t="str">
-        <v>Free size</v>
+        <v>soft organza saree</v>
       </c>
       <c r="C82" t="str">
         <v>Ladies Wear</v>
@@ -3775,19 +3777,19 @@
         <v/>
       </c>
       <c r="E82">
-        <v>45</v>
+        <v>89</v>
       </c>
       <c r="F82">
-        <v>48</v>
+        <v>95</v>
       </c>
       <c r="G82" t="str">
         <v>INSTOCK</v>
       </c>
       <c r="H82" t="str">
-        <v>Free size</v>
+        <v/>
       </c>
       <c r="I82" t="str">
-        <v>28151555-6c9c-4a86-b3bb-5fed1c7fcbdc.jpg</v>
+        <v>ff4a2947-89fa-412c-91d7-6ebe043c24f9.jpg</v>
       </c>
       <c r="J82" t="str">
         <v/>
@@ -3795,10 +3797,8 @@
       <c r="K82" t="str">
         <v/>
       </c>
-      <c r="L82" t="str" xml:space="preserve">
-        <v xml:space="preserve">Free size
-Chest  margin 34-40 inch 
-Alterable</v>
+      <c r="L82" t="str">
+        <v>unstitched blouse</v>
       </c>
       <c r="M82" t="str">
         <v>No</v>
@@ -3806,10 +3806,10 @@
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>LW-48</v>
+        <v>LW-49</v>
       </c>
       <c r="B83" t="str">
-        <v>soft organza saree</v>
+        <v>semi tusser silk</v>
       </c>
       <c r="C83" t="str">
         <v>Ladies Wear</v>
@@ -3818,10 +3818,10 @@
         <v/>
       </c>
       <c r="E83">
-        <v>89</v>
+        <v>76</v>
       </c>
       <c r="F83">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="G83" t="str">
         <v>INSTOCK</v>
@@ -3830,7 +3830,7 @@
         <v/>
       </c>
       <c r="I83" t="str">
-        <v>ff4a2947-89fa-412c-91d7-6ebe043c24f9.jpg</v>
+        <v>cf1b0bea-3bba-4185-936d-e21a7b9cb63e.jpg</v>
       </c>
       <c r="J83" t="str">
         <v/>
@@ -3839,7 +3839,7 @@
         <v/>
       </c>
       <c r="L83" t="str">
-        <v>unstitched blouse</v>
+        <v/>
       </c>
       <c r="M83" t="str">
         <v>No</v>
@@ -3847,10 +3847,10 @@
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>LW-49</v>
+        <v>LW-50</v>
       </c>
       <c r="B84" t="str">
-        <v>semi tusser silk</v>
+        <v>semi tusser saree</v>
       </c>
       <c r="C84" t="str">
         <v>Ladies Wear</v>
@@ -3871,7 +3871,7 @@
         <v/>
       </c>
       <c r="I84" t="str">
-        <v>cf1b0bea-3bba-4185-936d-e21a7b9cb63e.jpg</v>
+        <v>057421ca-10bb-4a81-9f23-570e65d9dd5d.jpg</v>
       </c>
       <c r="J84" t="str">
         <v/>
@@ -3888,10 +3888,10 @@
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>LW-50</v>
+        <v>LW-51</v>
       </c>
       <c r="B85" t="str">
-        <v>semi tusser saree</v>
+        <v>Semi tusser silk sarees</v>
       </c>
       <c r="C85" t="str">
         <v>Ladies Wear</v>
@@ -3900,10 +3900,10 @@
         <v/>
       </c>
       <c r="E85">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="F85">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="G85" t="str">
         <v>INSTOCK</v>
@@ -3912,7 +3912,7 @@
         <v/>
       </c>
       <c r="I85" t="str">
-        <v>057421ca-10bb-4a81-9f23-570e65d9dd5d.jpg</v>
+        <v>e5a4ba5d-7dfd-4106-830e-6f1527c6a7fc.jpg</v>
       </c>
       <c r="J85" t="str">
         <v/>
@@ -3929,10 +3929,10 @@
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>LW-51</v>
+        <v>LW-52</v>
       </c>
       <c r="B86" t="str">
-        <v>Semi tusser silk sarees</v>
+        <v>linen based saree</v>
       </c>
       <c r="C86" t="str">
         <v>Ladies Wear</v>
@@ -3941,10 +3941,10 @@
         <v/>
       </c>
       <c r="E86">
-        <v>83</v>
+        <v>69</v>
       </c>
       <c r="F86">
-        <v>90</v>
+        <v>75</v>
       </c>
       <c r="G86" t="str">
         <v>INSTOCK</v>
@@ -3953,7 +3953,7 @@
         <v/>
       </c>
       <c r="I86" t="str">
-        <v>e5a4ba5d-7dfd-4106-830e-6f1527c6a7fc.jpg</v>
+        <v>f74b6f56-6e30-4e27-ba40-0a4dc6f9b60d.jpg</v>
       </c>
       <c r="J86" t="str">
         <v/>
@@ -3965,12 +3965,1340 @@
         <v/>
       </c>
       <c r="M86" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="str">
+        <v>LW-53</v>
+      </c>
+      <c r="B87" t="str">
+        <v>saree</v>
+      </c>
+      <c r="C87" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D87" t="str">
+        <v/>
+      </c>
+      <c r="E87">
+        <v>75</v>
+      </c>
+      <c r="F87">
+        <v>80</v>
+      </c>
+      <c r="G87" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H87" t="str">
+        <v/>
+      </c>
+      <c r="I87" t="str">
+        <v>9ecbfa41-903e-4684-968b-1c5b91aae95c.jpg</v>
+      </c>
+      <c r="J87" t="str">
+        <v/>
+      </c>
+      <c r="K87" t="str">
+        <v/>
+      </c>
+      <c r="L87" t="str">
+        <v/>
+      </c>
+      <c r="M87" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="str">
+        <v>LW-54</v>
+      </c>
+      <c r="B88" t="str">
+        <v>Premium semi silk</v>
+      </c>
+      <c r="C88" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D88" t="str">
+        <v/>
+      </c>
+      <c r="E88">
+        <v>76</v>
+      </c>
+      <c r="F88">
+        <v>85</v>
+      </c>
+      <c r="G88" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H88" t="str">
+        <v>LARGE</v>
+      </c>
+      <c r="I88" t="str">
+        <v>89d9133d-adf4-4bc7-a9db-0fc8aa5517ee.jpg</v>
+      </c>
+      <c r="J88" t="str">
+        <v/>
+      </c>
+      <c r="K88" t="str">
+        <v/>
+      </c>
+      <c r="L88" t="str">
+        <v/>
+      </c>
+      <c r="M88" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="str">
+        <v>LW-55</v>
+      </c>
+      <c r="B89" t="str">
+        <v>PARTYWEAR</v>
+      </c>
+      <c r="C89" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D89" t="str">
+        <v/>
+      </c>
+      <c r="E89">
+        <v>94</v>
+      </c>
+      <c r="F89">
+        <v>100</v>
+      </c>
+      <c r="G89" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H89" t="str">
+        <v/>
+      </c>
+      <c r="I89" t="str">
+        <v>4c266a33-1972-4650-b3e7-313ba683168f.jpg</v>
+      </c>
+      <c r="J89" t="str">
+        <v/>
+      </c>
+      <c r="K89" t="str">
+        <v/>
+      </c>
+      <c r="L89" t="str">
+        <v/>
+      </c>
+      <c r="M89" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="str">
+        <v>LW-56</v>
+      </c>
+      <c r="B90" t="str">
+        <v>SEMITUSSER  SILK SAREE</v>
+      </c>
+      <c r="C90" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D90" t="str">
+        <v/>
+      </c>
+      <c r="E90">
+        <v>69</v>
+      </c>
+      <c r="F90">
+        <v>77</v>
+      </c>
+      <c r="G90" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H90" t="str">
+        <v/>
+      </c>
+      <c r="I90" t="str">
+        <v>60291a21-73c9-410a-93ac-23d5f8729998.jpg</v>
+      </c>
+      <c r="J90" t="str">
+        <v/>
+      </c>
+      <c r="K90" t="str">
+        <v/>
+      </c>
+      <c r="L90" t="str">
+        <v/>
+      </c>
+      <c r="M90" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="str">
+        <v>LW-57</v>
+      </c>
+      <c r="B91" t="str">
+        <v>PARTYWEAR SATIN SILK  SAREE</v>
+      </c>
+      <c r="C91" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D91" t="str">
+        <v/>
+      </c>
+      <c r="E91">
+        <v>99</v>
+      </c>
+      <c r="F91">
+        <v>110</v>
+      </c>
+      <c r="G91" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H91" t="str">
+        <v/>
+      </c>
+      <c r="I91" t="str">
+        <v>c191dd1d-dbfb-4ff0-b762-12e511577010.jpg</v>
+      </c>
+      <c r="J91" t="str">
+        <v/>
+      </c>
+      <c r="K91" t="str">
+        <v/>
+      </c>
+      <c r="L91" t="str">
+        <v>SATIN SILK   SEQUENCE SAREE</v>
+      </c>
+      <c r="M91" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="str">
+        <v>LW-58</v>
+      </c>
+      <c r="B92" t="str">
+        <v>Satin silk sequence saree</v>
+      </c>
+      <c r="C92" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D92" t="str">
+        <v/>
+      </c>
+      <c r="E92">
+        <v>99</v>
+      </c>
+      <c r="F92">
+        <v>110</v>
+      </c>
+      <c r="G92" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H92" t="str">
+        <v/>
+      </c>
+      <c r="I92" t="str">
+        <v>ec788d2b-6b6c-4be7-bd78-9caa1d2ab367.jpg</v>
+      </c>
+      <c r="J92" t="str">
+        <v/>
+      </c>
+      <c r="K92" t="str">
+        <v/>
+      </c>
+      <c r="L92" t="str">
+        <v>part wear Satin silk sequence saree</v>
+      </c>
+      <c r="M92" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="str">
+        <v>LW-59</v>
+      </c>
+      <c r="B93" t="str">
+        <v>Kids pattupavada</v>
+      </c>
+      <c r="C93" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D93" t="str">
+        <v/>
+      </c>
+      <c r="E93">
+        <v>50</v>
+      </c>
+      <c r="F93">
+        <v>58</v>
+      </c>
+      <c r="G93" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H93" t="str">
+        <v>6 YRS</v>
+      </c>
+      <c r="I93" t="str">
+        <v>bb662809-52a8-4a12-9e07-8d048b352c32.jpg</v>
+      </c>
+      <c r="J93" t="str">
+        <v/>
+      </c>
+      <c r="K93" t="str">
+        <v/>
+      </c>
+      <c r="L93" t="str">
+        <v>Kids silk lehenga</v>
+      </c>
+      <c r="M93" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="94" xml:space="preserve">
+      <c r="A94" t="str">
+        <v>LW-60</v>
+      </c>
+      <c r="B94" t="str">
+        <v>Premium readymade blouse</v>
+      </c>
+      <c r="C94" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D94" t="str">
+        <v/>
+      </c>
+      <c r="E94">
+        <v>48</v>
+      </c>
+      <c r="F94">
+        <v>55</v>
+      </c>
+      <c r="G94" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H94" t="str">
+        <v/>
+      </c>
+      <c r="I94" t="str">
+        <v>2ec0f1d4-933e-4861-ba67-ad0b6c2a25ba.jpg</v>
+      </c>
+      <c r="J94" t="str">
+        <v>17a2bc44-8920-4b25-ba8c-5e211eaabb4b.jpg</v>
+      </c>
+      <c r="K94" t="str">
+        <v>bb43e807-2f3d-43bf-a511-033a965a1dd7.jpg</v>
+      </c>
+      <c r="L94" t="str" xml:space="preserve">
+        <v xml:space="preserve">pure cotton printed work.
+Available shades - off-white, green, red and navy-blue
+Alterable- size margin 34-40</v>
+      </c>
+      <c r="M94" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="str">
+        <v>KW-12</v>
+      </c>
+      <c r="B95" t="str">
+        <v>Kids Lehenga</v>
+      </c>
+      <c r="C95" t="str">
+        <v>Kids Wear</v>
+      </c>
+      <c r="D95" t="str">
+        <v/>
+      </c>
+      <c r="E95">
+        <v>54</v>
+      </c>
+      <c r="F95">
+        <v>60</v>
+      </c>
+      <c r="G95" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H95" t="str">
+        <v>6 yr old</v>
+      </c>
+      <c r="I95" t="str">
+        <v>28ca42df-1516-4953-8280-da91035e7a66.jpg</v>
+      </c>
+      <c r="J95" t="str">
+        <v/>
+      </c>
+      <c r="K95" t="str">
+        <v/>
+      </c>
+      <c r="L95" t="str">
+        <v/>
+      </c>
+      <c r="M95" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="str">
+        <v>KW-13</v>
+      </c>
+      <c r="B96" t="str">
+        <v>kids lehenga</v>
+      </c>
+      <c r="C96" t="str">
+        <v>Kids Wear</v>
+      </c>
+      <c r="D96" t="str">
+        <v/>
+      </c>
+      <c r="E96">
+        <v>60</v>
+      </c>
+      <c r="F96">
+        <v>65</v>
+      </c>
+      <c r="G96" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H96" t="str">
+        <v>9 yrs old</v>
+      </c>
+      <c r="I96" t="str">
+        <v>9172a631-d694-4bbf-8e69-7d0eaf1a5062.jpg</v>
+      </c>
+      <c r="J96" t="str">
+        <v/>
+      </c>
+      <c r="K96" t="str">
+        <v/>
+      </c>
+      <c r="L96" t="str">
+        <v>colour - red</v>
+      </c>
+      <c r="M96" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="str">
+        <v>KW-14</v>
+      </c>
+      <c r="B97" t="str">
+        <v>Kids Lehenga</v>
+      </c>
+      <c r="C97" t="str">
+        <v>Kids Wear</v>
+      </c>
+      <c r="D97" t="str">
+        <v/>
+      </c>
+      <c r="E97">
+        <v>59</v>
+      </c>
+      <c r="F97">
+        <v>68</v>
+      </c>
+      <c r="G97" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H97" t="str">
+        <v>Age 10yrs</v>
+      </c>
+      <c r="I97" t="str">
+        <v>2fc67c86-c27e-4046-a1d9-14feb84e4abc.jpg</v>
+      </c>
+      <c r="J97" t="str">
+        <v/>
+      </c>
+      <c r="K97" t="str">
+        <v/>
+      </c>
+      <c r="L97" t="str">
+        <v/>
+      </c>
+      <c r="M97" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="str">
+        <v>LW-61</v>
+      </c>
+      <c r="B98" t="str">
+        <v>party wear saree</v>
+      </c>
+      <c r="C98" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D98" t="str">
+        <v/>
+      </c>
+      <c r="E98">
+        <v>89</v>
+      </c>
+      <c r="F98">
+        <v>99</v>
+      </c>
+      <c r="G98" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H98" t="str">
+        <v/>
+      </c>
+      <c r="I98" t="str">
+        <v>c1730041-3c0d-42ca-b0ae-1773c953d691.jpg</v>
+      </c>
+      <c r="J98" t="str">
+        <v/>
+      </c>
+      <c r="K98" t="str">
+        <v/>
+      </c>
+      <c r="L98" t="str">
+        <v>colour- Pari Grey</v>
+      </c>
+      <c r="M98" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="99" xml:space="preserve">
+      <c r="A99" t="str">
+        <v>LW-62</v>
+      </c>
+      <c r="B99" t="str">
+        <v>Readymade blouse</v>
+      </c>
+      <c r="C99" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D99" t="str">
+        <v/>
+      </c>
+      <c r="E99">
+        <v>45</v>
+      </c>
+      <c r="F99">
+        <v>50</v>
+      </c>
+      <c r="G99" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H99" t="str">
+        <v>BLOUSE -FREE SIZE</v>
+      </c>
+      <c r="I99" t="str">
+        <v>470d93c8-3d0e-46ac-b5e5-8262f1f8e237.jpg</v>
+      </c>
+      <c r="J99" t="str">
+        <v/>
+      </c>
+      <c r="K99" t="str">
+        <v/>
+      </c>
+      <c r="L99" t="str" xml:space="preserve">
+        <v xml:space="preserve">Alterable- chest margin 34-40 
+Viscose sequence embroidery blouse</v>
+      </c>
+      <c r="M99" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="100" xml:space="preserve">
+      <c r="A100" t="str">
+        <v>LW-63</v>
+      </c>
+      <c r="B100" t="str">
+        <v>Readymade blouse</v>
+      </c>
+      <c r="C100" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D100" t="str">
+        <v/>
+      </c>
+      <c r="E100">
+        <v>45</v>
+      </c>
+      <c r="F100">
+        <v>50</v>
+      </c>
+      <c r="G100" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H100" t="str">
+        <v/>
+      </c>
+      <c r="I100" t="str">
+        <v>4150b78e-1197-4f71-b6d7-4c665e69b386.jpg</v>
+      </c>
+      <c r="J100" t="str">
+        <v/>
+      </c>
+      <c r="K100" t="str">
+        <v/>
+      </c>
+      <c r="L100" t="str" xml:space="preserve">
+        <v xml:space="preserve">Alterable .
+Chest margin 34 to 40</v>
+      </c>
+      <c r="M100" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="101" xml:space="preserve">
+      <c r="A101" t="str">
+        <v>LW-64</v>
+      </c>
+      <c r="B101" t="str">
+        <v>Readymade blouse</v>
+      </c>
+      <c r="C101" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D101" t="str">
+        <v/>
+      </c>
+      <c r="E101">
+        <v>45</v>
+      </c>
+      <c r="F101">
+        <v>50</v>
+      </c>
+      <c r="G101" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H101" t="str">
+        <v/>
+      </c>
+      <c r="I101" t="str">
+        <v>fb81a1fc-af60-4fbc-907f-a286a7c33273.jpg</v>
+      </c>
+      <c r="J101" t="str">
+        <v/>
+      </c>
+      <c r="K101" t="str">
+        <v/>
+      </c>
+      <c r="L101" t="str" xml:space="preserve">
+        <v xml:space="preserve">Alterable .
+Chest margin 34 to 40</v>
+      </c>
+      <c r="M101" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="102" xml:space="preserve">
+      <c r="A102" t="str">
+        <v>LW-65</v>
+      </c>
+      <c r="B102" t="str">
+        <v>Readymadeblouse</v>
+      </c>
+      <c r="C102" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D102" t="str">
+        <v/>
+      </c>
+      <c r="E102">
+        <v>45</v>
+      </c>
+      <c r="F102">
+        <v>50</v>
+      </c>
+      <c r="G102" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H102" t="str">
+        <v/>
+      </c>
+      <c r="I102" t="str">
+        <v>2e19fe60-606c-4653-ac35-2e47405feab5.jpg</v>
+      </c>
+      <c r="J102" t="str">
+        <v/>
+      </c>
+      <c r="K102" t="str">
+        <v/>
+      </c>
+      <c r="L102" t="str" xml:space="preserve">
+        <v xml:space="preserve">Alterable .
+Chest margin 34 to 40</v>
+      </c>
+      <c r="M102" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="103" xml:space="preserve">
+      <c r="A103" t="str">
+        <v>LW-66</v>
+      </c>
+      <c r="B103" t="str">
+        <v>Readymade blouse</v>
+      </c>
+      <c r="C103" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D103" t="str">
+        <v/>
+      </c>
+      <c r="E103">
+        <v>45</v>
+      </c>
+      <c r="F103">
+        <v>52</v>
+      </c>
+      <c r="G103" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H103" t="str">
+        <v>Free size</v>
+      </c>
+      <c r="I103" t="str">
+        <v>afe93890-96e4-4a55-b8cc-b9e8f004c0fb.jpg</v>
+      </c>
+      <c r="J103" t="str">
+        <v/>
+      </c>
+      <c r="K103" t="str">
+        <v/>
+      </c>
+      <c r="L103" t="str" xml:space="preserve">
+        <v xml:space="preserve">Alterable .
+Chest margin 34 to 40</v>
+      </c>
+      <c r="M103" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="104" xml:space="preserve">
+      <c r="A104" t="str">
+        <v>LW-67</v>
+      </c>
+      <c r="B104" t="str">
+        <v>readymade blouse</v>
+      </c>
+      <c r="C104" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D104" t="str">
+        <v/>
+      </c>
+      <c r="E104">
+        <v>45</v>
+      </c>
+      <c r="F104">
+        <v>52</v>
+      </c>
+      <c r="G104" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H104" t="str">
+        <v/>
+      </c>
+      <c r="I104" t="str">
+        <v>8ce65bcf-affd-4fd5-8fd4-5147882e7712.jpg</v>
+      </c>
+      <c r="J104" t="str">
+        <v/>
+      </c>
+      <c r="K104" t="str">
+        <v/>
+      </c>
+      <c r="L104" t="str" xml:space="preserve">
+        <v xml:space="preserve">Alterable .
+Chest margin 34 to 40</v>
+      </c>
+      <c r="M104" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="105" xml:space="preserve">
+      <c r="A105" t="str">
+        <v>LW-68</v>
+      </c>
+      <c r="B105" t="str">
+        <v>Readymade blouse</v>
+      </c>
+      <c r="C105" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D105" t="str">
+        <v/>
+      </c>
+      <c r="E105">
+        <v>45</v>
+      </c>
+      <c r="F105">
+        <v>52</v>
+      </c>
+      <c r="G105" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H105" t="str">
+        <v/>
+      </c>
+      <c r="I105" t="str">
+        <v>f4ea5f8f-206d-4b9f-b44b-e59b11c9fc86.jpg</v>
+      </c>
+      <c r="J105" t="str">
+        <v/>
+      </c>
+      <c r="K105" t="str">
+        <v/>
+      </c>
+      <c r="L105" t="str" xml:space="preserve">
+        <v xml:space="preserve">Alterable .
+Chest margin 34 to 40</v>
+      </c>
+      <c r="M105" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="106" xml:space="preserve">
+      <c r="A106" t="str">
+        <v>LW-69</v>
+      </c>
+      <c r="B106" t="str">
+        <v>Readymade Blouse</v>
+      </c>
+      <c r="C106" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D106" t="str">
+        <v/>
+      </c>
+      <c r="E106">
+        <v>45</v>
+      </c>
+      <c r="F106">
+        <v>52</v>
+      </c>
+      <c r="G106" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H106" t="str">
+        <v/>
+      </c>
+      <c r="I106" t="str">
+        <v>74a37c06-c1ec-4c59-a0ba-056a68be512f.jpg</v>
+      </c>
+      <c r="J106" t="str">
+        <v/>
+      </c>
+      <c r="K106" t="str">
+        <v/>
+      </c>
+      <c r="L106" t="str" xml:space="preserve">
+        <v xml:space="preserve">Alterable .
+Chest margin 34 to 40</v>
+      </c>
+      <c r="M106" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="107" xml:space="preserve">
+      <c r="A107" t="str">
+        <v>LW-70</v>
+      </c>
+      <c r="B107" t="str">
+        <v>Readymade blouse</v>
+      </c>
+      <c r="C107" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D107" t="str">
+        <v/>
+      </c>
+      <c r="E107">
+        <v>45</v>
+      </c>
+      <c r="F107">
+        <v>55</v>
+      </c>
+      <c r="G107" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H107" t="str">
+        <v/>
+      </c>
+      <c r="I107" t="str">
+        <v>780a515d-4ed1-4e4f-95ea-ab974f2b9287.jpg</v>
+      </c>
+      <c r="J107" t="str">
+        <v/>
+      </c>
+      <c r="K107" t="str">
+        <v/>
+      </c>
+      <c r="L107" t="str" xml:space="preserve">
+        <v xml:space="preserve">Alterable .
+Chest margin 34 to 40</v>
+      </c>
+      <c r="M107" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="108" xml:space="preserve">
+      <c r="A108" t="str">
+        <v>LW-71</v>
+      </c>
+      <c r="B108" t="str">
+        <v>Readymade blouse</v>
+      </c>
+      <c r="C108" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D108" t="str">
+        <v/>
+      </c>
+      <c r="E108">
+        <v>45</v>
+      </c>
+      <c r="F108">
+        <v>55</v>
+      </c>
+      <c r="G108" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H108" t="str">
+        <v/>
+      </c>
+      <c r="I108" t="str">
+        <v>e67cac17-6a46-4492-b87e-a93067dbdcfa.jpg</v>
+      </c>
+      <c r="J108" t="str">
+        <v>ce57593d-776f-4525-9e9a-8d852bce2df7.jpg</v>
+      </c>
+      <c r="K108" t="str">
+        <v>b6f5ef18-6ad8-402a-be8d-2f3f263577fb.jpg</v>
+      </c>
+      <c r="L108" t="str" xml:space="preserve">
+        <v xml:space="preserve">Alterable .
+Chest margin 34 to 40
+Sleeve available , needs to be attached</v>
+      </c>
+      <c r="M108" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="109" xml:space="preserve">
+      <c r="A109" t="str">
+        <v>LW-72</v>
+      </c>
+      <c r="B109" t="str">
+        <v>Premium  partywear  readymade blouse</v>
+      </c>
+      <c r="C109" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D109" t="str">
+        <v/>
+      </c>
+      <c r="E109">
+        <v>56</v>
+      </c>
+      <c r="F109">
+        <v>65</v>
+      </c>
+      <c r="G109" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H109" t="str">
+        <v/>
+      </c>
+      <c r="I109" t="str">
+        <v>fcb23416-b8c6-4f32-864d-102539548426.jpg</v>
+      </c>
+      <c r="J109" t="str">
+        <v/>
+      </c>
+      <c r="K109" t="str">
+        <v/>
+      </c>
+      <c r="L109" t="str" xml:space="preserve">
+        <v xml:space="preserve">Alterable .
+Chest margin 34 to 40</v>
+      </c>
+      <c r="M109" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="110" xml:space="preserve">
+      <c r="A110" t="str">
+        <v>LW-73</v>
+      </c>
+      <c r="B110" t="str">
+        <v>Premium  worked readymade blouse</v>
+      </c>
+      <c r="C110" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D110" t="str">
+        <v/>
+      </c>
+      <c r="E110">
+        <v>56</v>
+      </c>
+      <c r="F110">
+        <v>69</v>
+      </c>
+      <c r="G110" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H110" t="str">
+        <v/>
+      </c>
+      <c r="I110" t="str">
+        <v>2b0d0c08-bbb5-4843-a026-7ab66ac4bbea.jpg</v>
+      </c>
+      <c r="J110" t="str">
+        <v/>
+      </c>
+      <c r="K110" t="str">
+        <v/>
+      </c>
+      <c r="L110" t="str" xml:space="preserve">
+        <v xml:space="preserve">Alterable .
+Chest margin 34 to 40</v>
+      </c>
+      <c r="M110" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="str">
+        <v>LW-74</v>
+      </c>
+      <c r="B111" t="str">
+        <v>Partywear heavy work readymade blouse</v>
+      </c>
+      <c r="C111" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D111" t="str">
+        <v/>
+      </c>
+      <c r="E111">
+        <v>56</v>
+      </c>
+      <c r="F111">
+        <v>69</v>
+      </c>
+      <c r="G111" t="str">
+        <v>SOLD OUT</v>
+      </c>
+      <c r="H111" t="str">
+        <v/>
+      </c>
+      <c r="I111" t="str">
+        <v>0122d0f2-1240-4939-9984-f1b3d6db3ae4.jpg</v>
+      </c>
+      <c r="J111" t="str">
+        <v/>
+      </c>
+      <c r="K111" t="str">
+        <v/>
+      </c>
+      <c r="L111" t="str">
+        <v/>
+      </c>
+      <c r="M111" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="112" xml:space="preserve">
+      <c r="A112" t="str">
+        <v>LW-75</v>
+      </c>
+      <c r="B112" t="str">
+        <v>Premium  readymade partywear blouse</v>
+      </c>
+      <c r="C112" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D112" t="str">
+        <v/>
+      </c>
+      <c r="E112">
+        <v>56</v>
+      </c>
+      <c r="F112">
+        <v>69</v>
+      </c>
+      <c r="G112" t="str">
+        <v>SOLD OUT</v>
+      </c>
+      <c r="H112" t="str">
+        <v/>
+      </c>
+      <c r="I112" t="str">
+        <v>95c79c68-6a79-4aab-921e-facedb177d50.jpg</v>
+      </c>
+      <c r="J112" t="str">
+        <v/>
+      </c>
+      <c r="K112" t="str">
+        <v/>
+      </c>
+      <c r="L112" t="str" xml:space="preserve">
+        <v xml:space="preserve">Alterable .
+Chest margin 34 to 40</v>
+      </c>
+      <c r="M112" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="str">
+        <v>LW-76</v>
+      </c>
+      <c r="B113" t="str">
+        <v>Tussar silk</v>
+      </c>
+      <c r="C113" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D113" t="str">
+        <v/>
+      </c>
+      <c r="E113">
+        <v>99</v>
+      </c>
+      <c r="F113">
+        <v>115</v>
+      </c>
+      <c r="G113" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H113" t="str">
+        <v/>
+      </c>
+      <c r="I113" t="str">
+        <v>7f00bd84-0930-4bdd-9c6d-7738f011ba75.jpg</v>
+      </c>
+      <c r="J113" t="str">
+        <v/>
+      </c>
+      <c r="K113" t="str">
+        <v/>
+      </c>
+      <c r="L113" t="str">
+        <v/>
+      </c>
+      <c r="M113" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="str">
+        <v>LW-77</v>
+      </c>
+      <c r="B114" t="str">
+        <v>Fendy Satin Silk sarees</v>
+      </c>
+      <c r="C114" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D114" t="str">
+        <v/>
+      </c>
+      <c r="E114">
+        <v>100</v>
+      </c>
+      <c r="F114">
+        <v>120</v>
+      </c>
+      <c r="G114" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H114" t="str">
+        <v/>
+      </c>
+      <c r="I114" t="str">
+        <v>214314d6-19d9-4831-9e57-8fca960820d1.jpg</v>
+      </c>
+      <c r="J114" t="str">
+        <v/>
+      </c>
+      <c r="K114" t="str">
+        <v/>
+      </c>
+      <c r="L114" t="str">
+        <v>exclusive collection.</v>
+      </c>
+      <c r="M114" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="str">
+        <v>LW-78</v>
+      </c>
+      <c r="B115" t="str">
+        <v>Chiffon silk party wear sarees</v>
+      </c>
+      <c r="C115" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D115" t="str">
+        <v/>
+      </c>
+      <c r="E115">
+        <v>79</v>
+      </c>
+      <c r="F115">
+        <v>95</v>
+      </c>
+      <c r="G115" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H115" t="str">
+        <v/>
+      </c>
+      <c r="I115" t="str">
+        <v>8c1fce62-0328-44cc-9643-86d00bb5891b.jpg</v>
+      </c>
+      <c r="J115" t="str">
+        <v/>
+      </c>
+      <c r="K115" t="str">
+        <v/>
+      </c>
+      <c r="L115" t="str">
+        <v/>
+      </c>
+      <c r="M115" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="str">
+        <v>LW-79</v>
+      </c>
+      <c r="B116" t="str">
+        <v>Space silk designer sarees</v>
+      </c>
+      <c r="C116" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D116" t="str">
+        <v/>
+      </c>
+      <c r="E116">
+        <v>62</v>
+      </c>
+      <c r="F116">
+        <v>70</v>
+      </c>
+      <c r="G116" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H116" t="str">
+        <v/>
+      </c>
+      <c r="I116" t="str">
+        <v>26fc8ba6-aea9-4d18-8e50-6857ef12a25f.jpg</v>
+      </c>
+      <c r="J116" t="str">
+        <v/>
+      </c>
+      <c r="K116" t="str">
+        <v/>
+      </c>
+      <c r="L116" t="str">
+        <v/>
+      </c>
+      <c r="M116" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="str">
+        <v>LW-80</v>
+      </c>
+      <c r="B117" t="str">
+        <v>Tissue silk ready to wear saree</v>
+      </c>
+      <c r="C117" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D117" t="str">
+        <v/>
+      </c>
+      <c r="E117">
+        <v>75</v>
+      </c>
+      <c r="F117">
+        <v>89</v>
+      </c>
+      <c r="G117" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H117" t="str">
+        <v/>
+      </c>
+      <c r="I117" t="str">
+        <v>9fa4bc2a-269f-4da6-9065-e9d83b63f4cd.jpg</v>
+      </c>
+      <c r="J117" t="str">
+        <v/>
+      </c>
+      <c r="K117" t="str">
+        <v/>
+      </c>
+      <c r="L117" t="str">
+        <v/>
+      </c>
+      <c r="M117" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="str">
+        <v>LW-81</v>
+      </c>
+      <c r="B118" t="str">
+        <v>Silk Cotton kids ethnic wear</v>
+      </c>
+      <c r="C118" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D118" t="str">
+        <v/>
+      </c>
+      <c r="E118">
+        <v>49</v>
+      </c>
+      <c r="F118">
+        <v>55</v>
+      </c>
+      <c r="G118" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H118" t="str">
+        <v/>
+      </c>
+      <c r="I118" t="str">
+        <v>41df6b6b-0af9-4dac-8417-816a8605224c.jpg</v>
+      </c>
+      <c r="J118" t="str">
+        <v/>
+      </c>
+      <c r="K118" t="str">
+        <v/>
+      </c>
+      <c r="L118" t="str">
+        <v>size -6 yr old</v>
+      </c>
+      <c r="M118" t="str">
         <v>No</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M86"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M118"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update store products via Admin Panel - 09/08/2026, 1:32:55 am
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M118"/>
+  <dimension ref="A1:M128"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -5296,9 +5296,419 @@
         <v>No</v>
       </c>
     </row>
+    <row r="119">
+      <c r="A119" t="str">
+        <v>KW-15</v>
+      </c>
+      <c r="B119" t="str">
+        <v>Premium  kids lehenga set</v>
+      </c>
+      <c r="C119" t="str">
+        <v>Kids Wear</v>
+      </c>
+      <c r="D119" t="str">
+        <v/>
+      </c>
+      <c r="E119">
+        <v>58</v>
+      </c>
+      <c r="F119">
+        <v>69</v>
+      </c>
+      <c r="G119" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H119" t="str">
+        <v/>
+      </c>
+      <c r="I119" t="str">
+        <v>7896c9fb-858b-4a24-b283-363135102ca6.jpg</v>
+      </c>
+      <c r="J119" t="str">
+        <v/>
+      </c>
+      <c r="K119" t="str">
+        <v/>
+      </c>
+      <c r="L119" t="str">
+        <v>age -6 yrs</v>
+      </c>
+      <c r="M119" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="str">
+        <v>KW-16</v>
+      </c>
+      <c r="B120" t="str">
+        <v>premium kids lehenga set</v>
+      </c>
+      <c r="C120" t="str">
+        <v>Kids Wear</v>
+      </c>
+      <c r="D120" t="str">
+        <v/>
+      </c>
+      <c r="E120">
+        <v>59</v>
+      </c>
+      <c r="F120">
+        <v>68</v>
+      </c>
+      <c r="G120" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H120" t="str">
+        <v/>
+      </c>
+      <c r="I120" t="str">
+        <v>placeholder.svg</v>
+      </c>
+      <c r="J120" t="str">
+        <v/>
+      </c>
+      <c r="K120" t="str">
+        <v/>
+      </c>
+      <c r="L120" t="str">
+        <v>Age -6 yrs and 8 yrs</v>
+      </c>
+      <c r="M120" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="str">
+        <v>LW-82</v>
+      </c>
+      <c r="B121" t="str">
+        <v>linen cotton</v>
+      </c>
+      <c r="C121" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D121" t="str">
+        <v/>
+      </c>
+      <c r="E121">
+        <v>63</v>
+      </c>
+      <c r="F121">
+        <v>70</v>
+      </c>
+      <c r="G121" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H121" t="str">
+        <v/>
+      </c>
+      <c r="I121" t="str">
+        <v>4487a279-99dc-4959-811f-57cd488b7abc.jpg</v>
+      </c>
+      <c r="J121" t="str">
+        <v/>
+      </c>
+      <c r="K121" t="str">
+        <v/>
+      </c>
+      <c r="L121" t="str">
+        <v/>
+      </c>
+      <c r="M121" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="str">
+        <v>LW-83</v>
+      </c>
+      <c r="B122" t="str">
+        <v>sarees</v>
+      </c>
+      <c r="C122" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D122" t="str">
+        <v/>
+      </c>
+      <c r="E122">
+        <v>54</v>
+      </c>
+      <c r="F122">
+        <v>65</v>
+      </c>
+      <c r="G122" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H122" t="str">
+        <v/>
+      </c>
+      <c r="I122" t="str">
+        <v>f697d427-c6b5-401e-bedc-f2b044a25d48.jpg</v>
+      </c>
+      <c r="J122" t="str">
+        <v/>
+      </c>
+      <c r="K122" t="str">
+        <v/>
+      </c>
+      <c r="L122" t="str">
+        <v/>
+      </c>
+      <c r="M122" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="str">
+        <v>LW-84</v>
+      </c>
+      <c r="B123" t="str">
+        <v>saree</v>
+      </c>
+      <c r="C123" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D123" t="str">
+        <v/>
+      </c>
+      <c r="E123">
+        <v>63</v>
+      </c>
+      <c r="F123">
+        <v>69</v>
+      </c>
+      <c r="G123" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H123" t="str">
+        <v/>
+      </c>
+      <c r="I123" t="str">
+        <v>ddc4c3dd-e1da-4a44-b003-c856bf973420.jpg</v>
+      </c>
+      <c r="J123" t="str">
+        <v/>
+      </c>
+      <c r="K123" t="str">
+        <v/>
+      </c>
+      <c r="L123" t="str">
+        <v/>
+      </c>
+      <c r="M123" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="str">
+        <v>LW-85</v>
+      </c>
+      <c r="B124" t="str">
+        <v>Soft dola kanjeevaram</v>
+      </c>
+      <c r="C124" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D124" t="str">
+        <v/>
+      </c>
+      <c r="E124">
+        <v>64</v>
+      </c>
+      <c r="F124">
+        <v>69</v>
+      </c>
+      <c r="G124" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H124" t="str">
+        <v/>
+      </c>
+      <c r="I124" t="str">
+        <v>ade2d2de-030b-4f8a-afeb-845911044361.jpg</v>
+      </c>
+      <c r="J124" t="str">
+        <v/>
+      </c>
+      <c r="K124" t="str">
+        <v/>
+      </c>
+      <c r="L124" t="str">
+        <v/>
+      </c>
+      <c r="M124" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="str">
+        <v>LW-86</v>
+      </c>
+      <c r="B125" t="str">
+        <v>Fendy double shaded saree</v>
+      </c>
+      <c r="C125" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D125" t="str">
+        <v/>
+      </c>
+      <c r="E125">
+        <v>83</v>
+      </c>
+      <c r="F125">
+        <v>99</v>
+      </c>
+      <c r="G125" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H125" t="str">
+        <v/>
+      </c>
+      <c r="I125" t="str">
+        <v>228360f5-e427-4219-a2db-77f125dc8791.jpg</v>
+      </c>
+      <c r="J125" t="str">
+        <v/>
+      </c>
+      <c r="K125" t="str">
+        <v/>
+      </c>
+      <c r="L125" t="str">
+        <v/>
+      </c>
+      <c r="M125" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="str">
+        <v>LW-87</v>
+      </c>
+      <c r="B126" t="str">
+        <v>soft dola silk</v>
+      </c>
+      <c r="C126" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D126" t="str">
+        <v/>
+      </c>
+      <c r="E126">
+        <v>70</v>
+      </c>
+      <c r="F126">
+        <v>88</v>
+      </c>
+      <c r="G126" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H126" t="str">
+        <v/>
+      </c>
+      <c r="I126" t="str">
+        <v>8e8f4aa7-50c7-41cd-b30e-11ac468906b1.jpg</v>
+      </c>
+      <c r="J126" t="str">
+        <v/>
+      </c>
+      <c r="K126" t="str">
+        <v/>
+      </c>
+      <c r="L126" t="str">
+        <v/>
+      </c>
+      <c r="M126" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="str">
+        <v>LW-88</v>
+      </c>
+      <c r="B127" t="str">
+        <v>set mundu</v>
+      </c>
+      <c r="C127" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D127" t="str">
+        <v/>
+      </c>
+      <c r="E127">
+        <v>49</v>
+      </c>
+      <c r="F127">
+        <v>55</v>
+      </c>
+      <c r="G127" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H127" t="str">
+        <v/>
+      </c>
+      <c r="I127" t="str">
+        <v>dd5084c5-8160-4bcc-8047-0c11e2307a41.jpg</v>
+      </c>
+      <c r="J127" t="str">
+        <v/>
+      </c>
+      <c r="K127" t="str">
+        <v/>
+      </c>
+      <c r="L127" t="str">
+        <v/>
+      </c>
+      <c r="M127" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="str">
+        <v>LW-89</v>
+      </c>
+      <c r="B128" t="str">
+        <v>stretchable blouse</v>
+      </c>
+      <c r="C128" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D128" t="str">
+        <v/>
+      </c>
+      <c r="E128">
+        <v>35</v>
+      </c>
+      <c r="F128">
+        <v>40</v>
+      </c>
+      <c r="G128" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H128" t="str">
+        <v>size XXL</v>
+      </c>
+      <c r="I128" t="str">
+        <v>0fa0d4aa-5d26-441e-80e1-78f485955936.jpg</v>
+      </c>
+      <c r="J128" t="str">
+        <v/>
+      </c>
+      <c r="K128" t="str">
+        <v/>
+      </c>
+      <c r="L128" t="str">
+        <v/>
+      </c>
+      <c r="M128" t="str">
+        <v>No</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M118"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M128"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update store products via Admin Panel - 22/08/2026, 7:34:02 am
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -7281,10 +7281,10 @@
         <v>Necklace</v>
       </c>
       <c r="E167">
-        <v>62</v>
+        <v>49</v>
       </c>
       <c r="F167">
-        <v>76</v>
+        <v>64</v>
       </c>
       <c r="G167" t="str">
         <v>INSTOCK</v>

</xml_diff>

<commit_message>
Update store products via Admin Panel - 22/08/2026, 7:35:47 am
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -753,10 +753,10 @@
         <v>Earring</v>
       </c>
       <c r="E9">
-        <v>6</v>
+        <v>9.99</v>
       </c>
       <c r="F9">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="G9" t="str">
         <v>INSTOCK</v>
@@ -2166,7 +2166,7 @@
         <v>29</v>
       </c>
       <c r="G43" t="str">
-        <v>INSTOCK</v>
+        <v>SOLD OUT</v>
       </c>
       <c r="H43" t="str">
         <v/>

</xml_diff>

<commit_message>
Update store products via Admin Panel - 25/08/2026, 11:01:00 am
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -4819,7 +4819,7 @@
         <v>55</v>
       </c>
       <c r="G107" t="str">
-        <v>INSTOCK</v>
+        <v>SOLD OUT</v>
       </c>
       <c r="H107" t="str">
         <v/>
@@ -6795,7 +6795,7 @@
         <v>50</v>
       </c>
       <c r="G155" t="str">
-        <v>INSTOCK</v>
+        <v>SOLD OUT</v>
       </c>
       <c r="H155" t="str">
         <v/>
@@ -8893,7 +8893,7 @@
         <v>50</v>
       </c>
       <c r="G205" t="str">
-        <v>INSTOCK</v>
+        <v>SOLD OUT</v>
       </c>
       <c r="H205" t="str">
         <v>BLOUSE -FREE SIZE</v>

</xml_diff>

<commit_message>
Update store products via Admin Panel - 25/08/2026, 11:48:07 pm
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M227"/>
+  <dimension ref="A1:M230"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -9829,9 +9829,132 @@
         <v>No</v>
       </c>
     </row>
+    <row r="228">
+      <c r="A228" t="str">
+        <v>LW-153</v>
+      </c>
+      <c r="B228" t="str">
+        <v>saree</v>
+      </c>
+      <c r="C228" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D228" t="str">
+        <v/>
+      </c>
+      <c r="E228">
+        <v>62</v>
+      </c>
+      <c r="F228">
+        <v>75</v>
+      </c>
+      <c r="G228" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H228" t="str">
+        <v/>
+      </c>
+      <c r="I228" t="str">
+        <v>2c904b61-ff56-49a6-8e90-f1e1a99ca6ff.jpg</v>
+      </c>
+      <c r="J228" t="str">
+        <v/>
+      </c>
+      <c r="K228" t="str">
+        <v/>
+      </c>
+      <c r="L228" t="str">
+        <v/>
+      </c>
+      <c r="M228" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="str">
+        <v>LW-154</v>
+      </c>
+      <c r="B229" t="str">
+        <v>off-white saree</v>
+      </c>
+      <c r="C229" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D229" t="str">
+        <v/>
+      </c>
+      <c r="E229">
+        <v>68</v>
+      </c>
+      <c r="F229">
+        <v>79</v>
+      </c>
+      <c r="G229" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H229" t="str">
+        <v/>
+      </c>
+      <c r="I229" t="str">
+        <v>44aabda1-308b-428a-ae9b-e8096c8aadf1.jpg</v>
+      </c>
+      <c r="J229" t="str">
+        <v/>
+      </c>
+      <c r="K229" t="str">
+        <v/>
+      </c>
+      <c r="L229" t="str">
+        <v>different shades available</v>
+      </c>
+      <c r="M229" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="str">
+        <v>LW-155</v>
+      </c>
+      <c r="B230" t="str">
+        <v>off-white saree with golden border</v>
+      </c>
+      <c r="C230" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D230" t="str">
+        <v/>
+      </c>
+      <c r="E230">
+        <v>68</v>
+      </c>
+      <c r="F230">
+        <v>74</v>
+      </c>
+      <c r="G230" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H230" t="str">
+        <v/>
+      </c>
+      <c r="I230" t="str">
+        <v>2e7bfdbd-bcaa-42f6-8f7c-2fb8984fc4cc.jpg</v>
+      </c>
+      <c r="J230" t="str">
+        <v/>
+      </c>
+      <c r="K230" t="str">
+        <v/>
+      </c>
+      <c r="L230" t="str">
+        <v>different shades available</v>
+      </c>
+      <c r="M230" t="str">
+        <v>No</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M227"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M230"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update store products via Admin Panel - 26/08/2026, 12:08:00 am
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M230"/>
+  <dimension ref="A1:M242"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -9952,9 +9952,501 @@
         <v>No</v>
       </c>
     </row>
+    <row r="231">
+      <c r="A231" t="str">
+        <v>GW-03</v>
+      </c>
+      <c r="B231" t="str">
+        <v>Mundu/Dhothi</v>
+      </c>
+      <c r="C231" t="str">
+        <v>Mens Wear</v>
+      </c>
+      <c r="D231" t="str">
+        <v/>
+      </c>
+      <c r="E231">
+        <v>38</v>
+      </c>
+      <c r="F231">
+        <v>46</v>
+      </c>
+      <c r="G231" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H231" t="str">
+        <v/>
+      </c>
+      <c r="I231" t="str">
+        <v>3d348698-2adf-42dc-85c6-aef020860866.jpg</v>
+      </c>
+      <c r="J231" t="str">
+        <v>3ae2f597-597e-468a-9335-882ab72a4fc6.jpg</v>
+      </c>
+      <c r="K231" t="str">
+        <v>7666aab4-33e1-42e2-aae4-f8389389469e.jpg</v>
+      </c>
+      <c r="L231" t="str">
+        <v>Available in white and off-white shades</v>
+      </c>
+      <c r="M231" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="str">
+        <v>GW-04</v>
+      </c>
+      <c r="B232" t="str">
+        <v>Shirt</v>
+      </c>
+      <c r="C232" t="str">
+        <v>Mens Wear</v>
+      </c>
+      <c r="D232" t="str">
+        <v/>
+      </c>
+      <c r="E232">
+        <v>48</v>
+      </c>
+      <c r="F232">
+        <v>50</v>
+      </c>
+      <c r="G232" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H232" t="str">
+        <v>44</v>
+      </c>
+      <c r="I232" t="str">
+        <v>73fbad63-cbd8-43ad-8fb9-6e7ee9d184f9.jpg</v>
+      </c>
+      <c r="J232" t="str">
+        <v/>
+      </c>
+      <c r="K232" t="str">
+        <v/>
+      </c>
+      <c r="L232" t="str">
+        <v/>
+      </c>
+      <c r="M232" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="str">
+        <v>GW-05</v>
+      </c>
+      <c r="B233" t="str">
+        <v>Shirt and Dhothi  combo</v>
+      </c>
+      <c r="C233" t="str">
+        <v>Mens Wear</v>
+      </c>
+      <c r="D233" t="str">
+        <v/>
+      </c>
+      <c r="E233">
+        <v>65</v>
+      </c>
+      <c r="F233">
+        <v>70</v>
+      </c>
+      <c r="G233" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H233" t="str">
+        <v>42</v>
+      </c>
+      <c r="I233" t="str">
+        <v>56ecb82e-326c-4ba8-bc5b-b9412d3a0e8c.jpg</v>
+      </c>
+      <c r="J233" t="str">
+        <v/>
+      </c>
+      <c r="K233" t="str">
+        <v/>
+      </c>
+      <c r="L233" t="str">
+        <v>Limited stock</v>
+      </c>
+      <c r="M233" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="str">
+        <v>GW-06</v>
+      </c>
+      <c r="B234" t="str">
+        <v>Shirt</v>
+      </c>
+      <c r="C234" t="str">
+        <v>Mens Wear</v>
+      </c>
+      <c r="D234" t="str">
+        <v/>
+      </c>
+      <c r="E234">
+        <v>43</v>
+      </c>
+      <c r="F234">
+        <v>52</v>
+      </c>
+      <c r="G234" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H234" t="str">
+        <v>42</v>
+      </c>
+      <c r="I234" t="str">
+        <v>1db824cf-c622-4bb2-90e2-34e22226b725.jpg</v>
+      </c>
+      <c r="J234" t="str">
+        <v/>
+      </c>
+      <c r="K234" t="str">
+        <v/>
+      </c>
+      <c r="L234" t="str">
+        <v>Different  shades available. Limited  stock</v>
+      </c>
+      <c r="M234" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="str">
+        <v>GW-07</v>
+      </c>
+      <c r="B235" t="str">
+        <v>Shirt</v>
+      </c>
+      <c r="C235" t="str">
+        <v>Mens Wear</v>
+      </c>
+      <c r="D235" t="str">
+        <v/>
+      </c>
+      <c r="E235">
+        <v>43</v>
+      </c>
+      <c r="F235">
+        <v>54</v>
+      </c>
+      <c r="G235" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H235" t="str">
+        <v>42</v>
+      </c>
+      <c r="I235" t="str">
+        <v>999e743a-0700-4a90-9331-b13f53a12162.jpg</v>
+      </c>
+      <c r="J235" t="str">
+        <v/>
+      </c>
+      <c r="K235" t="str">
+        <v/>
+      </c>
+      <c r="L235" t="str">
+        <v>Different  shades available. Limited  stock</v>
+      </c>
+      <c r="M235" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="str">
+        <v>LW-156</v>
+      </c>
+      <c r="B236" t="str">
+        <v>couple combo</v>
+      </c>
+      <c r="C236" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D236" t="str">
+        <v/>
+      </c>
+      <c r="E236">
+        <v>99</v>
+      </c>
+      <c r="F236">
+        <v>115</v>
+      </c>
+      <c r="G236" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H236" t="str">
+        <v>shirt 42</v>
+      </c>
+      <c r="I236" t="str">
+        <v>b6f29c53-9976-4ad7-a689-14b8f73a18f9.jpg</v>
+      </c>
+      <c r="J236" t="str">
+        <v/>
+      </c>
+      <c r="K236" t="str">
+        <v/>
+      </c>
+      <c r="L236" t="str">
+        <v>Different  shades available. Limited  stock</v>
+      </c>
+      <c r="M236" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="str">
+        <v>GW-08</v>
+      </c>
+      <c r="B237" t="str">
+        <v>shirt</v>
+      </c>
+      <c r="C237" t="str">
+        <v>Mens Wear</v>
+      </c>
+      <c r="D237" t="str">
+        <v/>
+      </c>
+      <c r="E237">
+        <v>46</v>
+      </c>
+      <c r="F237">
+        <v>53</v>
+      </c>
+      <c r="G237" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H237" t="str">
+        <v>42</v>
+      </c>
+      <c r="I237" t="str">
+        <v>b51d55fe-0cf3-4c14-b7db-5ba57a59337c.jpg</v>
+      </c>
+      <c r="J237" t="str">
+        <v/>
+      </c>
+      <c r="K237" t="str">
+        <v/>
+      </c>
+      <c r="L237" t="str">
+        <v>Limited  stock</v>
+      </c>
+      <c r="M237" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="str">
+        <v>GW-09</v>
+      </c>
+      <c r="B238" t="str">
+        <v>Shirt</v>
+      </c>
+      <c r="C238" t="str">
+        <v>Mens Wear</v>
+      </c>
+      <c r="D238" t="str">
+        <v/>
+      </c>
+      <c r="E238">
+        <v>44</v>
+      </c>
+      <c r="F238">
+        <v>53</v>
+      </c>
+      <c r="G238" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H238" t="str">
+        <v>L and XL</v>
+      </c>
+      <c r="I238" t="str">
+        <v>b857f5b8-b45e-420d-af23-55a4c3ccbe03.jpg</v>
+      </c>
+      <c r="J238" t="str">
+        <v/>
+      </c>
+      <c r="K238" t="str">
+        <v/>
+      </c>
+      <c r="L238" t="str">
+        <v>Limited  stock</v>
+      </c>
+      <c r="M238" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="str">
+        <v>GW-10</v>
+      </c>
+      <c r="B239" t="str">
+        <v>COMBO</v>
+      </c>
+      <c r="C239" t="str">
+        <v>Mens Wear</v>
+      </c>
+      <c r="D239" t="str">
+        <v/>
+      </c>
+      <c r="E239">
+        <v>66</v>
+      </c>
+      <c r="F239">
+        <v>78</v>
+      </c>
+      <c r="G239" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H239" t="str">
+        <v>40</v>
+      </c>
+      <c r="I239" t="str">
+        <v>90c4faa5-5c03-460b-ac8f-21a1d7bae3d2.jpg</v>
+      </c>
+      <c r="J239" t="str">
+        <v/>
+      </c>
+      <c r="K239" t="str">
+        <v/>
+      </c>
+      <c r="L239" t="str">
+        <v>Limited  stock</v>
+      </c>
+      <c r="M239" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="str">
+        <v>GW-11</v>
+      </c>
+      <c r="B240" t="str">
+        <v>COMBO</v>
+      </c>
+      <c r="C240" t="str">
+        <v>Mens Wear</v>
+      </c>
+      <c r="D240" t="str">
+        <v/>
+      </c>
+      <c r="E240">
+        <v>65</v>
+      </c>
+      <c r="F240">
+        <v>70</v>
+      </c>
+      <c r="G240" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H240" t="str">
+        <v>42</v>
+      </c>
+      <c r="I240" t="str">
+        <v>93ea743a-9078-4985-abf9-e8e93079dfe5.jpg</v>
+      </c>
+      <c r="J240" t="str">
+        <v/>
+      </c>
+      <c r="K240" t="str">
+        <v/>
+      </c>
+      <c r="L240" t="str">
+        <v>Limited  stock</v>
+      </c>
+      <c r="M240" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="str">
+        <v>GW-12</v>
+      </c>
+      <c r="B241" t="str">
+        <v>SHIRT</v>
+      </c>
+      <c r="C241" t="str">
+        <v>Mens Wear</v>
+      </c>
+      <c r="D241" t="str">
+        <v/>
+      </c>
+      <c r="E241">
+        <v>42</v>
+      </c>
+      <c r="F241">
+        <v>55</v>
+      </c>
+      <c r="G241" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H241" t="str">
+        <v>42</v>
+      </c>
+      <c r="I241" t="str">
+        <v>eabeb1e1-4a1e-420c-a5a4-85b855fa7bae.jpg</v>
+      </c>
+      <c r="J241" t="str">
+        <v/>
+      </c>
+      <c r="K241" t="str">
+        <v/>
+      </c>
+      <c r="L241" t="str">
+        <v>Limited  stock</v>
+      </c>
+      <c r="M241" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="str">
+        <v>LW-157</v>
+      </c>
+      <c r="B242" t="str">
+        <v>Kanchi cotton</v>
+      </c>
+      <c r="C242" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D242" t="str">
+        <v/>
+      </c>
+      <c r="E242">
+        <v>58</v>
+      </c>
+      <c r="F242">
+        <v>68</v>
+      </c>
+      <c r="G242" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H242" t="str">
+        <v/>
+      </c>
+      <c r="I242" t="str">
+        <v>414b307c-c59d-4396-ad98-a9becb2c677d.jpg</v>
+      </c>
+      <c r="J242" t="str">
+        <v>14bc9be3-b4d3-4dca-89f9-5e68bdbcbb85.jpg</v>
+      </c>
+      <c r="K242" t="str">
+        <v/>
+      </c>
+      <c r="L242" t="str">
+        <v>Available in brown,violet and green shades</v>
+      </c>
+      <c r="M242" t="str">
+        <v>No</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M230"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M242"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update store products via Admin Panel - 26/08/2026, 12:17:00 am
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M242"/>
+  <dimension ref="A1:M246"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -10444,9 +10444,173 @@
         <v>No</v>
       </c>
     </row>
+    <row r="243">
+      <c r="A243" t="str">
+        <v>KW-16</v>
+      </c>
+      <c r="B243" t="str">
+        <v>pattupavada</v>
+      </c>
+      <c r="C243" t="str">
+        <v>Kids Wear</v>
+      </c>
+      <c r="D243" t="str">
+        <v/>
+      </c>
+      <c r="E243">
+        <v>45</v>
+      </c>
+      <c r="F243">
+        <v>49</v>
+      </c>
+      <c r="G243" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H243" t="str">
+        <v>available in different sizes</v>
+      </c>
+      <c r="I243" t="str">
+        <v>1c3d33b9-d00f-465c-bf66-b8ea3bde3a91.jpg</v>
+      </c>
+      <c r="J243" t="str">
+        <v/>
+      </c>
+      <c r="K243" t="str">
+        <v/>
+      </c>
+      <c r="L243" t="str">
+        <v>Different sizes  available. Limited  stock</v>
+      </c>
+      <c r="M243" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="str">
+        <v>KW-17</v>
+      </c>
+      <c r="B244" t="str">
+        <v>Pattupavada</v>
+      </c>
+      <c r="C244" t="str">
+        <v>Kids Wear</v>
+      </c>
+      <c r="D244" t="str">
+        <v/>
+      </c>
+      <c r="E244">
+        <v>45</v>
+      </c>
+      <c r="F244">
+        <v>49</v>
+      </c>
+      <c r="G244" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H244" t="str">
+        <v>6 yrs</v>
+      </c>
+      <c r="I244" t="str">
+        <v>b1b908a9-58cd-4aea-85c6-a4b53e1218fa.jpg</v>
+      </c>
+      <c r="J244" t="str">
+        <v/>
+      </c>
+      <c r="K244" t="str">
+        <v/>
+      </c>
+      <c r="L244" t="str">
+        <v>Limited  stock</v>
+      </c>
+      <c r="M244" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="str">
+        <v>LW-158</v>
+      </c>
+      <c r="B245" t="str">
+        <v>saree</v>
+      </c>
+      <c r="C245" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D245" t="str">
+        <v/>
+      </c>
+      <c r="E245">
+        <v>55</v>
+      </c>
+      <c r="F245">
+        <v>65</v>
+      </c>
+      <c r="G245" t="str">
+        <v>SOLD OUT</v>
+      </c>
+      <c r="H245" t="str">
+        <v/>
+      </c>
+      <c r="I245" t="str">
+        <v>1c394569-ead3-4a6f-b4e6-32da72d74396.jpg</v>
+      </c>
+      <c r="J245" t="str">
+        <v/>
+      </c>
+      <c r="K245" t="str">
+        <v/>
+      </c>
+      <c r="L245" t="str">
+        <v/>
+      </c>
+      <c r="M245" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="str">
+        <v>LW-159</v>
+      </c>
+      <c r="B246" t="str">
+        <v>mulcotton saree</v>
+      </c>
+      <c r="C246" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D246" t="str">
+        <v/>
+      </c>
+      <c r="E246">
+        <v>49</v>
+      </c>
+      <c r="F246">
+        <v>55</v>
+      </c>
+      <c r="G246" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H246" t="str">
+        <v/>
+      </c>
+      <c r="I246" t="str">
+        <v>ec5ac18c-0c4e-4511-8a34-6f6d1e17a7fd.jpg</v>
+      </c>
+      <c r="J246" t="str">
+        <v/>
+      </c>
+      <c r="K246" t="str">
+        <v/>
+      </c>
+      <c r="L246" t="str">
+        <v>Limited  stock</v>
+      </c>
+      <c r="M246" t="str">
+        <v>No</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M242"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M246"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update store products via Admin Panel - 26/08/2026, 12:23:15 am
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M246"/>
+  <dimension ref="A1:M249"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -10608,9 +10608,132 @@
         <v>No</v>
       </c>
     </row>
+    <row r="247">
+      <c r="A247" t="str">
+        <v>GW-13</v>
+      </c>
+      <c r="B247" t="str">
+        <v>combo</v>
+      </c>
+      <c r="C247" t="str">
+        <v>Mens Wear</v>
+      </c>
+      <c r="D247" t="str">
+        <v/>
+      </c>
+      <c r="E247">
+        <v>66</v>
+      </c>
+      <c r="F247">
+        <v>70</v>
+      </c>
+      <c r="G247" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H247" t="str">
+        <v>40</v>
+      </c>
+      <c r="I247" t="str">
+        <v>0c84e23e-d5e2-407f-955f-051a7f17e7a8.jpg</v>
+      </c>
+      <c r="J247" t="str">
+        <v/>
+      </c>
+      <c r="K247" t="str">
+        <v/>
+      </c>
+      <c r="L247" t="str">
+        <v>Limited  stock</v>
+      </c>
+      <c r="M247" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="str">
+        <v>GW-14</v>
+      </c>
+      <c r="B248" t="str">
+        <v>combo</v>
+      </c>
+      <c r="C248" t="str">
+        <v>Mens Wear</v>
+      </c>
+      <c r="D248" t="str">
+        <v/>
+      </c>
+      <c r="E248">
+        <v>65</v>
+      </c>
+      <c r="F248">
+        <v>70</v>
+      </c>
+      <c r="G248" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H248" t="str">
+        <v>40</v>
+      </c>
+      <c r="I248" t="str">
+        <v>767fa8c0-a970-4817-88db-336fc7c72b0c.jpg</v>
+      </c>
+      <c r="J248" t="str">
+        <v/>
+      </c>
+      <c r="K248" t="str">
+        <v/>
+      </c>
+      <c r="L248" t="str">
+        <v>Limited  stock</v>
+      </c>
+      <c r="M248" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="str">
+        <v>GW-15</v>
+      </c>
+      <c r="B249" t="str">
+        <v>combo</v>
+      </c>
+      <c r="C249" t="str">
+        <v>Mens Wear</v>
+      </c>
+      <c r="D249" t="str">
+        <v/>
+      </c>
+      <c r="E249">
+        <v>65</v>
+      </c>
+      <c r="F249">
+        <v>70</v>
+      </c>
+      <c r="G249" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H249" t="str">
+        <v>40</v>
+      </c>
+      <c r="I249" t="str">
+        <v>248c5a7c-3b7e-48ff-8eb6-f55e443857f4.jpg</v>
+      </c>
+      <c r="J249" t="str">
+        <v/>
+      </c>
+      <c r="K249" t="str">
+        <v/>
+      </c>
+      <c r="L249" t="str">
+        <v>Limited  stock</v>
+      </c>
+      <c r="M249" t="str">
+        <v>No</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M246"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M249"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update store products via Admin Panel - 26/08/2026, 12:59:54 am
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M249"/>
+  <dimension ref="A1:M251"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -10731,9 +10731,91 @@
         <v>No</v>
       </c>
     </row>
+    <row r="250">
+      <c r="A250" t="str">
+        <v>GW-16</v>
+      </c>
+      <c r="B250" t="str">
+        <v>short kurtha</v>
+      </c>
+      <c r="C250" t="str">
+        <v>Mens Wear</v>
+      </c>
+      <c r="D250" t="str">
+        <v/>
+      </c>
+      <c r="E250">
+        <v>49</v>
+      </c>
+      <c r="F250">
+        <v>58</v>
+      </c>
+      <c r="G250" t="str">
+        <v>LIMITED STOCK</v>
+      </c>
+      <c r="H250" t="str">
+        <v>large</v>
+      </c>
+      <c r="I250" t="str">
+        <v>5a87bfc9-537f-4042-add7-4b086d0e7363.jpg</v>
+      </c>
+      <c r="J250" t="str">
+        <v/>
+      </c>
+      <c r="K250" t="str">
+        <v/>
+      </c>
+      <c r="L250" t="str">
+        <v/>
+      </c>
+      <c r="M250" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="str">
+        <v>LW-160</v>
+      </c>
+      <c r="B251" t="str">
+        <v>saree-partywear</v>
+      </c>
+      <c r="C251" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D251" t="str">
+        <v/>
+      </c>
+      <c r="E251">
+        <v>100</v>
+      </c>
+      <c r="F251">
+        <v>115</v>
+      </c>
+      <c r="G251" t="str">
+        <v>SOLD OUT</v>
+      </c>
+      <c r="H251" t="str">
+        <v/>
+      </c>
+      <c r="I251" t="str">
+        <v>ccb51645-5e50-4bf2-a1ce-c308c3cacd44.jpg</v>
+      </c>
+      <c r="J251" t="str">
+        <v/>
+      </c>
+      <c r="K251" t="str">
+        <v/>
+      </c>
+      <c r="L251" t="str">
+        <v/>
+      </c>
+      <c r="M251" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M249"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M251"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update store products via Admin Panel - 26/08/2026, 1:14:20 am
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M251"/>
+  <dimension ref="A1:M264"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -10813,9 +10813,542 @@
         <v>Yes</v>
       </c>
     </row>
+    <row r="252">
+      <c r="A252" t="str">
+        <v>LW-161</v>
+      </c>
+      <c r="B252" t="str">
+        <v>partywear saree</v>
+      </c>
+      <c r="C252" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D252" t="str">
+        <v/>
+      </c>
+      <c r="E252">
+        <v>94</v>
+      </c>
+      <c r="F252">
+        <v>100</v>
+      </c>
+      <c r="G252" t="str">
+        <v>LIMITED STOCK</v>
+      </c>
+      <c r="H252" t="str">
+        <v/>
+      </c>
+      <c r="I252" t="str">
+        <v>83844d90-bbb5-408a-9704-05b2c4ea1fda.jpg</v>
+      </c>
+      <c r="J252" t="str">
+        <v/>
+      </c>
+      <c r="K252" t="str">
+        <v/>
+      </c>
+      <c r="L252" t="str">
+        <v/>
+      </c>
+      <c r="M252" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="str">
+        <v>LW-162</v>
+      </c>
+      <c r="B253" t="str">
+        <v>Readymade blouse</v>
+      </c>
+      <c r="C253" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D253" t="str">
+        <v/>
+      </c>
+      <c r="E253">
+        <v>44</v>
+      </c>
+      <c r="F253">
+        <v>50</v>
+      </c>
+      <c r="G253" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H253" t="str">
+        <v>BLOUSE -FREE SIZE</v>
+      </c>
+      <c r="I253" t="str">
+        <v>6943ba73-f434-47bb-9cee-d9f4c37123df.jpg</v>
+      </c>
+      <c r="J253" t="str">
+        <v/>
+      </c>
+      <c r="K253" t="str">
+        <v/>
+      </c>
+      <c r="L253" t="str">
+        <v>limited stock</v>
+      </c>
+      <c r="M253" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="str">
+        <v>LW-163</v>
+      </c>
+      <c r="B254" t="str">
+        <v>saree</v>
+      </c>
+      <c r="C254" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D254" t="str">
+        <v/>
+      </c>
+      <c r="E254">
+        <v>89</v>
+      </c>
+      <c r="F254">
+        <v>95</v>
+      </c>
+      <c r="G254" t="str">
+        <v>LIMITED STOCK</v>
+      </c>
+      <c r="H254" t="str">
+        <v/>
+      </c>
+      <c r="I254" t="str">
+        <v>17b30f82-1e01-4599-8a5a-f0c621c031d1.jpg</v>
+      </c>
+      <c r="J254" t="str">
+        <v/>
+      </c>
+      <c r="K254" t="str">
+        <v/>
+      </c>
+      <c r="L254" t="str">
+        <v/>
+      </c>
+      <c r="M254" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="str">
+        <v>LW-164</v>
+      </c>
+      <c r="B255" t="str">
+        <v>partywear saree</v>
+      </c>
+      <c r="C255" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D255" t="str">
+        <v/>
+      </c>
+      <c r="E255">
+        <v>100</v>
+      </c>
+      <c r="F255">
+        <v>115</v>
+      </c>
+      <c r="G255" t="str">
+        <v>SOLD OUT</v>
+      </c>
+      <c r="H255" t="str">
+        <v/>
+      </c>
+      <c r="I255" t="str">
+        <v>5fb9fcb2-48ed-4738-8731-0f10ab0bf5ff.jpg</v>
+      </c>
+      <c r="J255" t="str">
+        <v/>
+      </c>
+      <c r="K255" t="str">
+        <v/>
+      </c>
+      <c r="L255" t="str">
+        <v>Velvet organza</v>
+      </c>
+      <c r="M255" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="str">
+        <v>LW-165</v>
+      </c>
+      <c r="B256" t="str">
+        <v>saree</v>
+      </c>
+      <c r="C256" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D256" t="str">
+        <v/>
+      </c>
+      <c r="E256">
+        <v>79</v>
+      </c>
+      <c r="F256">
+        <v>86</v>
+      </c>
+      <c r="G256" t="str">
+        <v>LIMITED STOCK</v>
+      </c>
+      <c r="H256" t="str">
+        <v/>
+      </c>
+      <c r="I256" t="str">
+        <v>d1cdd26b-84ed-4b21-b40c-95248903dd5f.jpg</v>
+      </c>
+      <c r="J256" t="str">
+        <v/>
+      </c>
+      <c r="K256" t="str">
+        <v/>
+      </c>
+      <c r="L256" t="str">
+        <v>semi tusser silk</v>
+      </c>
+      <c r="M256" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="str">
+        <v>LW-166</v>
+      </c>
+      <c r="B257" t="str">
+        <v>saree</v>
+      </c>
+      <c r="C257" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D257" t="str">
+        <v/>
+      </c>
+      <c r="E257">
+        <v>74</v>
+      </c>
+      <c r="F257">
+        <v>89</v>
+      </c>
+      <c r="G257" t="str">
+        <v>LIMITED STOCK</v>
+      </c>
+      <c r="H257" t="str">
+        <v/>
+      </c>
+      <c r="I257" t="str">
+        <v>74c75bb4-cc72-4f70-8fa1-7892675a9e2a.jpg</v>
+      </c>
+      <c r="J257" t="str">
+        <v/>
+      </c>
+      <c r="K257" t="str">
+        <v/>
+      </c>
+      <c r="L257" t="str">
+        <v>Semi tusser silk</v>
+      </c>
+      <c r="M257" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="str">
+        <v>LW-167</v>
+      </c>
+      <c r="B258" t="str">
+        <v>saree</v>
+      </c>
+      <c r="C258" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D258" t="str">
+        <v/>
+      </c>
+      <c r="E258">
+        <v>79</v>
+      </c>
+      <c r="F258">
+        <v>90</v>
+      </c>
+      <c r="G258" t="str">
+        <v>LIMITED STOCK</v>
+      </c>
+      <c r="H258" t="str">
+        <v/>
+      </c>
+      <c r="I258" t="str">
+        <v>b5229bc7-e36f-4de6-b982-d7693b07d0bd.jpg</v>
+      </c>
+      <c r="J258" t="str">
+        <v/>
+      </c>
+      <c r="K258" t="str">
+        <v/>
+      </c>
+      <c r="L258" t="str">
+        <v>Semi tusser silk</v>
+      </c>
+      <c r="M258" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="str">
+        <v>LW-168</v>
+      </c>
+      <c r="B259" t="str">
+        <v>saree</v>
+      </c>
+      <c r="C259" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D259" t="str">
+        <v/>
+      </c>
+      <c r="E259">
+        <v>76</v>
+      </c>
+      <c r="F259">
+        <v>89</v>
+      </c>
+      <c r="G259" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H259" t="str">
+        <v/>
+      </c>
+      <c r="I259" t="str">
+        <v>f0ede5dc-b458-494d-b1ff-c29afef6c669.jpg</v>
+      </c>
+      <c r="J259" t="str">
+        <v/>
+      </c>
+      <c r="K259" t="str">
+        <v/>
+      </c>
+      <c r="L259" t="str">
+        <v>Semi tusser silk</v>
+      </c>
+      <c r="M259" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="str">
+        <v>LW-169</v>
+      </c>
+      <c r="B260" t="str">
+        <v>saree</v>
+      </c>
+      <c r="C260" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D260" t="str">
+        <v/>
+      </c>
+      <c r="E260">
+        <v>55</v>
+      </c>
+      <c r="F260">
+        <v>65</v>
+      </c>
+      <c r="G260" t="str">
+        <v>SOLD OUT</v>
+      </c>
+      <c r="H260" t="str">
+        <v/>
+      </c>
+      <c r="I260" t="str">
+        <v>0d12ea0b-d8d1-4650-ad23-e09bfa797cd9.jpg</v>
+      </c>
+      <c r="J260" t="str">
+        <v/>
+      </c>
+      <c r="K260" t="str">
+        <v/>
+      </c>
+      <c r="L260" t="str">
+        <v>Raga tissue saree</v>
+      </c>
+      <c r="M260" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="str">
+        <v>LW-170</v>
+      </c>
+      <c r="B261" t="str">
+        <v>saree</v>
+      </c>
+      <c r="C261" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D261" t="str">
+        <v/>
+      </c>
+      <c r="E261">
+        <v>75</v>
+      </c>
+      <c r="F261">
+        <v>89</v>
+      </c>
+      <c r="G261" t="str">
+        <v>LIMITED STOCK</v>
+      </c>
+      <c r="H261" t="str">
+        <v/>
+      </c>
+      <c r="I261" t="str">
+        <v>e52500cd-caca-4aad-8061-02391d42dc77.jpg</v>
+      </c>
+      <c r="J261" t="str">
+        <v/>
+      </c>
+      <c r="K261" t="str">
+        <v/>
+      </c>
+      <c r="L261" t="str">
+        <v/>
+      </c>
+      <c r="M261" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="str">
+        <v>LW-171</v>
+      </c>
+      <c r="B262" t="str">
+        <v>chikankary Rayon  ready made set</v>
+      </c>
+      <c r="C262" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D262" t="str">
+        <v/>
+      </c>
+      <c r="E262">
+        <v>75</v>
+      </c>
+      <c r="F262">
+        <v>79</v>
+      </c>
+      <c r="G262" t="str">
+        <v>SOLD OUT</v>
+      </c>
+      <c r="H262" t="str">
+        <v>large</v>
+      </c>
+      <c r="I262" t="str">
+        <v>65957e11-c6e3-44f8-836f-a61d5f5b2368.jpg</v>
+      </c>
+      <c r="J262" t="str">
+        <v/>
+      </c>
+      <c r="K262" t="str">
+        <v/>
+      </c>
+      <c r="L262" t="str">
+        <v/>
+      </c>
+      <c r="M262" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="str">
+        <v>KW-18</v>
+      </c>
+      <c r="B263" t="str">
+        <v>Pattupavada</v>
+      </c>
+      <c r="C263" t="str">
+        <v>Kids Wear</v>
+      </c>
+      <c r="D263" t="str">
+        <v/>
+      </c>
+      <c r="E263">
+        <v>48</v>
+      </c>
+      <c r="F263">
+        <v>55</v>
+      </c>
+      <c r="G263" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H263" t="str">
+        <v>all sizes available</v>
+      </c>
+      <c r="I263" t="str">
+        <v>55a2ce11-3c68-4b77-b590-4b78bf8e5135.jpg</v>
+      </c>
+      <c r="J263" t="str">
+        <v/>
+      </c>
+      <c r="K263" t="str">
+        <v/>
+      </c>
+      <c r="L263" t="str">
+        <v>different sizes available until 10 yrs</v>
+      </c>
+      <c r="M263" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="str">
+        <v>LW-172</v>
+      </c>
+      <c r="B264" t="str">
+        <v>Davani</v>
+      </c>
+      <c r="C264" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D264" t="str">
+        <v/>
+      </c>
+      <c r="E264">
+        <v>100</v>
+      </c>
+      <c r="F264">
+        <v>115</v>
+      </c>
+      <c r="G264" t="str">
+        <v>SOLD OUT</v>
+      </c>
+      <c r="H264" t="str">
+        <v/>
+      </c>
+      <c r="I264" t="str">
+        <v>14ca9b4e-1a9e-4cb6-8c3c-6eaf3d1944ca.jpg</v>
+      </c>
+      <c r="J264" t="str">
+        <v/>
+      </c>
+      <c r="K264" t="str">
+        <v/>
+      </c>
+      <c r="L264" t="str">
+        <v/>
+      </c>
+      <c r="M264" t="str">
+        <v>No</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M251"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M264"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update store products via Admin Panel - 26/08/2026, 1:16:42 am
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M264"/>
+  <dimension ref="A1:M263"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -9931,7 +9931,7 @@
         <v>74</v>
       </c>
       <c r="G230" t="str">
-        <v>INSTOCK</v>
+        <v>SOLD OUT</v>
       </c>
       <c r="H230" t="str">
         <v/>
@@ -11020,7 +11020,7 @@
     </row>
     <row r="257">
       <c r="A257" t="str">
-        <v>LW-166</v>
+        <v>LW-167</v>
       </c>
       <c r="B257" t="str">
         <v>saree</v>
@@ -11032,10 +11032,10 @@
         <v/>
       </c>
       <c r="E257">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="F257">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="G257" t="str">
         <v>LIMITED STOCK</v>
@@ -11044,7 +11044,7 @@
         <v/>
       </c>
       <c r="I257" t="str">
-        <v>74c75bb4-cc72-4f70-8fa1-7892675a9e2a.jpg</v>
+        <v>b5229bc7-e36f-4de6-b982-d7693b07d0bd.jpg</v>
       </c>
       <c r="J257" t="str">
         <v/>
@@ -11061,7 +11061,7 @@
     </row>
     <row r="258">
       <c r="A258" t="str">
-        <v>LW-167</v>
+        <v>LW-168</v>
       </c>
       <c r="B258" t="str">
         <v>saree</v>
@@ -11073,19 +11073,19 @@
         <v/>
       </c>
       <c r="E258">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="F258">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="G258" t="str">
-        <v>LIMITED STOCK</v>
+        <v>INSTOCK</v>
       </c>
       <c r="H258" t="str">
         <v/>
       </c>
       <c r="I258" t="str">
-        <v>b5229bc7-e36f-4de6-b982-d7693b07d0bd.jpg</v>
+        <v>f0ede5dc-b458-494d-b1ff-c29afef6c669.jpg</v>
       </c>
       <c r="J258" t="str">
         <v/>
@@ -11102,7 +11102,7 @@
     </row>
     <row r="259">
       <c r="A259" t="str">
-        <v>LW-168</v>
+        <v>LW-169</v>
       </c>
       <c r="B259" t="str">
         <v>saree</v>
@@ -11114,19 +11114,19 @@
         <v/>
       </c>
       <c r="E259">
-        <v>76</v>
+        <v>55</v>
       </c>
       <c r="F259">
-        <v>89</v>
+        <v>65</v>
       </c>
       <c r="G259" t="str">
-        <v>INSTOCK</v>
+        <v>SOLD OUT</v>
       </c>
       <c r="H259" t="str">
         <v/>
       </c>
       <c r="I259" t="str">
-        <v>f0ede5dc-b458-494d-b1ff-c29afef6c669.jpg</v>
+        <v>0d12ea0b-d8d1-4650-ad23-e09bfa797cd9.jpg</v>
       </c>
       <c r="J259" t="str">
         <v/>
@@ -11135,7 +11135,7 @@
         <v/>
       </c>
       <c r="L259" t="str">
-        <v>Semi tusser silk</v>
+        <v>Raga tissue saree</v>
       </c>
       <c r="M259" t="str">
         <v>No</v>
@@ -11143,7 +11143,7 @@
     </row>
     <row r="260">
       <c r="A260" t="str">
-        <v>LW-169</v>
+        <v>LW-170</v>
       </c>
       <c r="B260" t="str">
         <v>saree</v>
@@ -11155,19 +11155,19 @@
         <v/>
       </c>
       <c r="E260">
-        <v>55</v>
+        <v>75</v>
       </c>
       <c r="F260">
-        <v>65</v>
+        <v>89</v>
       </c>
       <c r="G260" t="str">
-        <v>SOLD OUT</v>
+        <v>LIMITED STOCK</v>
       </c>
       <c r="H260" t="str">
         <v/>
       </c>
       <c r="I260" t="str">
-        <v>0d12ea0b-d8d1-4650-ad23-e09bfa797cd9.jpg</v>
+        <v>e52500cd-caca-4aad-8061-02391d42dc77.jpg</v>
       </c>
       <c r="J260" t="str">
         <v/>
@@ -11176,7 +11176,7 @@
         <v/>
       </c>
       <c r="L260" t="str">
-        <v>Raga tissue saree</v>
+        <v/>
       </c>
       <c r="M260" t="str">
         <v>No</v>
@@ -11184,10 +11184,10 @@
     </row>
     <row r="261">
       <c r="A261" t="str">
-        <v>LW-170</v>
+        <v>LW-171</v>
       </c>
       <c r="B261" t="str">
-        <v>saree</v>
+        <v>chikankary Rayon  ready made set</v>
       </c>
       <c r="C261" t="str">
         <v>Ladies Wear</v>
@@ -11199,16 +11199,16 @@
         <v>75</v>
       </c>
       <c r="F261">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="G261" t="str">
-        <v>LIMITED STOCK</v>
+        <v>SOLD OUT</v>
       </c>
       <c r="H261" t="str">
-        <v/>
+        <v>large</v>
       </c>
       <c r="I261" t="str">
-        <v>e52500cd-caca-4aad-8061-02391d42dc77.jpg</v>
+        <v>65957e11-c6e3-44f8-836f-a61d5f5b2368.jpg</v>
       </c>
       <c r="J261" t="str">
         <v/>
@@ -11225,31 +11225,31 @@
     </row>
     <row r="262">
       <c r="A262" t="str">
-        <v>LW-171</v>
+        <v>KW-18</v>
       </c>
       <c r="B262" t="str">
-        <v>chikankary Rayon  ready made set</v>
+        <v>Pattupavada</v>
       </c>
       <c r="C262" t="str">
-        <v>Ladies Wear</v>
+        <v>Kids Wear</v>
       </c>
       <c r="D262" t="str">
         <v/>
       </c>
       <c r="E262">
-        <v>75</v>
+        <v>48</v>
       </c>
       <c r="F262">
-        <v>79</v>
+        <v>55</v>
       </c>
       <c r="G262" t="str">
-        <v>SOLD OUT</v>
+        <v>INSTOCK</v>
       </c>
       <c r="H262" t="str">
-        <v>large</v>
+        <v>all sizes available</v>
       </c>
       <c r="I262" t="str">
-        <v>65957e11-c6e3-44f8-836f-a61d5f5b2368.jpg</v>
+        <v>55a2ce11-3c68-4b77-b590-4b78bf8e5135.jpg</v>
       </c>
       <c r="J262" t="str">
         <v/>
@@ -11258,7 +11258,7 @@
         <v/>
       </c>
       <c r="L262" t="str">
-        <v/>
+        <v>different sizes available until 10 yrs</v>
       </c>
       <c r="M262" t="str">
         <v>No</v>
@@ -11266,31 +11266,31 @@
     </row>
     <row r="263">
       <c r="A263" t="str">
-        <v>KW-18</v>
+        <v>LW-172</v>
       </c>
       <c r="B263" t="str">
-        <v>Pattupavada</v>
+        <v>Davani</v>
       </c>
       <c r="C263" t="str">
-        <v>Kids Wear</v>
+        <v>Ladies Wear</v>
       </c>
       <c r="D263" t="str">
         <v/>
       </c>
       <c r="E263">
-        <v>48</v>
+        <v>100</v>
       </c>
       <c r="F263">
-        <v>55</v>
+        <v>115</v>
       </c>
       <c r="G263" t="str">
-        <v>INSTOCK</v>
+        <v>SOLD OUT</v>
       </c>
       <c r="H263" t="str">
-        <v>all sizes available</v>
+        <v/>
       </c>
       <c r="I263" t="str">
-        <v>55a2ce11-3c68-4b77-b590-4b78bf8e5135.jpg</v>
+        <v>14ca9b4e-1a9e-4cb6-8c3c-6eaf3d1944ca.jpg</v>
       </c>
       <c r="J263" t="str">
         <v/>
@@ -11299,56 +11299,15 @@
         <v/>
       </c>
       <c r="L263" t="str">
-        <v>different sizes available until 10 yrs</v>
+        <v/>
       </c>
       <c r="M263" t="str">
-        <v>No</v>
-      </c>
-    </row>
-    <row r="264">
-      <c r="A264" t="str">
-        <v>LW-172</v>
-      </c>
-      <c r="B264" t="str">
-        <v>Davani</v>
-      </c>
-      <c r="C264" t="str">
-        <v>Ladies Wear</v>
-      </c>
-      <c r="D264" t="str">
-        <v/>
-      </c>
-      <c r="E264">
-        <v>100</v>
-      </c>
-      <c r="F264">
-        <v>115</v>
-      </c>
-      <c r="G264" t="str">
-        <v>SOLD OUT</v>
-      </c>
-      <c r="H264" t="str">
-        <v/>
-      </c>
-      <c r="I264" t="str">
-        <v>14ca9b4e-1a9e-4cb6-8c3c-6eaf3d1944ca.jpg</v>
-      </c>
-      <c r="J264" t="str">
-        <v/>
-      </c>
-      <c r="K264" t="str">
-        <v/>
-      </c>
-      <c r="L264" t="str">
-        <v/>
-      </c>
-      <c r="M264" t="str">
         <v>No</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M264"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M263"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update store products via Admin Panel - 26/08/2026, 1:33:52 am
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M263"/>
+  <dimension ref="A1:M272"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -11305,9 +11305,378 @@
         <v>No</v>
       </c>
     </row>
+    <row r="264">
+      <c r="A264" t="str">
+        <v>LW-173</v>
+      </c>
+      <c r="B264" t="str">
+        <v>Readymade salwar  set</v>
+      </c>
+      <c r="C264" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D264" t="str">
+        <v/>
+      </c>
+      <c r="E264">
+        <v>71</v>
+      </c>
+      <c r="F264">
+        <v>78</v>
+      </c>
+      <c r="G264" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H264" t="str">
+        <v>L</v>
+      </c>
+      <c r="I264" t="str">
+        <v>67898e22-8611-4727-8a91-20defc8e9b69.jpg</v>
+      </c>
+      <c r="J264" t="str">
+        <v/>
+      </c>
+      <c r="K264" t="str">
+        <v/>
+      </c>
+      <c r="L264" t="str">
+        <v>semi silk</v>
+      </c>
+      <c r="M264" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="str">
+        <v>LW-174</v>
+      </c>
+      <c r="B265" t="str">
+        <v>Premium  Blouse</v>
+      </c>
+      <c r="C265" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D265" t="str">
+        <v/>
+      </c>
+      <c r="E265">
+        <v>49</v>
+      </c>
+      <c r="F265">
+        <v>55</v>
+      </c>
+      <c r="G265" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H265" t="str">
+        <v>BLOUSE -FREE SIZE</v>
+      </c>
+      <c r="I265" t="str">
+        <v>09f3f54c-e96f-44d0-a875-0bab07c4c51e.jpg</v>
+      </c>
+      <c r="J265" t="str">
+        <v/>
+      </c>
+      <c r="K265" t="str">
+        <v/>
+      </c>
+      <c r="L265" t="str">
+        <v>Alterable, chest margin up to42</v>
+      </c>
+      <c r="M265" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="str">
+        <v>LW-175</v>
+      </c>
+      <c r="B266" t="str">
+        <v>3 piece readymade churidar</v>
+      </c>
+      <c r="C266" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D266" t="str">
+        <v/>
+      </c>
+      <c r="E266">
+        <v>69</v>
+      </c>
+      <c r="F266">
+        <v>78</v>
+      </c>
+      <c r="G266" t="str">
+        <v>LIMITED STOCK</v>
+      </c>
+      <c r="H266" t="str">
+        <v>xl,2xl,3xl</v>
+      </c>
+      <c r="I266" t="str">
+        <v>355f0ed8-3217-49b0-8573-d99749d12142.jpg</v>
+      </c>
+      <c r="J266" t="str">
+        <v/>
+      </c>
+      <c r="K266" t="str">
+        <v/>
+      </c>
+      <c r="L266" t="str">
+        <v>Mul chanderi fabric</v>
+      </c>
+      <c r="M266" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="str">
+        <v>JW-65</v>
+      </c>
+      <c r="B267" t="str">
+        <v>Necklace</v>
+      </c>
+      <c r="C267" t="str">
+        <v>Jewellery</v>
+      </c>
+      <c r="D267" t="str">
+        <v>Necklace</v>
+      </c>
+      <c r="E267">
+        <v>18</v>
+      </c>
+      <c r="F267">
+        <v>21.99</v>
+      </c>
+      <c r="G267" t="str">
+        <v>LIMITED STOCK</v>
+      </c>
+      <c r="H267" t="str">
+        <v/>
+      </c>
+      <c r="I267" t="str">
+        <v>7281cc57-59cd-4cc1-8b43-4707b71dd599.jpg</v>
+      </c>
+      <c r="J267" t="str">
+        <v/>
+      </c>
+      <c r="K267" t="str">
+        <v/>
+      </c>
+      <c r="L267" t="str">
+        <v/>
+      </c>
+      <c r="M267" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="str">
+        <v>JW-66</v>
+      </c>
+      <c r="B268" t="str">
+        <v>Necklace</v>
+      </c>
+      <c r="C268" t="str">
+        <v>Jewellery</v>
+      </c>
+      <c r="D268" t="str">
+        <v>Necklace</v>
+      </c>
+      <c r="E268">
+        <v>34</v>
+      </c>
+      <c r="F268">
+        <v>37</v>
+      </c>
+      <c r="G268" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H268" t="str">
+        <v/>
+      </c>
+      <c r="I268" t="str">
+        <v>9c8c799b-90fb-419e-b16d-f1e01266c2e6.jpg</v>
+      </c>
+      <c r="J268" t="str">
+        <v/>
+      </c>
+      <c r="K268" t="str">
+        <v/>
+      </c>
+      <c r="L268" t="str">
+        <v>Nagapadam</v>
+      </c>
+      <c r="M268" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="str">
+        <v>LW-176</v>
+      </c>
+      <c r="B269" t="str">
+        <v>Kaftan</v>
+      </c>
+      <c r="C269" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D269" t="str">
+        <v/>
+      </c>
+      <c r="E269">
+        <v>60</v>
+      </c>
+      <c r="F269">
+        <v>65</v>
+      </c>
+      <c r="G269" t="str">
+        <v>LIMITED STOCK</v>
+      </c>
+      <c r="H269" t="str">
+        <v>38</v>
+      </c>
+      <c r="I269" t="str">
+        <v>77c8ee93-e87e-4fe1-aeed-6b25d83c37e0.jpg</v>
+      </c>
+      <c r="J269" t="str">
+        <v/>
+      </c>
+      <c r="K269" t="str">
+        <v/>
+      </c>
+      <c r="L269" t="str">
+        <v/>
+      </c>
+      <c r="M269" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="str">
+        <v>LW-177</v>
+      </c>
+      <c r="B270" t="str">
+        <v>Readymade churidar</v>
+      </c>
+      <c r="C270" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D270" t="str">
+        <v/>
+      </c>
+      <c r="E270">
+        <v>69</v>
+      </c>
+      <c r="F270">
+        <v>78</v>
+      </c>
+      <c r="G270" t="str">
+        <v>LIMITED STOCK</v>
+      </c>
+      <c r="H270" t="str">
+        <v>Large</v>
+      </c>
+      <c r="I270" t="str">
+        <v>100e031c-c807-4250-869a-dbf5b1e146ca.jpg</v>
+      </c>
+      <c r="J270" t="str">
+        <v/>
+      </c>
+      <c r="K270" t="str">
+        <v/>
+      </c>
+      <c r="L270" t="str">
+        <v/>
+      </c>
+      <c r="M270" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="str">
+        <v>KW-19</v>
+      </c>
+      <c r="B271" t="str">
+        <v>Pattupavada</v>
+      </c>
+      <c r="C271" t="str">
+        <v>Kids Wear</v>
+      </c>
+      <c r="D271" t="str">
+        <v/>
+      </c>
+      <c r="E271">
+        <v>49</v>
+      </c>
+      <c r="F271">
+        <v>55</v>
+      </c>
+      <c r="G271" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H271" t="str">
+        <v>all sizes available</v>
+      </c>
+      <c r="I271" t="str">
+        <v>f21e8160-527b-4f42-87f2-db8556babe98.jpg</v>
+      </c>
+      <c r="J271" t="str">
+        <v/>
+      </c>
+      <c r="K271" t="str">
+        <v/>
+      </c>
+      <c r="L271" t="str">
+        <v>upto 9 yrs old</v>
+      </c>
+      <c r="M271" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="str">
+        <v>GW-17</v>
+      </c>
+      <c r="B272" t="str">
+        <v>Kurtha</v>
+      </c>
+      <c r="C272" t="str">
+        <v>Mens Wear</v>
+      </c>
+      <c r="D272" t="str">
+        <v/>
+      </c>
+      <c r="E272">
+        <v>65</v>
+      </c>
+      <c r="F272">
+        <v>78</v>
+      </c>
+      <c r="G272" t="str">
+        <v>SOLD OUT</v>
+      </c>
+      <c r="H272" t="str">
+        <v>L</v>
+      </c>
+      <c r="I272" t="str">
+        <v>85cfde47-871d-4480-a18b-ee96efee03d8.jpg</v>
+      </c>
+      <c r="J272" t="str">
+        <v/>
+      </c>
+      <c r="K272" t="str">
+        <v/>
+      </c>
+      <c r="L272" t="str">
+        <v/>
+      </c>
+      <c r="M272" t="str">
+        <v>No</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M263"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M272"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update store products via Admin Panel - 26/08/2026, 1:38:04 am
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M272"/>
+  <dimension ref="A1:M274"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -11674,9 +11674,91 @@
         <v>No</v>
       </c>
     </row>
+    <row r="273">
+      <c r="A273" t="str">
+        <v>KW-20</v>
+      </c>
+      <c r="B273" t="str">
+        <v>Kids frocks</v>
+      </c>
+      <c r="C273" t="str">
+        <v>Kids Wear</v>
+      </c>
+      <c r="D273" t="str">
+        <v/>
+      </c>
+      <c r="E273">
+        <v>44</v>
+      </c>
+      <c r="F273">
+        <v>49</v>
+      </c>
+      <c r="G273" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H273" t="str">
+        <v>UPTO SIZE 30</v>
+      </c>
+      <c r="I273" t="str">
+        <v>670a9ac3-ae40-4eba-bcd4-34920f53adca.jpg</v>
+      </c>
+      <c r="J273" t="str">
+        <v/>
+      </c>
+      <c r="K273" t="str">
+        <v/>
+      </c>
+      <c r="L273" t="str">
+        <v>Available in maroon shades also</v>
+      </c>
+      <c r="M273" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="str">
+        <v>JW-67</v>
+      </c>
+      <c r="B274" t="str">
+        <v>Premium  necklace set</v>
+      </c>
+      <c r="C274" t="str">
+        <v>Jewellery</v>
+      </c>
+      <c r="D274" t="str">
+        <v>Necklace</v>
+      </c>
+      <c r="E274">
+        <v>42</v>
+      </c>
+      <c r="F274">
+        <v>49</v>
+      </c>
+      <c r="G274" t="str">
+        <v>LIMITED STOCK</v>
+      </c>
+      <c r="H274" t="str">
+        <v/>
+      </c>
+      <c r="I274" t="str">
+        <v>6dc43f53-551e-4bc6-8bc2-91835fb7bf65.jpg</v>
+      </c>
+      <c r="J274" t="str">
+        <v/>
+      </c>
+      <c r="K274" t="str">
+        <v/>
+      </c>
+      <c r="L274" t="str">
+        <v>Matching ear rings available. Limited stock</v>
+      </c>
+      <c r="M274" t="str">
+        <v>No</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M272"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M274"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update store products via Admin Panel - 27/08/2026, 1:10:32 pm
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -1134,7 +1134,7 @@
         <v/>
       </c>
       <c r="E18">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="F18">
         <v>56</v>
@@ -4030,7 +4030,7 @@
         <v>85</v>
       </c>
       <c r="G88" t="str">
-        <v>INSTOCK</v>
+        <v>SOLD OUT</v>
       </c>
       <c r="H88" t="str">
         <v>LARGE</v>
@@ -5393,10 +5393,10 @@
         <v/>
       </c>
       <c r="E121">
-        <v>54</v>
+        <v>68</v>
       </c>
       <c r="F121">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="G121" t="str">
         <v>INSTOCK</v>
@@ -9890,7 +9890,7 @@
         <v>79</v>
       </c>
       <c r="G229" t="str">
-        <v>INSTOCK</v>
+        <v>SOLD OUT</v>
       </c>
       <c r="H229" t="str">
         <v/>

</xml_diff>

<commit_message>
Update store products via Admin Panel - 27/08/2026, 1:17:27 pm
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -4194,7 +4194,7 @@
         <v>110</v>
       </c>
       <c r="G92" t="str">
-        <v>INSTOCK</v>
+        <v>SOLD OUT</v>
       </c>
       <c r="H92" t="str">
         <v/>
@@ -9718,10 +9718,10 @@
         <v/>
       </c>
       <c r="E225">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="F225">
-        <v>112</v>
+        <v>125</v>
       </c>
       <c r="G225" t="str">
         <v>INSTOCK</v>
@@ -10587,7 +10587,7 @@
         <v>55</v>
       </c>
       <c r="G246" t="str">
-        <v>INSTOCK</v>
+        <v>SOLD OUT</v>
       </c>
       <c r="H246" t="str">
         <v/>
@@ -10669,7 +10669,7 @@
         <v>70</v>
       </c>
       <c r="G248" t="str">
-        <v>INSTOCK</v>
+        <v>SOLD OUT</v>
       </c>
       <c r="H248" t="str">
         <v>40</v>

</xml_diff>

<commit_message>
Update store products via Admin Panel - 06/09/2026, 12:22:01 am
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -5399,7 +5399,7 @@
         <v>74</v>
       </c>
       <c r="G121" t="str">
-        <v>INSTOCK</v>
+        <v>SOLD OUT</v>
       </c>
       <c r="H121" t="str">
         <v/>
@@ -11325,7 +11325,7 @@
         <v>78</v>
       </c>
       <c r="G264" t="str">
-        <v>INSTOCK</v>
+        <v>SOLD OUT</v>
       </c>
       <c r="H264" t="str">
         <v>L</v>

</xml_diff>

<commit_message>
Update store products via Admin Panel - 06/09/2026, 1:13:41 am
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M274"/>
+  <dimension ref="A1:M278"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -11756,9 +11756,173 @@
         <v>No</v>
       </c>
     </row>
+    <row r="275">
+      <c r="A275" t="str">
+        <v>JW-68</v>
+      </c>
+      <c r="B275" t="str">
+        <v>Necklace</v>
+      </c>
+      <c r="C275" t="str">
+        <v>Jewellery</v>
+      </c>
+      <c r="D275" t="str">
+        <v>Necklace</v>
+      </c>
+      <c r="E275">
+        <v>26</v>
+      </c>
+      <c r="F275">
+        <v>28</v>
+      </c>
+      <c r="G275" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H275" t="str">
+        <v/>
+      </c>
+      <c r="I275" t="str">
+        <v>d89f547f-6318-4301-abd2-ce3a5ba2b413.jpg</v>
+      </c>
+      <c r="J275" t="str">
+        <v>f2ce700f-48b4-43f6-a6cb-61a36e8f7630.jpg</v>
+      </c>
+      <c r="K275" t="str">
+        <v/>
+      </c>
+      <c r="L275" t="str">
+        <v/>
+      </c>
+      <c r="M275" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="str">
+        <v>JW-69</v>
+      </c>
+      <c r="B276" t="str">
+        <v>Coral stone  necklace</v>
+      </c>
+      <c r="C276" t="str">
+        <v>Jewellery</v>
+      </c>
+      <c r="D276" t="str">
+        <v>Necklace</v>
+      </c>
+      <c r="E276">
+        <v>44</v>
+      </c>
+      <c r="F276">
+        <v>50</v>
+      </c>
+      <c r="G276" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H276" t="str">
+        <v/>
+      </c>
+      <c r="I276" t="str">
+        <v>cf3f1c4c-56af-442c-b263-578fe3398ecb.jpg</v>
+      </c>
+      <c r="J276" t="str">
+        <v>53aeff17-14ff-4155-b250-241f6154f0e9.jpg</v>
+      </c>
+      <c r="K276" t="str">
+        <v/>
+      </c>
+      <c r="L276" t="str">
+        <v/>
+      </c>
+      <c r="M276" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="str">
+        <v>JW-70</v>
+      </c>
+      <c r="B277" t="str">
+        <v>Lotus Necklace</v>
+      </c>
+      <c r="C277" t="str">
+        <v>Jewellery</v>
+      </c>
+      <c r="D277" t="str">
+        <v>Necklace</v>
+      </c>
+      <c r="E277">
+        <v>24</v>
+      </c>
+      <c r="F277">
+        <v>36</v>
+      </c>
+      <c r="G277" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H277" t="str">
+        <v/>
+      </c>
+      <c r="I277" t="str">
+        <v>9d2ebc31-ea0f-49ab-a8ce-cffcaccf16c3.jpg</v>
+      </c>
+      <c r="J277" t="str">
+        <v>39ab9b5e-7afa-4301-b51a-281b998ae299.jpg</v>
+      </c>
+      <c r="K277" t="str">
+        <v/>
+      </c>
+      <c r="L277" t="str">
+        <v/>
+      </c>
+      <c r="M277" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="str">
+        <v>JW-71</v>
+      </c>
+      <c r="B278" t="str">
+        <v>Necklace</v>
+      </c>
+      <c r="C278" t="str">
+        <v>Jewellery</v>
+      </c>
+      <c r="D278" t="str">
+        <v>Necklace</v>
+      </c>
+      <c r="E278">
+        <v>26</v>
+      </c>
+      <c r="F278">
+        <v>32</v>
+      </c>
+      <c r="G278" t="str">
+        <v>INSTOCK</v>
+      </c>
+      <c r="H278" t="str">
+        <v/>
+      </c>
+      <c r="I278" t="str">
+        <v>e96f5952-ad89-4eec-8f5b-741770b1d45a.jpg</v>
+      </c>
+      <c r="J278" t="str">
+        <v/>
+      </c>
+      <c r="K278" t="str">
+        <v/>
+      </c>
+      <c r="L278" t="str">
+        <v/>
+      </c>
+      <c r="M278" t="str">
+        <v>No</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M274"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M278"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>